<commit_message>
Monitoreo 2026-09-16: gasoducto Cloud Connector y Corpus Christi Trains 8&9
Se agregan 2 proyectos nuevos a LNG: Cloud Connector Pipeline (Venture
Global, feedgas para Plaquemines LNG Fase 2) y Corpus Christi Midscale
Trains 8 & 9 (Cheniere/Bechtel, construcción >50% completa). Se
regenera proyectos.xlsx con el acumulado completo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3oVQuHdLVcM8Wz4Th4w2V
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -29,12 +29,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2594,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4342,6 +4337,80 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Corpus Christi Midscale Trains 8 &amp; 9 (+ debottlenecking)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>San Patricio County / Corpus Christi, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Cheniere Energy</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Bechtel Energy</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Construcción avanzada (FID positivo jun-2025, notice to proceed emitido a Bechtel; proyecto adyacente a Corpus Christi Stage 3, distinto de "Corpus Christi Stage 4"; 2 trenes midscale, &gt;3 MTPA adicionales; avance de obra reportado en &gt;50% a sep-2026; finalización esperada 2028)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>[LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-trains-8-and-9-project-more-than-50-percent-complete/196507/); [Businesswire FID](https://www.businesswire.com/news/home/20250623495479/en/Cheniere-Announces-Positive-Final-Investment-Decision-on-the-Corpus-Christi-Midscale-Trains-8-9-Project-and-Updated-Company-Outlook-through-2030)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Cloud Connector Pipeline</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Luisiana (recorrido intraestatal, no jurisdicción FERC), EE.UU.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Venture Global</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>No especificado (equipo mayor: Baker Hughes)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Construcción/Procura de equipo mayor (gasoducto intraestatal de ~300 millas, 48", feedgas para la expansión de Plaquemines LNG Fase 2; Baker Hughes recibió —13-sep-2026— una segunda orden de 13 sistemas de compresión, turbinas Frame 5/2E, ampliando la flota de compresión total del proyecto a 23 unidades)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/13/3360667/0/en/baker-hughes-and-venture-global-advance-next-phase-of-u-s-gas-infrastructure-growth.html)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-16: gasoducto Cloud Connector y Corpus Christi Trains 8&9 (#43)
Se agregan 2 proyectos nuevos a LNG: Cloud Connector Pipeline (Venture
Global, feedgas para Plaquemines LNG Fase 2) y Corpus Christi Midscale
Trains 8 & 9 (Cheniere/Bechtel, construcción >50% completa). Se
regenera proyectos.xlsx con el acumulado completo.


Claude-Session: https://claude.ai/code/session_01M3oVQuHdLVcM8Wz4Th4w2V

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -29,12 +29,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2594,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4342,6 +4337,80 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Corpus Christi Midscale Trains 8 &amp; 9 (+ debottlenecking)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>San Patricio County / Corpus Christi, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Cheniere Energy</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Bechtel Energy</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Construcción avanzada (FID positivo jun-2025, notice to proceed emitido a Bechtel; proyecto adyacente a Corpus Christi Stage 3, distinto de "Corpus Christi Stage 4"; 2 trenes midscale, &gt;3 MTPA adicionales; avance de obra reportado en &gt;50% a sep-2026; finalización esperada 2028)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>[LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-trains-8-and-9-project-more-than-50-percent-complete/196507/); [Businesswire FID](https://www.businesswire.com/news/home/20250623495479/en/Cheniere-Announces-Positive-Final-Investment-Decision-on-the-Corpus-Christi-Midscale-Trains-8-9-Project-and-Updated-Company-Outlook-through-2030)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Cloud Connector Pipeline</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Luisiana (recorrido intraestatal, no jurisdicción FERC), EE.UU.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Venture Global</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>No especificado (equipo mayor: Baker Hughes)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Construcción/Procura de equipo mayor (gasoducto intraestatal de ~300 millas, 48", feedgas para la expansión de Plaquemines LNG Fase 2; Baker Hughes recibió —13-sep-2026— una segunda orden de 13 sistemas de compresión, turbinas Frame 5/2E, ampliando la flota de compresión total del proyecto a 23 unidades)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/13/3360667/0/en/baker-hughes-and-venture-global-advance-next-phase-of-u-s-gas-infrastructure-growth.html)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-17: nuevo data center KIO MEX8 en CDMX
Se agrega KIO Data Centers MEX8 (Santa Fe, Ciudad de México) al tracker,
proyecto de centro de datos en construcción no documentado previamente.
Se regenera proyectos.xlsx con el acumulado completo de proyectos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RBvSgnUDvLxsZn9i3TY5gw
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,47 +419,47 @@
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2592,47 +2588,47 @@
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4428,47 +4424,47 @@
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -9110,50 +9106,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -13374,6 +13370,43 @@
       <c r="G115" t="inlineStr">
         <is>
           <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>KIO Data Centers MEX8</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Santa Fe, Ciudad de México, México</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>KIO Data Centers</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Construcción (inicio de obra anunciado 9/10-mar-2026; inversión US$70 millones; capacidad 4 MW, 60% ya pre-vendida; ~3,000 empleos directos e indirectos durante construcción; sistema de enfriamiento de circuito cerrado; inicio de operaciones previsto 1T2027)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/kio-begins-construction-of-mex8-facility-in-mexico-city/); [Reforma](https://www.reforma.com/invierte-kio-70-mdd-en-centro-de-datos-en-cdmx/ar3166439)</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-17: nuevo data center KIO MEX8 en CDMX (#44)
Se agrega KIO Data Centers MEX8 (Santa Fe, Ciudad de México) al tracker,
proyecto de centro de datos en construcción no documentado previamente.
Se regenera proyectos.xlsx con el acumulado completo de proyectos.


Claude-Session: https://claude.ai/code/session_01RBvSgnUDvLxsZn9i3TY5gw

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,47 +419,47 @@
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2592,47 +2588,47 @@
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4428,47 +4424,47 @@
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -9110,50 +9106,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -13374,6 +13370,43 @@
       <c r="G115" t="inlineStr">
         <is>
           <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>KIO Data Centers MEX8</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Santa Fe, Ciudad de México, México</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>KIO Data Centers</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Construcción (inicio de obra anunciado 9/10-mar-2026; inversión US$70 millones; capacidad 4 MW, 60% ya pre-vendida; ~3,000 empleos directos e indirectos durante construcción; sistema de enfriamiento de circuito cerrado; inicio de operaciones previsto 1T2027)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/kio-begins-construction-of-mex8-facility-in-mexico-city/); [Reforma](https://www.reforma.com/invierte-kio-70-mdd-en-centro-de-datos-en-cdmx/ar3166439)</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-21: 3 actualizaciones de fase (LNG, Mining, Data Centers)
- Commonwealth LNG (Cameron Parish, LA): Caturus anuncia expansión para casi
  duplicar capacidad (+7.75 MMtpa, total ~17.25 MMtpa).
- San Nicolás Copper-Zinc Project (Zacatecas): permisos federales confirmados
  como parte de paquete de 6 complejos mineros (~US$6,500M); acueducto de
  ~50km vía convenio con JIAPAZ.
- Aligned Data Centers "Project Phoenix" (Shippingport, PA): groundbreaking
  formal realizado 10-sep-2026, avanza de permitting a construcción.

Se regenera proyectos.xlsx completo (4 hojas por industria) a partir del
tracker.md acumulado. No se identificaron proyectos nuevos con evidencia
suficiente en esta corrida tras búsqueda dirigida en las 4 industrias.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EfeuvtJdZoTai1agzBfUsi
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -418,15 +418,6 @@
   </sheetPr>
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2587,15 +2578,6 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3064,17 +3046,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada 15-may-2026 bajo la entidad Caturus; cierre de financiamiento de USD 9,750 millones; Full NTP a Technip Energies; contrato de automatización principal a Yokogawa jul-2026; operaciones proyectadas 2030)</t>
+          <t>Construcción (FID alcanzada 15-may-2026 bajo la entidad Caturus; cierre de financiamiento de USD 9,750 millones; Full NTP a Technip Energies; contrato de automatización principal a Yokogawa jul-2026; operaciones proyectadas 2030) ; Caturus anunció (16-sep-2026) plan de expansión para casi duplicar la capacidad del proyecto, agregando 5 trenes de licuefacción adicionales (+7.75 MMtpa), llevando la capacidad total a ~17.25 MMtpa (vs. 9.5 MMtpa de la fase inicial ya en construcción)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); [PR Newswire/Caturus](https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); [PR Newswire/Caturus](https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html); [Rigzone](https://www.rigzone.com/news/kimmeridge_mubadala_to_nearly_double_commonwealth_lng_capacity-16-sep-2026-184634-article/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -4423,15 +4405,6 @@
   </sheetPr>
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4641,17 +4614,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026</t>
+          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026; confirmado (sep-2026) como parte de paquete de 6 complejos mineros en Zacatecas con autorizaciones federales principales (incl. Semarnat) ya obtenidas, inversión conjunta ~US$6,500 millones y ~15,000 empleos directos proyectados a partir de 2027; suministro de agua vía acueducto de ~50 km mediante convenio con la Junta Intermunicipal de Agua Potable y Alcantarillado de Zacatecas (JIAPAZ), con objetivo de reciclar el agua usada por la mina</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/) ; [Forbes México](https://forbes.com.mx/destraban-proyectos-mineros-en-zacatecas-por-6500-mdd/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -9108,15 +9081,6 @@
   </sheetPr>
   <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -12286,17 +12250,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Permitting avanzado/adquisición de sitio (uso condicional aprobado por el Concejo de Shippingport 28-ene-2026; Aligned cerró compra de ~651 acres por US$223 millones; pendientes permisos de mass grading, NPDES y stormwater; planta de gas natural de 3.6GW —reconversión de la ex-carboeléctrica Bruce Mansfield— co-ubicada con 3 edificios de datacenter de +600,000 pies² c/u; inversión total ~US$10,000 millones)</t>
+          <t>Construcción (groundbreaking formal realizado 10-sep-2026 junto con la comunidad de Shippingport; campus de 2GW, 3 edificios de datacenter de +600,000 pies² c/u sobre ~660 acres; planta de gas natural —reconversión de la ex-carboeléctrica Bruce Mansfield— co-ubicada como fuente de energía dedicada fuera de la red pública; ~3,000 empleos de construcción y ~640 empleos permanentes estimados; inversión total ~US$10,000 millones)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>[Beaver County Radio](https://beavercountyradio.com/news/align-data-centers-llc-closes-deal-to-build-data-center-campus-near-former-bruce-mansfield-power-plant-for-just-over-223-million/); [DCD](https://www.datacenterdynamics.com/en/news/shippingport-industrial-park/)</t>
+          <t>[Beaver County Radio](https://beavercountyradio.com/news/align-data-centers-llc-closes-deal-to-build-data-center-campus-near-former-bruce-mansfield-power-plant-for-just-over-223-million/); [DCD](https://www.datacenterdynamics.com/en/news/shippingport-industrial-park/); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/10/3359602/0/en/aligned-data-centers-and-shippingport-community-mark-revitalization-of-legacy-energy-site-with-groundbreaking-of-2-gw-project-phoenix-campus.html)</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-21: 3 actualizaciones de fase (LNG, Mining, Data Centers) (#45)
- Commonwealth LNG (Cameron Parish, LA): Caturus anuncia expansión para casi
  duplicar capacidad (+7.75 MMtpa, total ~17.25 MMtpa).
- San Nicolás Copper-Zinc Project (Zacatecas): permisos federales confirmados
  como parte de paquete de 6 complejos mineros (~US$6,500M); acueducto de
  ~50km vía convenio con JIAPAZ.
- Aligned Data Centers "Project Phoenix" (Shippingport, PA): groundbreaking
  formal realizado 10-sep-2026, avanza de permitting a construcción.

Se regenera proyectos.xlsx completo (4 hojas por industria) a partir del
tracker.md acumulado. No se identificaron proyectos nuevos con evidencia
suficiente en esta corrida tras búsqueda dirigida en las 4 industrias.


Claude-Session: https://claude.ai/code/session_01EfeuvtJdZoTai1agzBfUsi

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -418,15 +418,6 @@
   </sheetPr>
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2587,15 +2578,6 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3064,17 +3046,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada 15-may-2026 bajo la entidad Caturus; cierre de financiamiento de USD 9,750 millones; Full NTP a Technip Energies; contrato de automatización principal a Yokogawa jul-2026; operaciones proyectadas 2030)</t>
+          <t>Construcción (FID alcanzada 15-may-2026 bajo la entidad Caturus; cierre de financiamiento de USD 9,750 millones; Full NTP a Technip Energies; contrato de automatización principal a Yokogawa jul-2026; operaciones proyectadas 2030) ; Caturus anunció (16-sep-2026) plan de expansión para casi duplicar la capacidad del proyecto, agregando 5 trenes de licuefacción adicionales (+7.75 MMtpa), llevando la capacidad total a ~17.25 MMtpa (vs. 9.5 MMtpa de la fase inicial ya en construcción)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); [PR Newswire/Caturus](https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); [PR Newswire/Caturus](https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html); [Rigzone](https://www.rigzone.com/news/kimmeridge_mubadala_to_nearly_double_commonwealth_lng_capacity-16-sep-2026-184634-article/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -4423,15 +4405,6 @@
   </sheetPr>
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4641,17 +4614,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026</t>
+          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026; confirmado (sep-2026) como parte de paquete de 6 complejos mineros en Zacatecas con autorizaciones federales principales (incl. Semarnat) ya obtenidas, inversión conjunta ~US$6,500 millones y ~15,000 empleos directos proyectados a partir de 2027; suministro de agua vía acueducto de ~50 km mediante convenio con la Junta Intermunicipal de Agua Potable y Alcantarillado de Zacatecas (JIAPAZ), con objetivo de reciclar el agua usada por la mina</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/) ; [Forbes México](https://forbes.com.mx/destraban-proyectos-mineros-en-zacatecas-por-6500-mdd/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -9108,15 +9081,6 @@
   </sheetPr>
   <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -12286,17 +12250,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Permitting avanzado/adquisición de sitio (uso condicional aprobado por el Concejo de Shippingport 28-ene-2026; Aligned cerró compra de ~651 acres por US$223 millones; pendientes permisos de mass grading, NPDES y stormwater; planta de gas natural de 3.6GW —reconversión de la ex-carboeléctrica Bruce Mansfield— co-ubicada con 3 edificios de datacenter de +600,000 pies² c/u; inversión total ~US$10,000 millones)</t>
+          <t>Construcción (groundbreaking formal realizado 10-sep-2026 junto con la comunidad de Shippingport; campus de 2GW, 3 edificios de datacenter de +600,000 pies² c/u sobre ~660 acres; planta de gas natural —reconversión de la ex-carboeléctrica Bruce Mansfield— co-ubicada como fuente de energía dedicada fuera de la red pública; ~3,000 empleos de construcción y ~640 empleos permanentes estimados; inversión total ~US$10,000 millones)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>[Beaver County Radio](https://beavercountyradio.com/news/align-data-centers-llc-closes-deal-to-build-data-center-campus-near-former-bruce-mansfield-power-plant-for-just-over-223-million/); [DCD](https://www.datacenterdynamics.com/en/news/shippingport-industrial-park/)</t>
+          <t>[Beaver County Radio](https://beavercountyradio.com/news/align-data-centers-llc-closes-deal-to-build-data-center-campus-near-former-bruce-mansfield-power-plant-for-just-over-223-million/); [DCD](https://www.datacenterdynamics.com/en/news/shippingport-industrial-park/); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/10/3359602/0/en/aligned-data-centers-and-shippingport-community-mark-revitalization-of-legacy-energy-site-with-groundbreaking-of-2-gw-project-phoenix-campus.html)</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-22: nuevo data center Telxius Cancún (Data Centers)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ewX3AzNTn4BTCLDu7ZahD
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -418,6 +418,15 @@
   </sheetPr>
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2578,6 +2587,15 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4405,6 +4423,15 @@
   </sheetPr>
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9079,8 +9106,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -13371,6 +13407,43 @@
       <c r="G116" t="inlineStr">
         <is>
           <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Telxius Cancún — Landing Gateway &amp; Edge Data Center</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Cancún, Quintana Roo, México</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Telxius (Telefónica)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Construcción/Inaugurado (anunciado 3-sep-2026; instalación AI-ready Tier III con redundancia N+1/2N en energía y enfriamiento; funcionará como punto de aterrizaje del cable submarino Tikal —Puerto Barrios, Guatemala a Boca Raton, EE.UU., capacidad inicial ~380 Tbps, lanzamiento de Tikal previsto 1S2027—; añade ruta alterna de conectividad hacia el hub de data centers de Querétaro)</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/telxius-strengthens-caribbean-connectivity-with-a-new-edge-data-center-in-cancun/); [DPL News](https://dplnews.com/telxius-inaugura-data-center-edge-cancun/)</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-22: nuevo data center Telxius Cancún + actualizaciones acumuladas
Claude-Session: https://claude.ai/code/session_019ewX3AzNTn4BTCLDu7ZahD

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -418,6 +418,15 @@
   </sheetPr>
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2578,6 +2587,15 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4405,6 +4423,15 @@
   </sheetPr>
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9079,8 +9106,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -13371,6 +13407,43 @@
       <c r="G116" t="inlineStr">
         <is>
           <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Telxius Cancún — Landing Gateway &amp; Edge Data Center</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Cancún, Quintana Roo, México</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Telxius (Telefónica)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Construcción/Inaugurado (anunciado 3-sep-2026; instalación AI-ready Tier III con redundancia N+1/2N en energía y enfriamiento; funcionará como punto de aterrizaje del cable submarino Tikal —Puerto Barrios, Guatemala a Boca Raton, EE.UU., capacidad inicial ~380 Tbps, lanzamiento de Tikal previsto 1S2027—; añade ruta alterna de conectividad hacia el hub de data centers de Querétaro)</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/telxius-strengthens-caribbean-connectivity-with-a-new-edge-data-center-in-cancun/); [DPL News](https://dplnews.com/telxius-inaugura-data-center-edge-cancun/)</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-23: 2 nuevos data centers en West Texas
- DataBank Red Oak Data Center Campus (Red Oak, TX) — 480 MW, construcción
- Open Origin Presidio County/Marfa (data center + amoniaco) — planeación temprana

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VgTYXXJyMFv725CeFH2CS7
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -419,13 +419,13 @@
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2588,13 +2588,13 @@
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4424,13 +4424,13 @@
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9106,16 +9106,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13447,6 +13447,80 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>DataBank Red Oak Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Red Oak, Texas, EE.UU. (condado Ellis, sur de Dallas)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>DataBank</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Construcción (campus de 292 acres, 3.4 millones de pies² en 8 edificios de 2 pisos —425,000 pies² c/u—, 480 MW de capacidad crítica total; financiamiento de US$2,000 millones; primer edificio DFW9 con inicio de operación previsto ago-2026, ya arrendado a una empresa de IA; quinto edificio DFW15 —444,000 pies², US$425 millones— con groundbreaking previsto feb-2027 y terminación fines de 2029; campus completo previsto 3T2030)</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>[DataBank](https://www.databank.com/resources/news/inside-databanks-multibillion-dollar-red-oak-data-center-campus/); [Dallas Morning News](https://www.dallasnews.com/business/energy/article/construction-red-oak-databank-data-centers-campus-22316548.php); [Data Center Dynamics](https://www.datacenterdynamics.com/en/news/databank-announces-480mw-campus-in-dallas-texas/)</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Open Origin — Campus de Data Center + Amoniaco (Presidio County/Marfa)</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Presidio County, Texas, EE.UU. (sureste de Marfa; ranchos MacGuire y Antelope Springs)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Open Origin (terreno propiedad de Texas Mountain Cattle Company, de Brad Kelley; venta de tierra aún pendiente de finalizar)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Planeación muy temprana (campus propuesto de ~80,000 acres; combina centro de datos fuera de la red eléctrica con plantas de producción de amoniaco alimentadas por energía solar in situ; busca calificar para el RFP de capacidad de Stargate/OpenAI; consumo de agua subterránea estimado hasta 800 acre-pies/año genera oposición comunitaria activa; discusiones en curso con el condado de Presidio y la ciudad de Marfa, sin permisos ni EPC asegurados)</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/80000-acre-data-center-campus-proposed-in-west-texas/); [Big Bend Sentinel](https://bigbendsentinel.com/2025/10/01/proposed-marfa-data-center-still-in-discussions/); [Baxtel](https://baxtel.com/data-center/open-origin-presidio-county-tx)</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-09-23: 2 nuevos data centers en West Texas (#47)
- DataBank Red Oak Data Center Campus (Red Oak, TX) — 480 MW, construcción
- Open Origin Presidio County/Marfa (data center + amoniaco) — planeación temprana


Claude-Session: https://claude.ai/code/session_01VgTYXXJyMFv725CeFH2CS7

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -419,13 +419,13 @@
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2588,13 +2588,13 @@
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4424,13 +4424,13 @@
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9106,16 +9106,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13447,6 +13447,80 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>DataBank Red Oak Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Red Oak, Texas, EE.UU. (condado Ellis, sur de Dallas)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>DataBank</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Construcción (campus de 292 acres, 3.4 millones de pies² en 8 edificios de 2 pisos —425,000 pies² c/u—, 480 MW de capacidad crítica total; financiamiento de US$2,000 millones; primer edificio DFW9 con inicio de operación previsto ago-2026, ya arrendado a una empresa de IA; quinto edificio DFW15 —444,000 pies², US$425 millones— con groundbreaking previsto feb-2027 y terminación fines de 2029; campus completo previsto 3T2030)</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>[DataBank](https://www.databank.com/resources/news/inside-databanks-multibillion-dollar-red-oak-data-center-campus/); [Dallas Morning News](https://www.dallasnews.com/business/energy/article/construction-red-oak-databank-data-centers-campus-22316548.php); [Data Center Dynamics](https://www.datacenterdynamics.com/en/news/databank-announces-480mw-campus-in-dallas-texas/)</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Open Origin — Campus de Data Center + Amoniaco (Presidio County/Marfa)</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Presidio County, Texas, EE.UU. (sureste de Marfa; ranchos MacGuire y Antelope Springs)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Open Origin (terreno propiedad de Texas Mountain Cattle Company, de Brad Kelley; venta de tierra aún pendiente de finalizar)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Planeación muy temprana (campus propuesto de ~80,000 acres; combina centro de datos fuera de la red eléctrica con plantas de producción de amoniaco alimentadas por energía solar in situ; busca calificar para el RFP de capacidad de Stargate/OpenAI; consumo de agua subterránea estimado hasta 800 acre-pies/año genera oposición comunitaria activa; discusiones en curso con el condado de Presidio y la ciudad de Marfa, sin permisos ni EPC asegurados)</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/80000-acre-data-center-campus-proposed-in-west-texas/); [Big Bend Sentinel](https://bigbendsentinel.com/2025/10/01/proposed-marfa-data-center-still-in-discussions/); [Baxtel](https://baxtel.com/data-center/open-origin-presidio-county-tx)</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-09-24: nuevo proyecto La Negra (Querétaro) + 12 actualizaciones de fase
Petroquímica: Fermachem, CF Industries Blue Point, Topolobampo (GPO)
LNG: Corpus Christi Stage 4, Gasoducto Texas Gateway
Mining: nuevo La Negra Project (Silverco); Antler Copper, Bagdad Mine, Twin Metals, Kings Mountain Lithium
Data Centers: Texas Critical Data Centers, Fermi America Project Matador, Fleet Data Centers Peru Ridge/South Valley

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQJ1QoUQWsar6qQtSFngap
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -418,15 +418,6 @@
   </sheetPr>
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -525,17 +516,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción</t>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción; contrato EPC de Technip Energies valuado en más de €1,000 millones; capex conjunto 2026 proyectado en US$600 millones prorrateado entre CF Industries (40%), JERA y Mitsui</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/)</t>
+          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/); [DecarbonFuse](https://decarbonfuse.com/posts/blue-point-breaks-ground-what-changes-now-it-s-building)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -969,17 +960,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace) presionan por la cancelación del proyecto)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace, con protesta en el Zócalo) presionan por la cancelación del proyecto; GPO aceptó, como parte de las negociaciones, modificar la toma de agua —reubicándola al canal de residuos de CFE— y descargar la salmuera caliente fuera de la bahía de Ohuira, mientras mantiene pausadas las plantas de urea y metanol; sin resolución final reportada a la fecha)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/); [Bajo Palabra](https://www.bajopalabra.mx/sheinbaum-descarta-por-ahora-cancelar-megaplanta-de-amoniaco-en-topolobampo-ante-reclamos-ambientales/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -1487,17 +1478,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Construcción con retraso administrativo (obra pausada ~mes y medio por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento, reanudación de obra esperada en 1-2 semanas)</t>
+          <t>Construcción reanudada (obra había sido pausada por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento; gobernador Esteban Villegas confirmó 7-sep-2026 que la empresa cuenta con todos los permisos federales pese a objeciones del cabildo de Lerdo sobre permisos municipales; Sedeco Durango reafirmó 23-sep-2026 que el proyecto está "vigente al 100%" con todas las autorizaciones ambientales en regla; ya se completaron trabajos de compactación/preparación de 150 hectáreas en el ejido Sapioriz; construcción formal de la primera fase se proyecta en ~28 meses; inversión ~US$1,600 millones, capacidad 1 millón ton/año de urea granulada)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [Grem Noticieros](https://www.noticierosgrem.com.mx/costruccion-de-fermachem-podria-arrancar-en-dos-semanas-desarrollo-economico-de-durango/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [El Siglo de Torreón — Canacintra](https://www.elsiglodetorreon.com.mx/noticia/2026/fermachem-es-un-proyecto-auditado-legal-y-mexicano-sin-almacenamiento-de-amoniaco-canacintra.html); [Grem Noticieros — Sedeco](https://www.noticierosgrem.com.mx/vigente-al-100-proyecto-de-planta-fermachem-en-lerdo-sedeco/); [El Siglo de Torreón — Gobernador](https://www.elsiglodetorreon.com.mx/noticia/2026/planta-de-fermachen-en-lerdo-va-mas-que-firme-gobernador-de-durango.html)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2587,15 +2578,6 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3508,17 +3490,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Open season vinculante (hasta 8-dic-2026) / FAST-41; en servicio previsto nov-2029</t>
+          <t>Open season vinculante (hasta 8-dic-2026) / FAST-41; FERC emitió el 25-ago-2026 el Notice of Intent (NOI) para preparar el EIS bajo el docket CP26-547, con periodo de comentarios sobre alcance ambiental cerrado el 24-sep-2026; proyecto de 155 millas y capacidad firme mínima de 1.45 millones Dth/d, moverá gas desde hubs de Texas hacia centros de demanda industrial y terminales LNG en Luisiana; en servicio previsto nov-2029</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/); [PGJ](https://pgjonline.com/news/2026/september/enbridge-launches-open-season-for-proposed-texas-natgas-pipe); [OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55326964/boardwalk-launches-texas-gateway-project-open-season-aiming-to-deliver-natural-gas-to-gulf-coast)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -3767,17 +3749,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Permitting (solicitud FERC en proceso desde 17-feb-2026; DOE revisando solicitud de exportación; EIS borrador esperado sep-2026; incluye gasoducto de alimentación CCPL de 42"/26 millas)</t>
+          <t>Permitting (FERC emitió el 23-sep-2026 el Draft Environmental Impact Statement —EIS borrador— para el proyecto y su expansión de gasoducto asociada, Corpus Christi Pipeline/CCPL: ~25.8 millas de loop de 42", nueva estación de compresión, dos estaciones de medición y tres válvulas de línea principal, capacidad adicional de hasta 2.75 Bcf/d; FERC concluyó preliminarmente efectos ambientales adversos pero no significativos; periodo de comentarios públicos abierto hasta 9-nov-2026; EIS Final esperado 12-mar-2027; plazo de decisión federal de autorización —90 días— vence 10-jun-2027, encaminando el proyecto hacia FID en 2S-2027; DOE revisando solicitud de exportación)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/09/23/2026-19447/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi); [FERC](https://www.ferc.gov/news-events/news/ferc-staff-issues-draft-environmental-impact-statement-corpus-christi-liquefaction); [LNG Prime](https://lngprime.com/americas/ferc-issues-draft-eis-for-chenieres-corpus-christi-stage-4-project/197338/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -4421,17 +4403,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5677,17 +5650,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Permitting casi completo/inicio de construcción (BLM emitió Determinación de Adecuación NEPA; obras previstas 2do semestre 2026; embarque de concentrado previsto 2027)</t>
+          <t>Permitting casi completo/inicio de construcción (BLM emitió Determinación de Adecuación NEPA; obras previstas 2do semestre 2026; embarque de concentrado previsto 2027; el Federal Permitting Dashboard confirma el 22-sep-2026 como fecha estimada de finalización de la revisión ambiental NEPA —Environmental Assessment— del Mine Plan of Operations por el BLM, hito clave hacia construcción)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/); [Permitting Dashboard](https://www.permits.performance.gov/permitting-project/fast-41-transparency-projects/antler-copper-project)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -5788,17 +5761,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental revisado al alza ~30% a ~US$4,500 millones —antes ~US$3,500 millones—, reportado 7/8-ago-2026; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
+          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre y +10-12 Mlb/año molibdeno, posicionando a Bagdad como la 2ª mina más grande de Freeport en EE.UU. tras Morenci; capex incremental revisado al alza ~30% a ~US$3,500-4,500 millones, requiere precio de cobre ≥US$4.00/lb; US$150M asignados en 2026 para ingeniería y obras tempranas; Freeport planea presentar el plan a su consejo antes de fin de 2026 buscando FID positiva; Bagdad convirtió su flota de camiones a operación autónoma, primer sitio de EE.UU. de Freeport en adoptar la tecnología, reportado 18-sep-2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm); [ABC15](https://www.abc15.com/news/business/freeport-mcmoran-eyes-4-5b-expansion-of-arizona-mine-as-investment-decision-looms)</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm); [ABC15](https://www.abc15.com/news/business/freeport-mcmoran-eyes-4-5b-expansion-of-arizona-mine-as-investment-decision-looms); [Defense World](https://www.defenseworld.net/2026/09/18/freeport-mcmoran-eyes-leach-breakthrough-bagdad-growth-and-grasberg-recovery.html)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8415,17 +8388,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Permitting/Pre-EIS con retroceso regulatorio (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026 mediante orden ejecutiva que prohíbe minería no ferrosa en la cuenca del Rainy River Headwaters; el DNR de Minnesota canceló uno de los arrendamientos minerales de Twin Metals cerca de Babbitt por incumplimiento de requisitos de desempeño/producción, anunciado 14-sep-2026 y efectivo 10-nov-2026; grupos ambientalistas lo ven como precedente para cancelar los arrendamientos restantes; proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242); [KAXE](https://www.kaxe.org/local-news/2026-09-14/dnr-cancels-1-twin-metals-mineral-lease-near-babbitt); [Voyageurs Conservancy](https://www.voyageurs.org/news/2026/9/22/what-the-walz-order-and-the-twin-metals-lease-cancellation-mean-for-voyageurs)</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8637,17 +8610,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión)</t>
+          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión; DOE anunció 14-sep-2026 US$16 millones adicionales para programas de educación minera durante visita al sitio —14 escuelas mineras acreditadas—; proyecto sigue a la espera de permisos estatales y locales, tajo ya drenado)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf)</t>
+          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf); [WFAE](https://www.wfae.org/energy-environment/2026-09-14/trump-administration-announces-16-million-for-mining-education-at-kings-mountain-lithium-site)</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -9092,6 +9065,43 @@
       <c r="G126" t="inlineStr">
         <is>
           <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>La Negra Project (expansión)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Ciudad de Querétaro, Querétaro, México</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Silverco Mining (ex Nuevo Silver; adquisición completada may-2026)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Ingeniería/optimización (mina de plata-plomo-zinc-cobre tipo skarn en operación con más de 5 décadas de historia; PEA publicado 23-sep-2026 con VAN de US$329 millones sobre inversión de solo US$20.9 millones, vida de mina de 8.2 años; meta de expansión de capacidad de procesamiento a 2,500 tpd para 2S-2027, producción promedio estimada 4.1 millones oz eq. plata/año; programa de 15,000 m de perforación en curso para revalidar el depósito skarn)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/09/silverco-mining-proyecto-la-negra-en-queretaro-proyecta-van-de-us329-millones/); [Minart](https://minart.pe/2026/09/23/silverco-proyecta-us329-millones-de-valor-para-la-mina-la-negra-y-una-vida-util-de-82-anos/)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -9108,15 +9118,6 @@
   </sheetPr>
   <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9807,17 +9808,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; New Era aseguró permisos clave adicionales —Development Structure Permit, Drive Approach Permit— y presentó Notice of Intent ante TCEQ para nivelación de terreno, 17-ago-2026; capacidad combinada Fase 1+2 aumentó de ~650MW a 757MW vía nuevo permiso de aire TCEQ de Thunderhead (Fase 2: 450→550MW); construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; New Era aseguró permisos clave adicionales —Development Structure Permit, Drive Approach Permit— y presentó Notice of Intent ante TCEQ para nivelación de terreno, 17-ago-2026; capacidad combinada Fase 1+2 aumentó de ~650MW a 757MW vía nuevo permiso de aire TCEQ de Thunderhead (Fase 2: 450→550MW); construcción total prevista en 2026, primeros 100MW dic-2026; TCDC PowerCo LLC firmó 21-sep-2026 un PPA a 20 años con Luminant ET Services —afiliada de Vistra— por 200-207 MW para la Fase 1 (493 acres, escalando a 1.4GW), suministrado por la planta de gas natural de 1,180 MW de Vistra en Odessa, adyacente al sitio; entrega de energía firme prevista Q3 2027)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html); [Minichart](https://www.minichart.com.sg/2026/08/17/new-era-energy-secures-construction-permits-for-texas-data-center-campus/)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html); [Minichart](https://www.minichart.com.sg/2026/08/17/new-era-energy-secures-construction-permits-for-texas-data-center-campus/); [GlobeNewswire PPA](https://www.globenewswire.com/news-release/2026/09/21/3365358/0/en/new-era-energy-digital-secures-20-year-207-mw-ppa-with-vistra.html); [Data Center Dynamics](https://www.datacenterdynamics.com/en/news/new-era-signs-20-year-gas-ppa-with-vistra-subsidiary-to-power-250mw-data-center-in-ector-county-texas/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -10584,17 +10585,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -12878,17 +12879,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Solicitud regulatoria (dos plantas de gas natural dedicadas —motores de gas metano— para autogeneración: Peru Ridge Self-Generation Project (218 MW) y South Valley (planta temporal, 144 MW), alimentando dos campus de data centers en el mismo parque industrial; solicitud ante la Public Utility Commission of Nevada (PUCN), decisión final esperada 8-sep-2026)</t>
+          <t>Aprobado/pre-construcción (la Public Utilities Commission of Nevada —PUCN— aprobó el 17-sep-2026 las solicitudes para construir dos plantas de generación de gas natural temporales, behind-the-meter: Peru Ridge Self-Generation Project —218 MW, 23.4 acres en TRIC, Reno— y South Valley —144 MW, 37.4 acres, Sparks—, 362 MW combinados, alimentando dos campus de data centers en el mismo parque industrial; construcción prevista para inicios de 2027 —~6 meses—, operación temporal de 2-3 años hasta que llegue servicio permanente de la red)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>[Nevada Current](https://nevadacurrent.com/2026/09/01/private-gas-plants-to-power-data-centers-would-skirt-states-renewable-energy-law/); [The Nevada Independent](https://thenevadaindependent.com/article/why-a-northern-nevada-data-center-wants-to-build-its-own-temporary-natural-gas-power-plant)</t>
+          <t>[Nevada Current](https://nevadacurrent.com/2026/09/01/private-gas-plants-to-power-data-centers-would-skirt-states-renewable-energy-law/); [The Nevada Independent](https://thenevadaindependent.com/article/why-a-northern-nevada-data-center-wants-to-build-its-own-temporary-natural-gas-power-plant); [ConstructConnect](https://news.constructconnect.com/nevada-regulators-approve-362-mw-of-temporary-power-projects-for-data-centers); [Nevada Current — Aprobación](https://nevadacurrent.com/2026/09/18/public-utility-commission-approves-gas-plants-to-power-data-centers/)</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-24: nuevo La Negra (Querétaro) + 12 actualizaciones (#48)
Petroquímica: Fermachem, CF Industries Blue Point, Topolobampo (GPO)
LNG: Corpus Christi Stage 4, Gasoducto Texas Gateway
Mining: nuevo La Negra Project (Silverco); Antler Copper, Bagdad Mine, Twin Metals, Kings Mountain Lithium
Data Centers: Texas Critical Data Centers, Fermi America Project Matador, Fleet Data Centers Peru Ridge/South Valley


Claude-Session: https://claude.ai/code/session_01EQJ1QoUQWsar6qQtSFngap

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -418,15 +418,6 @@
   </sheetPr>
   <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -525,17 +516,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción</t>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción; contrato EPC de Technip Energies valuado en más de €1,000 millones; capex conjunto 2026 proyectado en US$600 millones prorrateado entre CF Industries (40%), JERA y Mitsui</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/)</t>
+          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/); [DecarbonFuse](https://decarbonfuse.com/posts/blue-point-breaks-ground-what-changes-now-it-s-building)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -969,17 +960,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace) presionan por la cancelación del proyecto)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace, con protesta en el Zócalo) presionan por la cancelación del proyecto; GPO aceptó, como parte de las negociaciones, modificar la toma de agua —reubicándola al canal de residuos de CFE— y descargar la salmuera caliente fuera de la bahía de Ohuira, mientras mantiene pausadas las plantas de urea y metanol; sin resolución final reportada a la fecha)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/); [Bajo Palabra](https://www.bajopalabra.mx/sheinbaum-descarta-por-ahora-cancelar-megaplanta-de-amoniaco-en-topolobampo-ante-reclamos-ambientales/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -1487,17 +1478,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Construcción con retraso administrativo (obra pausada ~mes y medio por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento, reanudación de obra esperada en 1-2 semanas)</t>
+          <t>Construcción reanudada (obra había sido pausada por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento; gobernador Esteban Villegas confirmó 7-sep-2026 que la empresa cuenta con todos los permisos federales pese a objeciones del cabildo de Lerdo sobre permisos municipales; Sedeco Durango reafirmó 23-sep-2026 que el proyecto está "vigente al 100%" con todas las autorizaciones ambientales en regla; ya se completaron trabajos de compactación/preparación de 150 hectáreas en el ejido Sapioriz; construcción formal de la primera fase se proyecta en ~28 meses; inversión ~US$1,600 millones, capacidad 1 millón ton/año de urea granulada)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [Grem Noticieros](https://www.noticierosgrem.com.mx/costruccion-de-fermachem-podria-arrancar-en-dos-semanas-desarrollo-economico-de-durango/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [El Siglo de Torreón — Canacintra](https://www.elsiglodetorreon.com.mx/noticia/2026/fermachem-es-un-proyecto-auditado-legal-y-mexicano-sin-almacenamiento-de-amoniaco-canacintra.html); [Grem Noticieros — Sedeco](https://www.noticierosgrem.com.mx/vigente-al-100-proyecto-de-planta-fermachem-en-lerdo-sedeco/); [El Siglo de Torreón — Gobernador](https://www.elsiglodetorreon.com.mx/noticia/2026/planta-de-fermachen-en-lerdo-va-mas-que-firme-gobernador-de-durango.html)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2587,15 +2578,6 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3508,17 +3490,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Open season vinculante (hasta 8-dic-2026) / FAST-41; en servicio previsto nov-2029</t>
+          <t>Open season vinculante (hasta 8-dic-2026) / FAST-41; FERC emitió el 25-ago-2026 el Notice of Intent (NOI) para preparar el EIS bajo el docket CP26-547, con periodo de comentarios sobre alcance ambiental cerrado el 24-sep-2026; proyecto de 155 millas y capacidad firme mínima de 1.45 millones Dth/d, moverá gas desde hubs de Texas hacia centros de demanda industrial y terminales LNG en Luisiana; en servicio previsto nov-2029</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/); [PGJ](https://pgjonline.com/news/2026/september/enbridge-launches-open-season-for-proposed-texas-natgas-pipe); [OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55326964/boardwalk-launches-texas-gateway-project-open-season-aiming-to-deliver-natural-gas-to-gulf-coast)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -3767,17 +3749,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Permitting (solicitud FERC en proceso desde 17-feb-2026; DOE revisando solicitud de exportación; EIS borrador esperado sep-2026; incluye gasoducto de alimentación CCPL de 42"/26 millas)</t>
+          <t>Permitting (FERC emitió el 23-sep-2026 el Draft Environmental Impact Statement —EIS borrador— para el proyecto y su expansión de gasoducto asociada, Corpus Christi Pipeline/CCPL: ~25.8 millas de loop de 42", nueva estación de compresión, dos estaciones de medición y tres válvulas de línea principal, capacidad adicional de hasta 2.75 Bcf/d; FERC concluyó preliminarmente efectos ambientales adversos pero no significativos; periodo de comentarios públicos abierto hasta 9-nov-2026; EIS Final esperado 12-mar-2027; plazo de decisión federal de autorización —90 días— vence 10-jun-2027, encaminando el proyecto hacia FID en 2S-2027; DOE revisando solicitud de exportación)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/09/23/2026-19447/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi); [FERC](https://www.ferc.gov/news-events/news/ferc-staff-issues-draft-environmental-impact-statement-corpus-christi-liquefaction); [LNG Prime](https://lngprime.com/americas/ferc-issues-draft-eis-for-chenieres-corpus-christi-stage-4-project/197338/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -4421,17 +4403,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5677,17 +5650,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Permitting casi completo/inicio de construcción (BLM emitió Determinación de Adecuación NEPA; obras previstas 2do semestre 2026; embarque de concentrado previsto 2027)</t>
+          <t>Permitting casi completo/inicio de construcción (BLM emitió Determinación de Adecuación NEPA; obras previstas 2do semestre 2026; embarque de concentrado previsto 2027; el Federal Permitting Dashboard confirma el 22-sep-2026 como fecha estimada de finalización de la revisión ambiental NEPA —Environmental Assessment— del Mine Plan of Operations por el BLM, hito clave hacia construcción)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/); [Permitting Dashboard](https://www.permits.performance.gov/permitting-project/fast-41-transparency-projects/antler-copper-project)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -5788,17 +5761,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental revisado al alza ~30% a ~US$4,500 millones —antes ~US$3,500 millones—, reportado 7/8-ago-2026; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
+          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre y +10-12 Mlb/año molibdeno, posicionando a Bagdad como la 2ª mina más grande de Freeport en EE.UU. tras Morenci; capex incremental revisado al alza ~30% a ~US$3,500-4,500 millones, requiere precio de cobre ≥US$4.00/lb; US$150M asignados en 2026 para ingeniería y obras tempranas; Freeport planea presentar el plan a su consejo antes de fin de 2026 buscando FID positiva; Bagdad convirtió su flota de camiones a operación autónoma, primer sitio de EE.UU. de Freeport en adoptar la tecnología, reportado 18-sep-2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm); [ABC15](https://www.abc15.com/news/business/freeport-mcmoran-eyes-4-5b-expansion-of-arizona-mine-as-investment-decision-looms)</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm); [ABC15](https://www.abc15.com/news/business/freeport-mcmoran-eyes-4-5b-expansion-of-arizona-mine-as-investment-decision-looms); [Defense World](https://www.defenseworld.net/2026/09/18/freeport-mcmoran-eyes-leach-breakthrough-bagdad-growth-and-grasberg-recovery.html)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8415,17 +8388,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Permitting/Pre-EIS con retroceso regulatorio (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026 mediante orden ejecutiva que prohíbe minería no ferrosa en la cuenca del Rainy River Headwaters; el DNR de Minnesota canceló uno de los arrendamientos minerales de Twin Metals cerca de Babbitt por incumplimiento de requisitos de desempeño/producción, anunciado 14-sep-2026 y efectivo 10-nov-2026; grupos ambientalistas lo ven como precedente para cancelar los arrendamientos restantes; proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242); [KAXE](https://www.kaxe.org/local-news/2026-09-14/dnr-cancels-1-twin-metals-mineral-lease-near-babbitt); [Voyageurs Conservancy](https://www.voyageurs.org/news/2026/9/22/what-the-walz-order-and-the-twin-metals-lease-cancellation-mean-for-voyageurs)</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8637,17 +8610,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión)</t>
+          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión; DOE anunció 14-sep-2026 US$16 millones adicionales para programas de educación minera durante visita al sitio —14 escuelas mineras acreditadas—; proyecto sigue a la espera de permisos estatales y locales, tajo ya drenado)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf)</t>
+          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf); [WFAE](https://www.wfae.org/energy-environment/2026-09-14/trump-administration-announces-16-million-for-mining-education-at-kings-mountain-lithium-site)</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -9092,6 +9065,43 @@
       <c r="G126" t="inlineStr">
         <is>
           <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>La Negra Project (expansión)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Ciudad de Querétaro, Querétaro, México</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Silverco Mining (ex Nuevo Silver; adquisición completada may-2026)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Ingeniería/optimización (mina de plata-plomo-zinc-cobre tipo skarn en operación con más de 5 décadas de historia; PEA publicado 23-sep-2026 con VAN de US$329 millones sobre inversión de solo US$20.9 millones, vida de mina de 8.2 años; meta de expansión de capacidad de procesamiento a 2,500 tpd para 2S-2027, producción promedio estimada 4.1 millones oz eq. plata/año; programa de 15,000 m de perforación en curso para revalidar el depósito skarn)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/09/silverco-mining-proyecto-la-negra-en-queretaro-proyecta-van-de-us329-millones/); [Minart](https://minart.pe/2026/09/23/silverco-proyecta-us329-millones-de-valor-para-la-mina-la-negra-y-una-vida-util-de-82-anos/)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -9108,15 +9118,6 @@
   </sheetPr>
   <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9807,17 +9808,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; New Era aseguró permisos clave adicionales —Development Structure Permit, Drive Approach Permit— y presentó Notice of Intent ante TCEQ para nivelación de terreno, 17-ago-2026; capacidad combinada Fase 1+2 aumentó de ~650MW a 757MW vía nuevo permiso de aire TCEQ de Thunderhead (Fase 2: 450→550MW); construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; New Era aseguró permisos clave adicionales —Development Structure Permit, Drive Approach Permit— y presentó Notice of Intent ante TCEQ para nivelación de terreno, 17-ago-2026; capacidad combinada Fase 1+2 aumentó de ~650MW a 757MW vía nuevo permiso de aire TCEQ de Thunderhead (Fase 2: 450→550MW); construcción total prevista en 2026, primeros 100MW dic-2026; TCDC PowerCo LLC firmó 21-sep-2026 un PPA a 20 años con Luminant ET Services —afiliada de Vistra— por 200-207 MW para la Fase 1 (493 acres, escalando a 1.4GW), suministrado por la planta de gas natural de 1,180 MW de Vistra en Odessa, adyacente al sitio; entrega de energía firme prevista Q3 2027)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html); [Minichart](https://www.minichart.com.sg/2026/08/17/new-era-energy-secures-construction-permits-for-texas-data-center-campus/)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html); [Minichart](https://www.minichart.com.sg/2026/08/17/new-era-energy-secures-construction-permits-for-texas-data-center-campus/); [GlobeNewswire PPA](https://www.globenewswire.com/news-release/2026/09/21/3365358/0/en/new-era-energy-digital-secures-20-year-207-mw-ppa-with-vistra.html); [Data Center Dynamics](https://www.datacenterdynamics.com/en/news/new-era-signs-20-year-gas-ppa-with-vistra-subsidiary-to-power-250mw-data-center-in-ector-county-texas/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -10584,17 +10585,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -12878,17 +12879,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Solicitud regulatoria (dos plantas de gas natural dedicadas —motores de gas metano— para autogeneración: Peru Ridge Self-Generation Project (218 MW) y South Valley (planta temporal, 144 MW), alimentando dos campus de data centers en el mismo parque industrial; solicitud ante la Public Utility Commission of Nevada (PUCN), decisión final esperada 8-sep-2026)</t>
+          <t>Aprobado/pre-construcción (la Public Utilities Commission of Nevada —PUCN— aprobó el 17-sep-2026 las solicitudes para construir dos plantas de generación de gas natural temporales, behind-the-meter: Peru Ridge Self-Generation Project —218 MW, 23.4 acres en TRIC, Reno— y South Valley —144 MW, 37.4 acres, Sparks—, 362 MW combinados, alimentando dos campus de data centers en el mismo parque industrial; construcción prevista para inicios de 2027 —~6 meses—, operación temporal de 2-3 años hasta que llegue servicio permanente de la red)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>[Nevada Current](https://nevadacurrent.com/2026/09/01/private-gas-plants-to-power-data-centers-would-skirt-states-renewable-energy-law/); [The Nevada Independent](https://thenevadaindependent.com/article/why-a-northern-nevada-data-center-wants-to-build-its-own-temporary-natural-gas-power-plant)</t>
+          <t>[Nevada Current](https://nevadacurrent.com/2026/09/01/private-gas-plants-to-power-data-centers-would-skirt-states-renewable-energy-law/); [The Nevada Independent](https://thenevadaindependent.com/article/why-a-northern-nevada-data-center-wants-to-build-its-own-temporary-natural-gas-power-plant); [ConstructConnect](https://news.constructconnect.com/nevada-regulators-approve-362-mw-of-temporary-power-projects-for-data-centers); [Nevada Current — Aprobación](https://nevadacurrent.com/2026/09/18/public-utility-commission-approves-gas-plants-to-power-data-centers/)</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-25: nuevo Terranova San Miguel de Allende (Guanajuato)
Data Centers: nuevo campus Terranova San Miguel de Allende / corredor Querétaro-Guanajuato (Actis), 8.12MW escalable a 20MW, parte de plan LATAM de US$1,500M

Investigación exhaustiva en Petroquímica, LNG y Mining no arrojó proyectos genuinamente nuevos ni cambios de fase verificables adicionales a lo ya documentado.

Claude-Session: https://claude.ai/code/session_01F1cxr5GYcmQrknFZTTrCGN

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -9116,7 +9116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13522,6 +13522,43 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Terranova San Miguel de Allende Data Center (corredor Querétaro-Guanajuato)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>San Miguel de Allende, Guanajuato, México</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Terranova (plataforma hyperscale LATAM respaldada por el fondo de infraestructura Actis)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Operando (primer sitio de Terranova en México, entró en operación con 8.12 MW iniciales, escalable a 20 MW; diseño y construcción completados en ~1 año; parte de un plan de inversión de US$1,500 millones de Terranova para desarrollar campus hyperscale en Brasil, México y Chile, con terreno y suministro eléctrico asegurados para escalar hasta 1GW en la región; sitio conectado al corredor de fibra Phoenix-Querétaro)</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/terranova-launches-in-mexico-with-its-first-data-center-campus/); [BNamericas](https://www.bnamericas.com/en/news/actis-backed-terranova-opens-first-mexico-data-center)</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-09-25: nuevo Terranova San Miguel de Allende (Guanajuato) (#49)
Data Centers: nuevo campus Terranova San Miguel de Allende / corredor Querétaro-Guanajuato (Actis), 8.12MW escalable a 20MW, parte de plan LATAM de US$1,500M

Investigación exhaustiva en Petroquímica, LNG y Mining no arrojó proyectos genuinamente nuevos ni cambios de fase verificables adicionales a lo ya documentado.

Claude-Session: https://claude.ai/code/session_01F1cxr5GYcmQrknFZTTrCGN

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -9116,7 +9116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13522,6 +13522,43 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Terranova San Miguel de Allende Data Center (corredor Querétaro-Guanajuato)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>San Miguel de Allende, Guanajuato, México</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Terranova (plataforma hyperscale LATAM respaldada por el fondo de infraestructura Actis)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Operando (primer sitio de Terranova en México, entró en operación con 8.12 MW iniciales, escalable a 20 MW; diseño y construcción completados en ~1 año; parte de un plan de inversión de US$1,500 millones de Terranova para desarrollar campus hyperscale en Brasil, México y Chile, con terreno y suministro eléctrico asegurados para escalar hasta 1GW en la región; sitio conectado al corredor de fibra Phoenix-Querétaro)</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/terranova-launches-in-mexico-with-its-first-data-center-campus/); [BNamericas](https://www.bnamericas.com/en/news/actis-backed-terranova-opens-first-mexico-data-center)</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-09-28: 1 nuevo (Encinal Gas Power Plant, TX) + 5 actualizaciones de fase
- Nuevo: Encinal Gas Power Plant (Webb County, TX) — acuerdo Corea del Sur-EE.UU. de 6.3GW, aún no confirmado (watch-list).
- Actualizaciones: Golden Triangle Polymers (comisionamiento/arranque inminente), Santa Cruz Copper Project (PFS 2026, box cut oct-2026), Stibnite Gold Project (avance de construcción 28-sep), Fermi America Project Matador (acuerdo O&M con NAES), Stargate Abilene Campus (pausa estatal TCEQ de permisos para data centers en Texas).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ae71eLABEqPVs1ixQhvtTM
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -416,8 +416,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -590,17 +599,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento) ; arranque ahora esperado en 2027 (retrasado al menos 6 meses respecto a 2026), según East Daley Analytics, por menor demanda de etano proyectada</t>
+          <t>Comisionamiento/arranque inminente (CEO de QatarEnergy, Saad al-Kaabi, declaró 20-sep-2026 en el Qatar Economic Forum que el complejo de US$8,500 millones "está iniciando comisionamiento y debería arrancar en las próximas semanas"; versión previa de East Daley Analytics estimaba arranque hasta 2027 por menor demanda de etano proyectada)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
+          <t>[MEES](https://www.mees.com/2026/9/25/corporate/qatarenergy-poised-to-start-up-texas-ethane-cracker/0ff02300-b8df-11f1-8f86-2b8776a66cca); [BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -792,106 +801,106 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Proyecto Escolín (amoniaco/urea)</t>
+          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Poza Rica, Veracruz, México</t>
+          <t>Lázaro Cárdenas, Michoacán, México</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mota-Engil México (EPC confirmado, US$1,200 millones, 47 meses); Duro Felguera (España) se integró formalmente 17-ago-2026 al contrato para gestión de proyecto y coordinación técnica de la ingeniería (supervisión de ingeniería externa, coordinación de suministros del tecnólogo, gestión de sistemas auxiliares); Casale (proveedor de tecnología)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ingeniería/inicio de construcción (inversión confirmada US$1,553 millones; capacidad objetivo &gt;700,000 ton/año de amoniaco, urea y AdBlue; citado explícitamente por la Presidenta Sheinbaum en su Segundo Informe de Gobierno —1-sep-2026— como parte del "rescate de la petroquímica" junto con Cosoleacaque, Morelos y Cangrejera)</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/); [El Español](https://www.elespanol.com/invertia/empresas/energia/20260817/duro-felguera-convoca-junta-extraordinaria-septiembre-aprobar-proyecto-clave-mota-engil-mexico/1003744355543_0.html); [La Política en Rosa](https://www.lapoliticaenrosa.com/2026/09/01/desde-veracruz-inicia-rescate-de-petroquimica-del-pais-destaca-claudia-sheinbaum-en-segundo-informe-de-gobierno/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
+          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas, Michoacán, México</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Transition Industries</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
+          <t>Construcción (colocación de primera piedra/groundbreaking simbólico 24-abr-2026; trabajos de ingeniería de campo y preparación de sitio iniciados en may-2026; inicio de construcción completa programado para finales de 2026; planta de metanol azul/ultra bajo carbono más grande del mundo, ~1.8 Mt/año metanol azul + 350,000 t/año ultra bajo carbono; operación esperada 2029-2030)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/); [BusinessWire](https://www.businesswire.com/news/home/20260423775301/en/Pacfico-Mexinol-Celebrates-the-Symbolic-Groundbreaking-in-Topolobampo-Positioning-Mexico-in-the-New-Low-Carbon-Chemical-Industry)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
+          <t>First Ammonia (amoniaco verde)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Victoria, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Transition Industries</t>
+          <t>First Ammonia / Cox Group USA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
+          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (colocación de primera piedra/groundbreaking simbólico 24-abr-2026; trabajos de ingeniería de campo y preparación de sitio iniciados en may-2026; inicio de construcción completa programado para finales de 2026; planta de metanol azul/ultra bajo carbono más grande del mundo, ~1.8 Mt/año metanol azul + 350,000 t/año ultra bajo carbono; operación esperada 2029-2030)</t>
+          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / inicio de construcción reprogramado para inicios de octubre de 2026 en el Puerto de Victoria, Texas (planta de 200 MW, fase 1); cierre financiero esperado antes de fin de 2026, operación comercial estimada 2029</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/); [BusinessWire](https://www.businesswire.com/news/home/20260423775301/en/Pacfico-Mexinol-Celebrates-the-Symbolic-Groundbreaking-in-Topolobampo-Positioning-Mexico-in-the-New-Low-Carbon-Chemical-Industry)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -903,165 +912,165 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>First Ammonia (amoniaco verde)</t>
+          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Victoria, Texas, EE.UU.</t>
+          <t>Topolobampo, Ahome, Sinaloa, México</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>First Ammonia / Cox Group USA</t>
+          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / inicio de construcción reprogramado para inicios de octubre de 2026 en el Puerto de Victoria, Texas (planta de 200 MW, fase 1); cierre financiero esperado antes de fin de 2026, operación comercial estimada 2029</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace, con protesta en el Zócalo) presionan por la cancelación del proyecto; GPO aceptó, como parte de las negociaciones, modificar la toma de agua —reubicándola al canal de residuos de CFE— y descargar la salmuera caliente fuera de la bahía de Ohuira, mientras mantiene pausadas las plantas de urea y metanol; sin resolución final reportada a la fecha)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/); [Bajo Palabra](https://www.bajopalabra.mx/sheinbaum-descarta-por-ahora-cancelar-megaplanta-de-amoniaco-en-topolobampo-ante-reclamos-ambientales/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
+          <t>Lake Charles Methanol II</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Topolobampo, Ahome, Sinaloa, México</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
+          <t>Lake Charles Methanol II LLC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Zachry Group (FEED)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace, con protesta en el Zócalo) presionan por la cancelación del proyecto; GPO aceptó, como parte de las negociaciones, modificar la toma de agua —reubicándola al canal de residuos de CFE— y descargar la salmuera caliente fuera de la bahía de Ohuira, mientras mantiene pausadas las plantas de urea y metanol; sin resolución final reportada a la fecha)</t>
+          <t>Ingeniería (FEED) / FID prevista</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/); [Bajo Palabra](https://www.bajopalabra.mx/sheinbaum-descarta-por-ahora-cancelar-megaplanta-de-amoniaco-en-topolobampo-ante-reclamos-ambientales/)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II</t>
+          <t>Planta Coquizadora Salina Cruz</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
+          <t>Salina Cruz, Oaxaca, México</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II LLC</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Zachry Group (FEED)</t>
+          <t>ICA Fluor</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / FID prevista</t>
+          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Planta Coquizadora Salina Cruz</t>
+          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Salina Cruz, Oaxaca, México</t>
+          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Shintech Louisiana, LLC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ICA Fluor</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
+          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
+          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
+          <t>Texas City, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Shintech Louisiana, LLC</t>
+          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1071,86 +1080,86 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
+          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
+          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Texas City, Texas, EE.UU.</t>
+          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
+          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Air Liquide (unidad propia); OXEA no especificado</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
+          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
+          <t>Targa Resources East Driver Gas Processing Plant</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
+          <t>Condado de Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Air Liquide (unidad propia); OXEA no especificado</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
+          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1162,32 +1171,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Targa Resources East Driver Gas Processing Plant</t>
+          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Condado de Midland, Texas, EE.UU.</t>
+          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
+          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1199,32 +1208,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
+          <t>MPLX Secretariat II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
+          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
+          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1236,12 +1245,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MPLX Secretariat II Gas Processing Plant</t>
+          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
+          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1256,12 +1265,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
+          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1273,32 +1282,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
+          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
+          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Northern Plains Nitrogen LLC</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>EPC no designado</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
+          <t>Pre-FEED completo / FID buscada 4T2026</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1310,54 +1319,54 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
+          <t>Iron Mesa (planta de gas)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
+          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen LLC</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EPC no designado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pre-FEED completo / FID buscada 4T2026</t>
+          <t>Construcción (arranque previsto Q1 2027)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Iron Mesa (planta de gas)</t>
+          <t>Yeti II (planta de gas)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Targa Resources</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1367,12 +1376,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Construcción (arranque previsto Q1 2027)</t>
+          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1384,32 +1393,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Yeti II (planta de gas)</t>
+          <t>Refinería Francisco I. Madero (rehabilitación)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Ciudad Madero, Tamaulipas, México</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Targa Resources</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
+          <t>Licitación/bidding</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1421,106 +1430,106 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Refinería Francisco I. Madero (rehabilitación)</t>
+          <t>Fermachem Planta de Urea/Amoniaco</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ciudad Madero, Tamaulipas, México</t>
+          <t>Ejido Sapioris, Lerdo, Durango, México</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Fermaca Dreams (Fermachem)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
+          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación/bidding</t>
+          <t>Construcción reanudada (obra había sido pausada por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento; gobernador Esteban Villegas confirmó 7-sep-2026 que la empresa cuenta con todos los permisos federales pese a objeciones del cabildo de Lerdo sobre permisos municipales; Sedeco Durango reafirmó 23-sep-2026 que el proyecto está "vigente al 100%" con todas las autorizaciones ambientales en regla; ya se completaron trabajos de compactación/preparación de 150 hectáreas en el ejido Sapioriz; construcción formal de la primera fase se proyecta en ~28 meses; inversión ~US$1,600 millones, capacidad 1 millón ton/año de urea granulada)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [El Siglo de Torreón — Canacintra](https://www.elsiglodetorreon.com.mx/noticia/2026/fermachem-es-un-proyecto-auditado-legal-y-mexicano-sin-almacenamiento-de-amoniaco-canacintra.html); [Grem Noticieros — Sedeco](https://www.noticierosgrem.com.mx/vigente-al-100-proyecto-de-planta-fermachem-en-lerdo-sedeco/); [El Siglo de Torreón — Gobernador](https://www.elsiglodetorreon.com.mx/noticia/2026/planta-de-fermachen-en-lerdo-va-mas-que-firme-gobernador-de-durango.html)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fermachem Planta de Urea/Amoniaco</t>
+          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ejido Sapioris, Lerdo, Durango, México</t>
+          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fermaca Dreams (Fermachem)</t>
+          <t>Clean Hydrogen Works</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
+          <t>McDermott (FEED)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Construcción reanudada (obra había sido pausada por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento; gobernador Esteban Villegas confirmó 7-sep-2026 que la empresa cuenta con todos los permisos federales pese a objeciones del cabildo de Lerdo sobre permisos municipales; Sedeco Durango reafirmó 23-sep-2026 que el proyecto está "vigente al 100%" con todas las autorizaciones ambientales en regla; ya se completaron trabajos de compactación/preparación de 150 hectáreas en el ejido Sapioriz; construcción formal de la primera fase se proyecta en ~28 meses; inversión ~US$1,600 millones, capacidad 1 millón ton/año de urea granulada)</t>
+          <t>Ingeniería (FEED) / Pre-FID</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [El Siglo de Torreón — Canacintra](https://www.elsiglodetorreon.com.mx/noticia/2026/fermachem-es-un-proyecto-auditado-legal-y-mexicano-sin-almacenamiento-de-amoniaco-canacintra.html); [Grem Noticieros — Sedeco](https://www.noticierosgrem.com.mx/vigente-al-100-proyecto-de-planta-fermachem-en-lerdo-sedeco/); [El Siglo de Torreón — Gobernador](https://www.elsiglodetorreon.com.mx/noticia/2026/planta-de-fermachen-en-lerdo-va-mas-que-firme-gobernador-de-durango.html)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
+          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Clean Hydrogen Works</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>McDermott (FEED)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / Pre-FID</t>
+          <t>Ingeniería (sancionado; en línea 2028)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1532,128 +1541,128 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
+          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
+          <t>Gothenburg, Nebraska, EE.UU.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ingeniería (sancionado; en línea 2028)</t>
+          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
+          <t>Wabash Low-Carbon Ammonia Project</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gothenburg, Nebraska, EE.UU.</t>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
+          <t>Wabash Valley Resources</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Wabash Low-Carbon Ammonia Project</t>
+          <t>Green Fuels Operating — Refinería Duncan</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>West Terre Haute, Indiana, EE.UU.</t>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Wabash Valley Resources</t>
+          <t>Green Fuels Operating</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Green Fuels Operating — Refinería Duncan</t>
+          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+          <t>Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Green Fuels Operating</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1663,34 +1672,34 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
+          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>ONEOK Inc.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1700,49 +1709,49 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
+          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
+          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
+          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ONEOK Inc.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
+          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
+          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1754,86 +1763,86 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
+          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
+          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
+          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
+          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
+          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
+          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1848,7 +1857,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1858,39 +1867,39 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1902,54 +1911,54 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Southern Energy Renewables</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+          <t>Richland, Washington, EE.UU.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables</t>
+          <t>Atlas Agro</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1959,145 +1968,145 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
+          <t>Hydrogen City (complejo Power-to-X / e-metanol / amoniaco verde)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Richland, Washington, EE.UU.</t>
+          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU. (corredor Corpus Christi–Brownsville; hub de ~50,000 acres)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Atlas Agro</t>
+          <t>Green Hydrogen International (GHI), en asociación con INPEX Corporation (Japón) para el componente de amoniaco</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>ABB (automatización/control, vía MOU)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
+          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; INPEX y GHI firmaron Joint Study Agreement para avanzar el componente de amoniaco verde de exportación —Fase 1: 280,000 ton/año de H2 verde para producir 1 millón ton/año de amoniaco verde, alimentado por 3.75 GW de renovables—, sin FID formal ni EPC adjudicado aún; construcción planeada desde 2026, primera producción de amoniaco estimada 2029, e-metanol 2030)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/renewable-sustainability-h2-esg/green-hydrogen-international-and-inpex-corporation-project-south-texas/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Hydrogen City (complejo Power-to-X / e-metanol / amoniaco verde)</t>
+          <t>Targa Resources Falcon II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU. (corredor Corpus Christi–Brownsville; hub de ~50,000 acres)</t>
+          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Green Hydrogen International (GHI), en asociación con INPEX Corporation (Japón) para el componente de amoniaco</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ABB (automatización/control, vía MOU)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; INPEX y GHI firmaron Joint Study Agreement para avanzar el componente de amoniaco verde de exportación —Fase 1: 280,000 ton/año de H2 verde para producir 1 millón ton/año de amoniaco verde, alimentado por 3.75 GW de renovables—, sin FID formal ni EPC adjudicado aún; construcción planeada desde 2026, primera producción de amoniaco estimada 2029, e-metanol 2030)</t>
+          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/renewable-sustainability-h2-esg/green-hydrogen-international-and-inpex-corporation-project-south-texas/)</t>
+          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Targa Resources Falcon II Gas Processing Plant</t>
+          <t>Cassidy II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
+          <t>Condado de Glasscock, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Brazos Midstream</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
+          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cassidy II Gas Processing Plant</t>
+          <t>Kings Landing II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Condado de Glasscock, Texas, EE.UU.</t>
+          <t>Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Brazos Midstream</t>
+          <t>Kinetik Holdings</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2107,34 +2116,34 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
+          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
+          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kings Landing II Gas Processing Plant</t>
+          <t>Apollo Gas Plant</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Nuevo México, EE.UU.</t>
+          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Kinetik Holdings</t>
+          <t>Trace Midstream Partners II</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2144,12 +2153,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
+          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
+          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2161,17 +2170,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Apollo Gas Plant</t>
+          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
+          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Trace Midstream Partners II</t>
+          <t>IGP Methanol LLC</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2181,12 +2190,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
+          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
+          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2198,91 +2207,91 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
+          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
+          <t>Culbertson, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>IGP Methanol LLC</t>
+          <t>Cyan H2</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
+          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
+          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
+          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Culbertson, Montana, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Cyan H2</t>
+          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
+          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
+          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
+          <t>México Amoníaco y Urea (MAYU)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
+          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
+          <t>México Amoníaco y Urea (desarrollador privado)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2292,34 +2301,34 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
+          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
+          <t>[MAYU](https://mayu.com.mx/en/)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (MAYU)</t>
+          <t>Ampliación Terminal de Exportación NGL Nederland</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
+          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (desarrollador privado)</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2329,34 +2338,34 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
+          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>[MAYU](https://mayu.com.mx/en/)</t>
+          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ampliación Terminal de Exportación NGL Nederland</t>
+          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
+          <t>El Dorado, Arkansas, EE.UU.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>LSB Industries</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2366,34 +2375,34 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
+          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
+          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
+          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>El Dorado, Arkansas, EE.UU.</t>
+          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LSB Industries</t>
+          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2403,12 +2412,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
+          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
+          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2420,91 +2429,91 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
+          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
+          <t>Tuscola, Illinois, EE.UU.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
+          <t>Cronus Chemicals LLC</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
+          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
+          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
+          <t>CHS/OCP North America — Planta de Fertilizante Fosfatado</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Tuscola, Illinois, EE.UU.</t>
+          <t>Cornerstone Energy Park, Waggaman, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Cronus Chemicals LLC</t>
+          <t>CHS Inc. / OCP North America (JV 50/50)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
+          <t>Planeación/pre-construcción (JV anunciada 26-ago-2026 en ceremonia con la Secretaria de Agricultura de EE.UU., Brooke Rollins; sería la primera planta nueva de fertilizante fosfatado construida en EE.UU. desde 1984; capacidad hasta 1.3 millones ton/año, inversión hasta US$450 millones; solicitud de financiamiento presentada al programa USDA FIELDS; construcción prevista antes de fin de 2026, producción posible a fines de 2028)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
+          <t>[CHS Inc.](https://www.chsinc.com/news-and-stories/2026/08/26/chs-ocp-domestic-fertilizer-production-announcement); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/chs-ocp-plan-up-to-450m-louisiana-fertilizer-plant/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CHS/OCP North America — Planta de Fertilizante Fosfatado</t>
+          <t>CITGO Lake Charles Refinery — Depentanizer Project (mejora de naphtha upgrading)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cornerstone Energy Park, Waggaman, Luisiana, EE.UU.</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CHS Inc. / OCP North America (JV 50/50)</t>
+          <t>CITGO Petroleum Corporation</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2514,52 +2523,15 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (JV anunciada 26-ago-2026 en ceremonia con la Secretaria de Agricultura de EE.UU., Brooke Rollins; sería la primera planta nueva de fertilizante fosfatado construida en EE.UU. desde 1984; capacidad hasta 1.3 millones ton/año, inversión hasta US$450 millones; solicitud de financiamiento presentada al programa USDA FIELDS; construcción prevista antes de fin de 2026, producción posible a fines de 2028)</t>
+          <t>Aprobado/Ingeniería (proyecto de US$310 millones aprobado 1-sep-2026; agrega instalaciones y equipo para mejorar el upgrading de nafta, convirtiendo corrientes de menor valor en componentes de gasolina de mayor valor; entrada en operación prevista 2029)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[CHS Inc.](https://www.chsinc.com/news-and-stories/2026/08/26/chs-ocp-domestic-fertilizer-production-announcement); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/chs-ocp-plan-up-to-450m-louisiana-fertilizer-plant/)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/09/citgo-to-invest-310-mm-to-improve-naphtha-upgrading-at-lake-charles-refinery-us/); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/citgo-strengthens-lake-charles-refinerys-future-with-310-million-project/)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>CITGO Lake Charles Refinery — Depentanizer Project (mejora de naphtha upgrading)</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>CITGO Petroleum Corporation</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Aprobado/Ingeniería (proyecto de US$310 millones aprobado 1-sep-2026; agrega instalaciones y equipo para mejorar el upgrading de nafta, convirtiendo corrientes de menor valor en componentes de gasolina de mayor valor; entrada en operación prevista 2029)</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/09/citgo-to-invest-310-mm-to-improve-naphtha-upgrading-at-lake-charles-refinery-us/); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/citgo-strengthens-lake-charles-refinerys-future-with-310-million-project/)</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
@@ -2578,6 +2550,15 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4403,8 +4384,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4466,17 +4456,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins; excavación del box-cut programada para 3T2026</t>
+          <t>Construcción (Estudio de Prefactibilidad —PFS— 2026 publicado 23-sep-2026: capex inicial elevado a US$1,430 millones, costo operativo US$1.47/lb, VPN después de impuestos US$3,500 millones, TIR 30%; mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; "box cut" —corte de acceso a la mina— previsto para iniciar octubre 2026; carta preliminar de US$1,100 millones del Export-Import Bank de EE.UU., aprobación final esperada primavera 2027; primera producción de cátodo de cobre prevista 2029) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/) ; [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
+          <t>[Ivanhoe Electric — PFS 2026](https://ivanhoeelectric.com/news/2026-preliminary-feasibility-study-for-the-santa-cruz-copper-project-in-arizona-confirms-high-grade-low-cost-project-with-strong-economics/); [Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -4873,17 +4863,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Directorio del Export-Import Bank de EE.UU. aprobó por unanimidad, 20-ago-2026, el préstamo garantizado senior de USD 2,900 millones para financiar el desarrollo; Corte Federal de Distrito de Idaho confirmó 18-ago-2026 la mayoría de las aprobaciones federales del USFS, aunque encontró insuficientes las declaraciones de captura incidental para carcayú y trucha toro, lo que motivó una apelación ante el Noveno Circuito presentada ~25-ago-2026 por una coalición conservacionista —la Tribu Nez Perce mantiene demanda separada—, sin que ello detenga la obra; actualización de construcción del 31-ago-2026 reporta fabricación/enrolado en Europa de los componentes del doble autoclave y avance ~50% en la entrega de módulos de vivienda permanente para trabajadores —ATCO—, con primer oro previsto 2029)</t>
+          <t>Construcción (actualización de construcción y exploración del 28-sep-2026 confirma actividades activas de "critical path": ruta Burntlog, vivienda para trabajadores, desarrollo de infraestructura de línea de transmisión; postes de energía y equipo auxiliar ya entregados en los patios de acopio —laydown areas— de Donnelly y Cascade, Idaho; permisos federales asegurados desde 2025; corte federal de Idaho negó en jun-2026 moción para detener obras; EXIM Bank aprobó 20-ago-2026 préstamo garantizado senior de USD 2,900 millones; apelación ante el Noveno Circuito sobre declaraciones de captura incidental —presentada ~25-ago-2026— continúa sin detener la obra; primer oro previsto 2029)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html); [Northern Miner](https://www.northernminer.com/news/court-ruling-backs-perpetuas-1-3b-stibnite-build/1003894465/); [PRNewswire](https://www.prnewswire.com/news-releases/perpetua-resources-provides-construction-update-on-the-stibnite-gold-project-and-exploration-activities-302864546.html); [Center for Biological Diversity](https://biologicaldiversity.org/w/news/press-releases/appeal-targets-federal-approval-of-massive-idaho-gold-mine-2026-08-25/)</t>
+          <t>[PR Newswire — actualización 28-sep-2026](https://www.prnewswire.com/news-releases/perpetua-resources-provides-construction--exploration-update-302891031.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html); [Northern Miner](https://www.northernminer.com/news/court-ruling-backs-perpetuas-1-3b-stibnite-build/1003894465/); [Center for Biological Diversity](https://biologicaldiversity.org/w/news/press-releases/appeal-targets-federal-approval-of-massive-idaho-gold-mine-2026-08-25/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -7147,12 +7137,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Angangueo</t>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Angangueo, Michoacán, México</t>
+          <t>Empalme, Sonora, México</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -7167,7 +7157,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos con gobierno federal)</t>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -7184,17 +7174,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Chalchihuites</t>
+          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Chalchihuites, Zacatecas, México</t>
+          <t>Condado de Coosa, Alabama, EE.UU.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Westwater Resources Inc.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7204,34 +7194,34 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Modernización Complejo Metalúrgico Empalme</t>
+          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Empalme, Sonora, México</t>
+          <t>Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Global Advanced Metals</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7241,34 +7231,34 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
+          <t>Boron Americas Project (Fort Cady)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Condado de Coosa, Alabama, EE.UU.</t>
+          <t>California, EE.UU.</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Westwater Resources Inc.</t>
+          <t>5E Advanced Materials</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7278,12 +7268,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -7295,54 +7285,54 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
+          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Pensilvania, EE.UU.</t>
+          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Global Advanced Metals</t>
+          <t>Ramaco Resources</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
+          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Boron Americas Project (Fort Cady)</t>
+          <t>Dewey-Burdock Uranium ISR Project</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>California, EE.UU.</t>
+          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>5E Advanced Materials</t>
+          <t>enCore Energy (Powertech USA)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7352,71 +7342,71 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
+          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
+          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
+          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ramaco Resources</t>
+          <t>Niron Magnetics</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
+          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
+          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Dewey-Burdock Uranium ISR Project</t>
+          <t>Louisiana Strategic Metals Complex</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
+          <t>Alexandria, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>enCore Energy (Powertech USA)</t>
+          <t>Ucore Rare Metals Inc.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7426,34 +7416,34 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
+          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
+          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
+          <t>Distrito Copper Creek / San Manuel</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
+          <t>Condado de Pinal, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Niron Magnetics</t>
+          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7463,71 +7453,71 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
+          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
+          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Louisiana Strategic Metals Complex</t>
+          <t>IMA Mine</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Alexandria, Luisiana, EE.UU.</t>
+          <t>Condado de Lemhi, Idaho, EE.UU.</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Ucore Rare Metals Inc.</t>
+          <t>American Tungsten Corp.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
+          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
+          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Distrito Copper Creek / San Manuel</t>
+          <t>Railroad Valley Minerals / Super-Brine Complex</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Condado de Pinal, Arizona, EE.UU.</t>
+          <t>Railroad Valley, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
+          <t>3 Proton Lithium (3PL Operating Inc.)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -7537,12 +7527,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
+          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
+          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -7554,32 +7544,32 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IMA Mine</t>
+          <t>New Amalga Gold Project</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Condado de Lemhi, Idaho, EE.UU.</t>
+          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>American Tungsten Corp.</t>
+          <t>Grande Portage Resources Ltd.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
+          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -7591,17 +7581,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Railroad Valley Minerals / Super-Brine Complex</t>
+          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Railroad Valley, Nevada, EE.UU.</t>
+          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>3 Proton Lithium (3PL Operating Inc.)</t>
+          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7611,71 +7601,71 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
+          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
+          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>New Amalga Gold Project</t>
+          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
+          <t>Marion, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Grande Portage Resources Ltd.</t>
+          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
+          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
+          <t>La Preciosa Project</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
+          <t>Durango, México</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -7685,71 +7675,71 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
+          <t>Great Salt Lake Lithium Facility</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Marion, Indiana, EE.UU.</t>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>La Preciosa Project</t>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Durango, México</t>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+          <t>Nth Cycle, Inc.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -7759,49 +7749,49 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Great Salt Lake Lithium Facility</t>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Condado de Box Elder, Utah, EE.UU.</t>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -7813,106 +7803,106 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+          <t>Copperwood Project</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Nth Cycle, Inc.</t>
+          <t>Highland Copper Company</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>DRA Americas Inc. (FEED)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+          <t>Modernización Refinería de Cobre El Paso</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
+          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Copperwood Project</t>
+          <t>Round Top Rare Earth Project</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
+          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Highland Copper Company</t>
+          <t>USA Rare Earth Inc.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>DRA Americas Inc. (FEED)</t>
+          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
+          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -7924,32 +7914,32 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Modernización Refinería de Cobre El Paso</t>
+          <t>Expansión Fundición de Antimonio Thompson Falls</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Thompson Falls, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>United States Antimony Corporation (USAC)</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
+          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
+          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -7961,32 +7951,32 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Round Top Rare Earth Project</t>
+          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
+          <t>Morenci, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>USA Rare Earth Inc.</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
+          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
+          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -7998,17 +7988,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Expansión Fundición de Antimonio Thompson Falls</t>
+          <t>Reconstrucción Fundición y Refinería Kennecott</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Thompson Falls, Montana, EE.UU.</t>
+          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>United States Antimony Corporation (USAC)</t>
+          <t>Rio Tinto (Kennecott Utah Copper)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8018,12 +8008,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
+          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
+          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8035,32 +8025,32 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
+          <t>Fourmile (decline Bullion Hill)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Morenci, Arizona, EE.UU.</t>
+          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
+          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -8072,17 +8062,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Reconstrucción Fundición y Refinería Kennecott</t>
+          <t>Puerto del Aire (distrito Mulatos)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Rio Tinto (Kennecott Utah Copper)</t>
+          <t>Alamos Gold Inc.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8092,12 +8082,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
+          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
+          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -8109,54 +8099,54 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Fourmile (decline Bullion Hill)</t>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
+          <t>Clarksville, Tennessee, EE.UU.</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Puerto del Aire (distrito Mulatos)</t>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Alamos Gold Inc.</t>
+          <t>Aclara Resources Inc.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8166,34 +8156,34 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+          <t>Archimedes Project (i-80 Gold)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Clarksville, Tennessee, EE.UU.</t>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+          <t>i-80 Gold Corp</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8203,12 +8193,12 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -8220,17 +8210,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Aclara Heavy Rare Earth Separation Facility</t>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Aclara Resources Inc.</t>
+          <t>Sweetwater Uranium, Inc.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8240,12 +8230,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -8257,17 +8247,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Archimedes Project (i-80 Gold)</t>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+          <t>San Juan County, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>i-80 Gold Corp</t>
+          <t>Anfield Energy Inc.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8277,12 +8267,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -8294,350 +8284,350 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+          <t>Twin Metals Minnesota</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Sweetwater County, Wyoming, EE.UU.</t>
+          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium, Inc.</t>
+          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+          <t>Permitting/Pre-EIS con retroceso regulatorio (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026 mediante orden ejecutiva que prohíbe minería no ferrosa en la cuenca del Rainy River Headwaters; el DNR de Minnesota canceló uno de los arrendamientos minerales de Twin Metals cerca de Babbitt por incumplimiento de requisitos de desempeño/producción, anunciado 14-sep-2026 y efectivo 10-nov-2026; grupos ambientalistas lo ven como precedente para cancelar los arrendamientos restantes; proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242); [KAXE](https://www.kaxe.org/local-news/2026-09-14/dnr-cancels-1-twin-metals-mineral-lease-near-babbitt); [Voyageurs Conservancy](https://www.voyageurs.org/news/2026/9/22/what-the-walz-order-and-the-twin-metals-lease-cancellation-mean-for-voyageurs)</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Velvet-Wood Uranium-Vanadium Project</t>
+          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>San Juan County, Utah, EE.UU.</t>
+          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Anfield Energy Inc.</t>
+          <t>Falcon Copper Corp. (MOU con Glencore)</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Twin Metals Minnesota</t>
+          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
+          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
+          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>Metso Finland Oy (estudio de alcance)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS con retroceso regulatorio (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026 mediante orden ejecutiva que prohíbe minería no ferrosa en la cuenca del Rainy River Headwaters; el DNR de Minnesota canceló uno de los arrendamientos minerales de Twin Metals cerca de Babbitt por incumplimiento de requisitos de desempeño/producción, anunciado 14-sep-2026 y efectivo 10-nov-2026; grupos ambientalistas lo ven como precedente para cancelar los arrendamientos restantes; proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242); [KAXE](https://www.kaxe.org/local-news/2026-09-14/dnr-cancels-1-twin-metals-mineral-lease-near-babbitt); [Voyageurs Conservancy](https://www.voyageurs.org/news/2026/9/22/what-the-walz-order-and-the-twin-metals-lease-cancellation-mean-for-voyageurs)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
+          <t>Spring Valley Gold Mine</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
+          <t>Condado de Pershing, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Falcon Copper Corp. (MOU con Glencore)</t>
+          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
+          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
+          <t>Pitarrilla Project (plata-plomo-zinc)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
+          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
+          <t>Endeavour Silver Corp.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Metso Finland Oy (estudio de alcance)</t>
+          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
+          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Spring Valley Gold Mine</t>
+          <t>Red Dog Mine Life Extension Project</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Condado de Pershing, Nevada, EE.UU.</t>
+          <t>Distrito Minero de NANA, noroeste de Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
+          <t>Teck American Incorporated (Teck Resources), en tierras de NANA Regional Corporation</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>U.S. Army Corps of Engineers (agencia líder de permisos)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
+          <t>Prefactibilidad (estudio en curso; Teck destina US$200-250 millones en 2026 a obras tempranas —camino de acceso todo-el-año, perforación— y avance del estudio de prefactibilidad; minado subterráneo por realces largos (long-hole stoping) propuesto para los yacimientos Aktigiruq y Anarraaq, alimentando el molino existente de Red Dog; minerales: zinc, plomo, plata, germanio; proyecto obtuvo cobertura FAST-41 en sep-2026)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
+          <t>[Permitting.gov](https://www.permitting.gov/newsroom/press-releases/red-dog-mine-life-extension-project-gains-fast-41-coverage); [Mining News North](https://www.miningnewsnorth.com/story/2026/09/04/news/red-dog-extension-gains-fast-41-permitting/9851.html)</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Pitarrilla Project (plata-plomo-zinc)</t>
+          <t>Kings Mountain Lithium Material Processing Plant</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
+          <t>Kings Mountain, Carolina del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Endeavour Silver Corp.</t>
+          <t>Albemarle Corporation</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
+          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión; DOE anunció 14-sep-2026 US$16 millones adicionales para programas de educación minera durante visita al sitio —14 escuelas mineras acreditadas—; proyecto sigue a la espera de permisos estatales y locales, tajo ya drenado)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
+          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf); [WFAE](https://www.wfae.org/energy-environment/2026-09-14/trump-administration-announces-16-million-for-mining-education-at-kings-mountain-lithium-site)</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Red Dog Mine Life Extension Project</t>
+          <t>Tonopah Flats Lithium Project</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Distrito Minero de NANA, noroeste de Alaska, EE.UU.</t>
+          <t>Condados de Esmeralda y Nye, Nevada, EE.UU. (~11 km al noroeste de Tonopah)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Teck American Incorporated (Teck Resources), en tierras de NANA Regional Corporation</t>
+          <t>American Battery Technology Company (ABTC)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>U.S. Army Corps of Engineers (agencia líder de permisos)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Prefactibilidad (estudio en curso; Teck destina US$200-250 millones en 2026 a obras tempranas —camino de acceso todo-el-año, perforación— y avance del estudio de prefactibilidad; minado subterráneo por realces largos (long-hole stoping) propuesto para los yacimientos Aktigiruq y Anarraaq, alimentando el molino existente de Red Dog; minerales: zinc, plomo, plata, germanio; proyecto obtuvo cobertura FAST-41 en sep-2026)</t>
+          <t>Permitting (BLM aceptó formalmente el Plan of Operations de mina y refinería el 8-sep-2026, hito mayor hacia autorización NEPA; proyecto usa proceso propietario de lixiviación selectiva —SLE—; recurso estimado de 21.3 millones de toneladas de hidróxido de litio monohidratado accesible; mina y refinería en pleno desarrollo proyectadas a producir hasta 30,000 t/año de hidróxido de litio, ~1,300 empleos de construcción)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>[Permitting.gov](https://www.permitting.gov/newsroom/press-releases/red-dog-mine-life-extension-project-gains-fast-41-coverage); [Mining News North](https://www.miningnewsnorth.com/story/2026/09/04/news/red-dog-extension-gains-fast-41-permitting/9851.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/08/3357682/0/en/american-battery-technology-company-achieves-major-milestone-with-u-s-blm-acceptance-of-plan-of-operations-for-tonopah-flats-lithium-project.html); [Mining Technology](https://www.mining-technology.com/projects/tonopah-flats-lithium-project-us/)</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Kings Mountain Lithium Material Processing Plant</t>
+          <t>Angel Island Lithium Project</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Kings Mountain, Carolina del Norte, EE.UU.</t>
+          <t>Esmeralda County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Albemarle Corporation</t>
+          <t>Century Lithium Corp.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Fluor Corporation</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión; DOE anunció 14-sep-2026 US$16 millones adicionales para programas de educación minera durante visita al sitio —14 escuelas mineras acreditadas—; proyecto sigue a la espera de permisos estatales y locales, tajo ya drenado)</t>
+          <t>Permitting (presentó Plan de Operaciones Minero y solicitud de Permiso de Reclamación de Nevada ante BLM el 3-sep-2026; proyecto bajo programa FAST-41; meta de completar permisos federales para feb-2028)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf); [WFAE](https://www.wfae.org/energy-environment/2026-09-14/trump-administration-announces-16-million-for-mining-education-at-kings-mountain-lithium-site)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/CYDVF/century-lithium-files-mine-plan-of-operations-for-angel-island-0v6ql6hprbzu.html)</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Tonopah Flats Lithium Project</t>
+          <t>Silver Peak Lithium Mine (Expansión)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Condados de Esmeralda y Nye, Nevada, EE.UU. (~11 km al noroeste de Tonopah)</t>
+          <t>Esmeralda County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>American Battery Technology Company (ABTC)</t>
+          <t>Albemarle Corporation</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -8647,49 +8637,49 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Permitting (BLM aceptó formalmente el Plan of Operations de mina y refinería el 8-sep-2026, hito mayor hacia autorización NEPA; proyecto usa proceso propietario de lixiviación selectiva —SLE—; recurso estimado de 21.3 millones de toneladas de hidróxido de litio monohidratado accesible; mina y refinería en pleno desarrollo proyectadas a producir hasta 30,000 t/año de hidróxido de litio, ~1,300 empleos de construcción)</t>
+          <t>Permitting completo (BLM completó el permitting federal el 27-feb-2026; autorizada operación/expansión en 8,058 acres; incluye construcción de 2 estaciones de bombeo, 2 piscinas de salmuera y tuberías de proceso)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/08/3357682/0/en/american-battery-technology-company-achieves-major-milestone-with-u-s-blm-acceptance-of-plan-of-operations-for-tonopah-flats-lithium-project.html); [Mining Technology](https://www.mining-technology.com/projects/tonopah-flats-lithium-project-us/)</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-silver-peak-lithium-mine-expansion); [Permitting.gov](https://www.permitting.gov/newsroom/press-releases/silver-peak-lithium-mine-project-completes-federal-permitting)</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Angel Island Lithium Project</t>
+          <t>McDermitt Lithium Project (lado Jindalee)</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Esmeralda County, Nevada, EE.UU.</t>
+          <t>Condado de Malheur, Oregón (límite con Nevada), EE.UU.</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Century Lithium Corp.</t>
+          <t>Jindalee Lithium (ASX:JLL / OTCQX:JNDAF)</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (contratista de perforación contratado)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Permitting (presentó Plan de Operaciones Minero y solicitud de Permiso de Reclamación de Nevada ante BLM el 3-sep-2026; proyecto bajo programa FAST-41; meta de completar permisos federales para feb-2028)</t>
+          <t>Exploración (permiso estatal de Oregón obtenido para perforación; inicio de perforación de Fase 1 de exploración contratado para sep-2026; etapa muy temprana)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/CYDVF/century-lithium-files-mine-plan-of-operations-for-angel-island-0v6ql6hprbzu.html)</t>
+          <t>[Kalkine](https://kalkine.com.au/news/announcements/jindalee-lithium-secures-state-permit-for-mcdermitt-drilling-program-contractor-engaged-for-september-2026-start)</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -8701,32 +8691,32 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Silver Peak Lithium Mine (Expansión)</t>
+          <t>Burke Hollow ISR Uranium Project</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Esmeralda County, Nevada, EE.UU.</t>
+          <t>Sur de Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Albemarle Corporation</t>
+          <t>Uranium Energy Corp (UEC)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (operación propia, ISR)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Permitting completo (BLM completó el permitting federal el 27-feb-2026; autorizada operación/expansión en 8,058 acres; incluye construcción de 2 estaciones de bombeo, 2 piscinas de salmuera y tuberías de proceso)</t>
+          <t>Producción (iniciada abr-2026; primera mina ISR nueva en EE.UU. en más de una década; procesa vía Hobson Central Processing Plant bajo modelo hub-and-spoke; expansión continua con nuevos "spokes" satélite en desarrollo en el cinturón de uranio de Texas — infraestructura de tuberías de proceso en expansión activa)</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/press-release/blm-approves-silver-peak-lithium-mine-expansion); [Permitting.gov](https://www.permitting.gov/newsroom/press-releases/silver-peak-lithium-mine-project-completes-federal-permitting)</t>
+          <t>[ANS Nuclear Newswire](https://www.ans.org/news/2026-04-17/article-7945/uranium-energy-corp-begins-production-at-burke-hollow/)</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -8738,32 +8728,32 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>McDermitt Lithium Project (lado Jindalee)</t>
+          <t>Sage Plain Potash Project</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Condado de Malheur, Oregón (límite con Nevada), EE.UU.</t>
+          <t>San Juan County, Utah (cuenca Paradox), EE.UU.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Jindalee Lithium (ASX:JLL / OTCQX:JNDAF)</t>
+          <t>Sage Potash Corp / Critical Mineral Co.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>No especificado (contratista de perforación contratado)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Exploración (permiso estatal de Oregón obtenido para perforación; inicio de perforación de Fase 1 de exploración contratado para sep-2026; etapa muy temprana)</t>
+          <t>Prefactibilidad (avanzando hacia estudio de factibilidad, jun-2026; recibió subvención USDA de US$14 millones —Fertilizer Production Expansion Program—; meta de 300,000 t/año de potasa)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>[Kalkine](https://kalkine.com.au/news/announcements/jindalee-lithium-secures-state-permit-for-mcdermitt-drilling-program-contractor-engaged-for-september-2026-start)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/sage-plain-potash-project-usda-grant/); [Streetwise Reports](https://www.streetwisereports.com/article/2026/06/24/critical-mineral-co-advances-high-grade-utah-potash-project-toward-feasibility.html)</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -8775,32 +8765,32 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Burke Hollow ISR Uranium Project</t>
+          <t>Ann Mason Copper-Molybdenum Project</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sur de Texas, EE.UU.</t>
+          <t>Yerington, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Uranium Energy Corp (UEC)</t>
+          <t>Hudbay Minerals (vía Mason Resources)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>No especificado (operación propia, ISR)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Producción (iniciada abr-2026; primera mina ISR nueva en EE.UU. en más de una década; procesa vía Hobson Central Processing Plant bajo modelo hub-and-spoke; expansión continua con nuevos "spokes" satélite en desarrollo en el cinturón de uranio de Texas — infraestructura de tuberías de proceso en expansión activa)</t>
+          <t>Evaluación Económica Preliminar (PEA) avanzada; 4° depósito porfídico de cobre más grande de Norteamérica; vida de mina de 21 años proyectada; aún no en permisos/construcción formal</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>[ANS Nuclear Newswire](https://www.ans.org/news/2026-04-17/article-7945/uranium-energy-corp-begins-production-at-burke-hollow/)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/projects/ann-mason-copper-molybdenum-project-nevada/)</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -8812,17 +8802,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Sage Plain Potash Project</t>
+          <t>Fresnillo — Portafolio próxima generación (Rodeo, Tajitos, Guanajuato Sur, Novador)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>San Juan County, Utah (cuenca Paradox), EE.UU.</t>
+          <t>Sonora y Guanajuato, México (varias ubicaciones)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Sage Potash Corp / Critical Mineral Co.</t>
+          <t>Fresnillo plc</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -8832,12 +8822,12 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Prefactibilidad (avanzando hacia estudio de factibilidad, jun-2026; recibió subvención USDA de US$14 millones —Fertilizer Production Expansion Program—; meta de 300,000 t/año de potasa)</t>
+          <t>Exploración/prefactibilidad/ingeniería temprana (anunciado 7-sep-2026; Tajitos: capex preliminar US$400-450M, proyecto brownfield junto a Herradura, Sonora; Rodeo: PEA revisada, ~90-110k oz Au/año, arranque fin-2029/2030 sujeto a permisos; Guanajuato Sur: 15-17M oz Ag/año desde ~2033; Novador: ~200k oz Au/año potencial; etapa muy temprana, solo para monitoreo)</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/sage-plain-potash-project-usda-grant/); [Streetwise Reports](https://www.streetwisereports.com/article/2026/06/24/critical-mineral-co-advances-high-grade-utah-potash-project-toward-feasibility.html)</t>
+          <t>[MineAcademy](https://mineacademy.mx/fresnillo-plc-fortalece-su-cartera-de-proyectos-para-sostener-el-crecimiento-de-largo-plazo/)</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -8849,17 +8839,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Ann Mason Copper-Molybdenum Project</t>
+          <t>Reina del Cobre (proyecto polimetálico)</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Yerington, Nevada, EE.UU.</t>
+          <t>Cuencamé, Durango, México (junto a Velardeña)</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Hudbay Minerals (vía Mason Resources)</t>
+          <t>Industrias Peñoles</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -8869,12 +8859,12 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Evaluación Económica Preliminar (PEA) avanzada; 4° depósito porfídico de cobre más grande de Norteamérica; vida de mina de 21 años proyectada; aún no en permisos/construcción formal</t>
+          <t>Exploración (11,071 m perforados en 16 barrenos completos, ago-2026; recursos inferidos ~28.8-30 Mt @ ~2.0% CuEq; estudio económico preliminar planeado; etapa muy temprana)</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/projects/ann-mason-copper-molybdenum-project-nevada/)</t>
+          <t>[Milenio](https://www.milenio.com/estados/mina-velardena-pieza-clave-produccion-zinc-penoles)</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -8886,17 +8876,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Fresnillo — Portafolio próxima generación (Rodeo, Tajitos, Guanajuato Sur, Novador)</t>
+          <t>Springer Tungsten Complex</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sonora y Guanajuato, México (varias ubicaciones)</t>
+          <t>Imlay, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Fresnillo plc</t>
+          <t>Blue Moon Metals Inc. (mina y molino) / JV planta APT: The Elmet Group (70%), Blue Moon Metals (20%), EQ Resources (10%)</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -8906,34 +8896,34 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Exploración/prefactibilidad/ingeniería temprana (anunciado 7-sep-2026; Tajitos: capex preliminar US$400-450M, proyecto brownfield junto a Herradura, Sonora; Rodeo: PEA revisada, ~90-110k oz Au/año, arranque fin-2029/2030 sujeto a permisos; Guanajuato Sur: 15-17M oz Ag/año desde ~2033; Novador: ~200k oz Au/año potencial; etapa muy temprana, solo para monitoreo)</t>
+          <t>Reactivación anunciada (inversión US$150-175 millones, 11-14-sep-2026: mina open-pit + subterránea, molino de 1,200 tpd, y planta de paratungstato de amonio —APT— hasta 4,000 ton/año; Departamento de Guerra de EE.UU. comprometió US$450 millones adicionales a The Elmet Group, 14-sep-2026, para asegurar cadena de suministro de tungsteno; reinicio mina/molino previsto Q4 2027, planta APT H2 2028)</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>[MineAcademy](https://mineacademy.mx/fresnillo-plc-fortalece-su-cartera-de-proyectos-para-sostener-el-crecimiento-de-largo-plazo/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/blue-moon-the-elmet-group-and-eq-resources-announce-a-us150-175-million-investment-into-the-springer-tungsten-complex-nevada-to-strengthen-the-us-tungsten-supply-chain-302877075.html); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/14/3360841/0/en/department-of-war-makes-landmark-450-million-committed-investment-in-the-elmet-group-to-secure-america-s-tungsten-supply-chain.html)</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Reina del Cobre (proyecto polimetálico)</t>
+          <t>Sunshine Complex (Molino, Refinería Plata-Cobre y Planta de Antimonio)</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Cuencamé, Durango, México (junto a Velardeña)</t>
+          <t>Kellogg, Idaho (Silver Valley), EE.UU.</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Industrias Peñoles</t>
+          <t>Sunshine Silver Mining &amp; Refining Co.</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -8943,12 +8933,12 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Exploración (11,071 m perforados en 16 barrenos completos, ago-2026; recursos inferidos ~28.8-30 Mt @ ~2.0% CuEq; estudio económico preliminar planeado; etapa muy temprana)</t>
+          <t>Estudios de factibilidad en curso (desmantelación del molino existente para construir uno nuevo, a completarse fin de 2026; estudios de factibilidad para reabrir la Refinería Plata-Cobre y construir una nueva Planta de Antimonio —hasta 34.5 millones lb/año—, entrega prevista inicios de 2027; estudio de factibilidad de la mina concluye Q2 2027; meta de reinicio de producción de plata fin de 2028)</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>[Milenio](https://www.milenio.com/estados/mina-velardena-pieza-clave-produccion-zinc-penoles)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/sunshine-silver-mining--refining-reports-second-quarter-2026-results-302850131.html); [World Energy](https://www.world-energy.org/article/54143.html)</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -8960,17 +8950,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Springer Tungsten Complex</t>
+          <t>USA Rare Earth — Planta de Metal y Magnetos Blacksburg</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Imlay, Nevada, EE.UU.</t>
+          <t>Blacksburg, Carolina del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Blue Moon Metals Inc. (mina y molino) / JV planta APT: The Elmet Group (70%), Blue Moon Metals (20%), EQ Resources (10%)</t>
+          <t>USA Rare Earth (recién fusionada con Serra Verde Group, anunciado 4-sep-2026)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -8980,34 +8970,34 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Reactivación anunciada (inversión US$150-175 millones, 11-14-sep-2026: mina open-pit + subterránea, molino de 1,200 tpd, y planta de paratungstato de amonio —APT— hasta 4,000 ton/año; Departamento de Guerra de EE.UU. comprometió US$450 millones adicionales a The Elmet Group, 14-sep-2026, para asegurar cadena de suministro de tungsteno; reinicio mina/molino previsto Q4 2027, planta APT H2 2028)</t>
+          <t>Construcción (groundbreaking 9-sep-2026; inversión ~US$1,200 millones; ~490 empleos; planta de metal y manufactura de magnetos de tierras raras)</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/blue-moon-the-elmet-group-and-eq-resources-announce-a-us150-175-million-investment-into-the-springer-tungsten-complex-nevada-to-strengthen-the-us-tungsten-supply-chain-302877075.html); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/14/3360841/0/en/department-of-war-makes-landmark-450-million-committed-investment-in-the-elmet-group-to-secure-america-s-tungsten-supply-chain.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/09/3358813/0/en/usa-rare-earth-breaks-ground-on-advanced-rare-earth-metal-and-magnet-manufacturing-facility-in-blacksburg-south-carolina.html)</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Sunshine Complex (Molino, Refinería Plata-Cobre y Planta de Antimonio)</t>
+          <t>La Negra Project (expansión)</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Kellogg, Idaho (Silver Valley), EE.UU.</t>
+          <t>Ciudad de Querétaro, Querétaro, México</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Sunshine Silver Mining &amp; Refining Co.</t>
+          <t>Silverco Mining (ex Nuevo Silver; adquisición completada may-2026)</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -9017,89 +9007,15 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Estudios de factibilidad en curso (desmantelación del molino existente para construir uno nuevo, a completarse fin de 2026; estudios de factibilidad para reabrir la Refinería Plata-Cobre y construir una nueva Planta de Antimonio —hasta 34.5 millones lb/año—, entrega prevista inicios de 2027; estudio de factibilidad de la mina concluye Q2 2027; meta de reinicio de producción de plata fin de 2028)</t>
+          <t>Ingeniería/optimización (mina de plata-plomo-zinc-cobre tipo skarn en operación con más de 5 décadas de historia; PEA publicado 23-sep-2026 con VAN de US$329 millones sobre inversión de solo US$20.9 millones, vida de mina de 8.2 años; meta de expansión de capacidad de procesamiento a 2,500 tpd para 2S-2027, producción promedio estimada 4.1 millones oz eq. plata/año; programa de 15,000 m de perforación en curso para revalidar el depósito skarn)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/sunshine-silver-mining--refining-reports-second-quarter-2026-results-302850131.html); [World Energy](https://www.world-energy.org/article/54143.html)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/09/silverco-mining-proyecto-la-negra-en-queretaro-proyecta-van-de-us329-millones/); [Minart](https://minart.pe/2026/09/23/silverco-proyecta-us329-millones-de-valor-para-la-mina-la-negra-y-una-vida-util-de-82-anos/)</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>USA Rare Earth — Planta de Metal y Magnetos Blacksburg</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Blacksburg, Carolina del Sur, EE.UU.</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>USA Rare Earth (recién fusionada con Serra Verde Group, anunciado 4-sep-2026)</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Construcción (groundbreaking 9-sep-2026; inversión ~US$1,200 millones; ~490 empleos; planta de metal y manufactura de magnetos de tierras raras)</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/09/3358813/0/en/usa-rare-earth-breaks-ground-on-advanced-rare-earth-metal-and-magnet-manufacturing-facility-in-blacksburg-south-carolina.html)</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>La Negra Project (expansión)</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Ciudad de Querétaro, Querétaro, México</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Silverco Mining (ex Nuevo Silver; adquisición completada may-2026)</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Ingeniería/optimización (mina de plata-plomo-zinc-cobre tipo skarn en operación con más de 5 décadas de historia; PEA publicado 23-sep-2026 con VAN de US$329 millones sobre inversión de solo US$20.9 millones, vida de mina de 8.2 años; meta de expansión de capacidad de procesamiento a 2,500 tpd para 2S-2027, producción promedio estimada 4.1 millones oz eq. plata/año; programa de 15,000 m de perforación en curso para revalidar el depósito skarn)</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/09/silverco-mining-proyecto-la-negra-en-queretaro-proyecta-van-de-us329-millones/); [Minart](https://minart.pe/2026/09/23/silverco-proyecta-us329-millones-de-valor-para-la-mina-la-negra-y-una-vida-util-de-82-anos/)</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
@@ -9116,8 +9032,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9253,17 +9178,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales</t>
+          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales (expansión de 10 a 49 turbinas); TCEQ otorgó reunión pública sobre esta solicitud a petición del representante estatal Stan Lambert (~10-sep-2026), periodo de comentarios abierto; además, el gobernador Greg Abbott ordenó el 21-sep-2026 a la TCEQ pausar toda emisión de permisos nuevos para proyectos de data centers en Texas —incluidas instalaciones con generación propia "behind-the-meter"— hasta que ERCOT complete una auditoría de red (esperada mediados de dic-2026; TCEQ debe reportar cumplimiento al 19-oct-2026), lo que podría retrasar trámites pendientes de este y otros proyectos texanos del tracker</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/); [Texas Tribune](https://www.texastribune.org/2026/09/21/texas-data-center-moratorium-water-energy/); [Bracewell](https://www.bracewell.com/resources/governor-abbott-orders-tceq-to-pause-all-permit-issuance-for-data-center-projects/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -10585,17 +10510,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total); Fermi Inc. anunció 28-sep-2026 acuerdo de operación y mantenimiento (O&amp;M) con NAES Corporation —mayor operador independiente de plantas de energía de EE.UU.— para operar y mantener la flota de turbinas de gas natural del campus; Fermi retiene la propiedad de los activos, NAES opera; primeras turbinas de gas Siemens Energy SGT6-5000F ya llegaron a sitio; a inicios de sep-2026 Fermi también contrató a CBRE para operar/mantener su primer data center en Matador</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [StockTitan — NAES O&amp;M](https://www.stocktitan.net/news/FRMI/fermi-selects-naes-to-operate-and-maintain-its-natural-gas-turbine-qvztuks7g3tn.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -13556,6 +13481,43 @@
       <c r="G120" t="inlineStr">
         <is>
           <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Encinal Gas Power Plant</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Encinal, Webb County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Propuesta como JV 50/50 entre inversionistas surcoreanos (bajo el pacto comercial Corea-EE.UU. de US$350,000 millones) y socios estadounidenses; sin hyperscaler/cliente de cómputo IA nombrado aún</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Negociación/no confirmado (acuerdo de ~US$22,300 millones para planta de 6.3 GW —sería la más grande de ERCOT, ninguna planta de gas en Texas supera ~2 GW hoy—, destinada a alimentar data centers de IA y plantas de semiconductores; Fase 2 convertiría turbinas de Fase 1 a ciclo combinado y añadiría 4.9 GW; el Ministerio de Industria de Corea del Sur desmintió que el acuerdo esté cerrado, señalando que las consultas con Washington continúan, pendiente revisión parlamentaria coreana y aprobación de comité de inversión de EE.UU.; mantener en watch-list hasta anuncio oficial)</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>[TechRadar Pro](https://www.techradar.com/pro/south-korea-us-agree-on-usd22-billion-deal-for-6-3-gw-texas-gas-power-plant-encinal-facility-to-feed-ai-data-centers-under-washington-and-seouls-usd350-billion-pact); [Construction Review Online](https://constructionreviewonline.com/south-korea-eyes-22-3bn-encinal-gas-fired-power-plant-in-texas-for-ai-data-center-operations/); [Korean Tech Texas](https://koreantechtexas.com/korea-encinal-texas-gas-power-plant/)</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-28: 1 nuevo (Encinal Gas Power Plant, TX) + 5 actualizaciones de fase (#50)
- Nuevo: Encinal Gas Power Plant (Webb County, TX) — acuerdo Corea del Sur-EE.UU. de 6.3GW, aún no confirmado (watch-list).
- Actualizaciones: Golden Triangle Polymers (comisionamiento/arranque inminente), Santa Cruz Copper Project (PFS 2026, box cut oct-2026), Stibnite Gold Project (avance de construcción 28-sep), Fermi America Project Matador (acuerdo O&M con NAES), Stargate Abilene Campus (pausa estatal TCEQ de permisos para data centers en Texas).


Claude-Session: https://claude.ai/code/session_01Ae71eLABEqPVs1ixQhvtTM

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -416,8 +416,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -590,17 +599,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento) ; arranque ahora esperado en 2027 (retrasado al menos 6 meses respecto a 2026), según East Daley Analytics, por menor demanda de etano proyectada</t>
+          <t>Comisionamiento/arranque inminente (CEO de QatarEnergy, Saad al-Kaabi, declaró 20-sep-2026 en el Qatar Economic Forum que el complejo de US$8,500 millones "está iniciando comisionamiento y debería arrancar en las próximas semanas"; versión previa de East Daley Analytics estimaba arranque hasta 2027 por menor demanda de etano proyectada)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
+          <t>[MEES](https://www.mees.com/2026/9/25/corporate/qatarenergy-poised-to-start-up-texas-ethane-cracker/0ff02300-b8df-11f1-8f86-2b8776a66cca); [BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -792,106 +801,106 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Proyecto Escolín (amoniaco/urea)</t>
+          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Poza Rica, Veracruz, México</t>
+          <t>Lázaro Cárdenas, Michoacán, México</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mota-Engil México (EPC confirmado, US$1,200 millones, 47 meses); Duro Felguera (España) se integró formalmente 17-ago-2026 al contrato para gestión de proyecto y coordinación técnica de la ingeniería (supervisión de ingeniería externa, coordinación de suministros del tecnólogo, gestión de sistemas auxiliares); Casale (proveedor de tecnología)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ingeniería/inicio de construcción (inversión confirmada US$1,553 millones; capacidad objetivo &gt;700,000 ton/año de amoniaco, urea y AdBlue; citado explícitamente por la Presidenta Sheinbaum en su Segundo Informe de Gobierno —1-sep-2026— como parte del "rescate de la petroquímica" junto con Cosoleacaque, Morelos y Cangrejera)</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/); [El Español](https://www.elespanol.com/invertia/empresas/energia/20260817/duro-felguera-convoca-junta-extraordinaria-septiembre-aprobar-proyecto-clave-mota-engil-mexico/1003744355543_0.html); [La Política en Rosa](https://www.lapoliticaenrosa.com/2026/09/01/desde-veracruz-inicia-rescate-de-petroquimica-del-pais-destaca-claudia-sheinbaum-en-segundo-informe-de-gobierno/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
+          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas, Michoacán, México</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Transition Industries</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
+          <t>Construcción (colocación de primera piedra/groundbreaking simbólico 24-abr-2026; trabajos de ingeniería de campo y preparación de sitio iniciados en may-2026; inicio de construcción completa programado para finales de 2026; planta de metanol azul/ultra bajo carbono más grande del mundo, ~1.8 Mt/año metanol azul + 350,000 t/año ultra bajo carbono; operación esperada 2029-2030)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/); [BusinessWire](https://www.businesswire.com/news/home/20260423775301/en/Pacfico-Mexinol-Celebrates-the-Symbolic-Groundbreaking-in-Topolobampo-Positioning-Mexico-in-the-New-Low-Carbon-Chemical-Industry)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
+          <t>First Ammonia (amoniaco verde)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Victoria, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Transition Industries</t>
+          <t>First Ammonia / Cox Group USA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
+          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (colocación de primera piedra/groundbreaking simbólico 24-abr-2026; trabajos de ingeniería de campo y preparación de sitio iniciados en may-2026; inicio de construcción completa programado para finales de 2026; planta de metanol azul/ultra bajo carbono más grande del mundo, ~1.8 Mt/año metanol azul + 350,000 t/año ultra bajo carbono; operación esperada 2029-2030)</t>
+          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / inicio de construcción reprogramado para inicios de octubre de 2026 en el Puerto de Victoria, Texas (planta de 200 MW, fase 1); cierre financiero esperado antes de fin de 2026, operación comercial estimada 2029</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/); [BusinessWire](https://www.businesswire.com/news/home/20260423775301/en/Pacfico-Mexinol-Celebrates-the-Symbolic-Groundbreaking-in-Topolobampo-Positioning-Mexico-in-the-New-Low-Carbon-Chemical-Industry)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -903,165 +912,165 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>First Ammonia (amoniaco verde)</t>
+          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Victoria, Texas, EE.UU.</t>
+          <t>Topolobampo, Ahome, Sinaloa, México</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>First Ammonia / Cox Group USA</t>
+          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / inicio de construcción reprogramado para inicios de octubre de 2026 en el Puerto de Victoria, Texas (planta de 200 MW, fase 1); cierre financiero esperado antes de fin de 2026, operación comercial estimada 2029</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace, con protesta en el Zócalo) presionan por la cancelación del proyecto; GPO aceptó, como parte de las negociaciones, modificar la toma de agua —reubicándola al canal de residuos de CFE— y descargar la salmuera caliente fuera de la bahía de Ohuira, mientras mantiene pausadas las plantas de urea y metanol; sin resolución final reportada a la fecha)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/); [Bajo Palabra](https://www.bajopalabra.mx/sheinbaum-descarta-por-ahora-cancelar-megaplanta-de-amoniaco-en-topolobampo-ante-reclamos-ambientales/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
+          <t>Lake Charles Methanol II</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Topolobampo, Ahome, Sinaloa, México</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
+          <t>Lake Charles Methanol II LLC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Zachry Group (FEED)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto; plantón alcanzó 100 días ininterrumpidos (6-sep-2026); nueva ronda de revisión técnica federal programada 7 al 11-sep-2026; presidenta Sheinbaum confirmó (7-sep-2026) que el proyecto no está cancelado y que la decisión final se tomará tras consulta pública con las comunidades afectadas; grupos ambientalistas (incl. Greenpeace, con protesta en el Zócalo) presionan por la cancelación del proyecto; GPO aceptó, como parte de las negociaciones, modificar la toma de agua —reubicándola al canal de residuos de CFE— y descargar la salmuera caliente fuera de la bahía de Ohuira, mientras mantiene pausadas las plantas de urea y metanol; sin resolución final reportada a la fecha)</t>
+          <t>Ingeniería (FEED) / FID prevista</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/); [La Jornada](https://www.jornada.com.mx/2026/09/08/politica/011n2pol?partner=rss); [El Financiero](https://www.elfinanciero.com.mx/nacional/2026/09/07/ambientalistas-presionan-para-cancelar-planta-de-amonioaco-en-topolobampo/); [El Imparcial](https://www.elimparcial.com/mexico/2026/09/06/campamento-en-topolobampo-cumple-100-dias-de-bloqueo-ininterrumpido-contra-la-planta-de-amoniaco-mientras-pescadores-y-comunidades-indigenas-de-sinaloa-sostienen-la-resistencia-para-proteger-la-bahia-de-ohuira/); [Bajo Palabra](https://www.bajopalabra.mx/sheinbaum-descarta-por-ahora-cancelar-megaplanta-de-amoniaco-en-topolobampo-ante-reclamos-ambientales/)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II</t>
+          <t>Planta Coquizadora Salina Cruz</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
+          <t>Salina Cruz, Oaxaca, México</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II LLC</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Zachry Group (FEED)</t>
+          <t>ICA Fluor</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / FID prevista</t>
+          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Planta Coquizadora Salina Cruz</t>
+          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Salina Cruz, Oaxaca, México</t>
+          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Shintech Louisiana, LLC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ICA Fluor</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
+          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
+          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
+          <t>Texas City, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Shintech Louisiana, LLC</t>
+          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1071,86 +1080,86 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
+          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
+          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Texas City, Texas, EE.UU.</t>
+          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
+          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Air Liquide (unidad propia); OXEA no especificado</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
+          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
+          <t>Targa Resources East Driver Gas Processing Plant</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
+          <t>Condado de Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Air Liquide (unidad propia); OXEA no especificado</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
+          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1162,32 +1171,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Targa Resources East Driver Gas Processing Plant</t>
+          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Condado de Midland, Texas, EE.UU.</t>
+          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
+          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1199,32 +1208,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
+          <t>MPLX Secretariat II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
+          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
+          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1236,12 +1245,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MPLX Secretariat II Gas Processing Plant</t>
+          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
+          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1256,12 +1265,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
+          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1273,32 +1282,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
+          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
+          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Northern Plains Nitrogen LLC</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>EPC no designado</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
+          <t>Pre-FEED completo / FID buscada 4T2026</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1310,54 +1319,54 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
+          <t>Iron Mesa (planta de gas)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
+          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen LLC</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EPC no designado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pre-FEED completo / FID buscada 4T2026</t>
+          <t>Construcción (arranque previsto Q1 2027)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Iron Mesa (planta de gas)</t>
+          <t>Yeti II (planta de gas)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Targa Resources</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1367,12 +1376,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Construcción (arranque previsto Q1 2027)</t>
+          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1384,32 +1393,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Yeti II (planta de gas)</t>
+          <t>Refinería Francisco I. Madero (rehabilitación)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Ciudad Madero, Tamaulipas, México</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Targa Resources</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
+          <t>Licitación/bidding</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1421,106 +1430,106 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Refinería Francisco I. Madero (rehabilitación)</t>
+          <t>Fermachem Planta de Urea/Amoniaco</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ciudad Madero, Tamaulipas, México</t>
+          <t>Ejido Sapioris, Lerdo, Durango, México</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Fermaca Dreams (Fermachem)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
+          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación/bidding</t>
+          <t>Construcción reanudada (obra había sido pausada por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento; gobernador Esteban Villegas confirmó 7-sep-2026 que la empresa cuenta con todos los permisos federales pese a objeciones del cabildo de Lerdo sobre permisos municipales; Sedeco Durango reafirmó 23-sep-2026 que el proyecto está "vigente al 100%" con todas las autorizaciones ambientales en regla; ya se completaron trabajos de compactación/preparación de 150 hectáreas en el ejido Sapioriz; construcción formal de la primera fase se proyecta en ~28 meses; inversión ~US$1,600 millones, capacidad 1 millón ton/año de urea granulada)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [El Siglo de Torreón — Canacintra](https://www.elsiglodetorreon.com.mx/noticia/2026/fermachem-es-un-proyecto-auditado-legal-y-mexicano-sin-almacenamiento-de-amoniaco-canacintra.html); [Grem Noticieros — Sedeco](https://www.noticierosgrem.com.mx/vigente-al-100-proyecto-de-planta-fermachem-en-lerdo-sedeco/); [El Siglo de Torreón — Gobernador](https://www.elsiglodetorreon.com.mx/noticia/2026/planta-de-fermachen-en-lerdo-va-mas-que-firme-gobernador-de-durango.html)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fermachem Planta de Urea/Amoniaco</t>
+          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ejido Sapioris, Lerdo, Durango, México</t>
+          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fermaca Dreams (Fermachem)</t>
+          <t>Clean Hydrogen Works</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
+          <t>McDermott (FEED)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Construcción reanudada (obra había sido pausada por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento; gobernador Esteban Villegas confirmó 7-sep-2026 que la empresa cuenta con todos los permisos federales pese a objeciones del cabildo de Lerdo sobre permisos municipales; Sedeco Durango reafirmó 23-sep-2026 que el proyecto está "vigente al 100%" con todas las autorizaciones ambientales en regla; ya se completaron trabajos de compactación/preparación de 150 hectáreas en el ejido Sapioriz; construcción formal de la primera fase se proyecta en ~28 meses; inversión ~US$1,600 millones, capacidad 1 millón ton/año de urea granulada)</t>
+          <t>Ingeniería (FEED) / Pre-FID</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [El Siglo de Torreón — Canacintra](https://www.elsiglodetorreon.com.mx/noticia/2026/fermachem-es-un-proyecto-auditado-legal-y-mexicano-sin-almacenamiento-de-amoniaco-canacintra.html); [Grem Noticieros — Sedeco](https://www.noticierosgrem.com.mx/vigente-al-100-proyecto-de-planta-fermachem-en-lerdo-sedeco/); [El Siglo de Torreón — Gobernador](https://www.elsiglodetorreon.com.mx/noticia/2026/planta-de-fermachen-en-lerdo-va-mas-que-firme-gobernador-de-durango.html)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
+          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Clean Hydrogen Works</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>McDermott (FEED)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / Pre-FID</t>
+          <t>Ingeniería (sancionado; en línea 2028)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1532,128 +1541,128 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
+          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
+          <t>Gothenburg, Nebraska, EE.UU.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ingeniería (sancionado; en línea 2028)</t>
+          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
+          <t>Wabash Low-Carbon Ammonia Project</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gothenburg, Nebraska, EE.UU.</t>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
+          <t>Wabash Valley Resources</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Wabash Low-Carbon Ammonia Project</t>
+          <t>Green Fuels Operating — Refinería Duncan</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>West Terre Haute, Indiana, EE.UU.</t>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Wabash Valley Resources</t>
+          <t>Green Fuels Operating</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Green Fuels Operating — Refinería Duncan</t>
+          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+          <t>Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Green Fuels Operating</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1663,34 +1672,34 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
+          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>ONEOK Inc.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1700,49 +1709,49 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
+          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
+          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
+          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ONEOK Inc.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
+          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
+          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1754,86 +1763,86 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
+          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
+          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
+          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
+          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
+          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
+          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1848,7 +1857,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1858,39 +1867,39 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1902,54 +1911,54 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Southern Energy Renewables</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+          <t>Richland, Washington, EE.UU.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables</t>
+          <t>Atlas Agro</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1959,145 +1968,145 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
+          <t>Hydrogen City (complejo Power-to-X / e-metanol / amoniaco verde)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Richland, Washington, EE.UU.</t>
+          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU. (corredor Corpus Christi–Brownsville; hub de ~50,000 acres)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Atlas Agro</t>
+          <t>Green Hydrogen International (GHI), en asociación con INPEX Corporation (Japón) para el componente de amoniaco</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>ABB (automatización/control, vía MOU)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
+          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; INPEX y GHI firmaron Joint Study Agreement para avanzar el componente de amoniaco verde de exportación —Fase 1: 280,000 ton/año de H2 verde para producir 1 millón ton/año de amoniaco verde, alimentado por 3.75 GW de renovables—, sin FID formal ni EPC adjudicado aún; construcción planeada desde 2026, primera producción de amoniaco estimada 2029, e-metanol 2030)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/renewable-sustainability-h2-esg/green-hydrogen-international-and-inpex-corporation-project-south-texas/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Hydrogen City (complejo Power-to-X / e-metanol / amoniaco verde)</t>
+          <t>Targa Resources Falcon II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU. (corredor Corpus Christi–Brownsville; hub de ~50,000 acres)</t>
+          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Green Hydrogen International (GHI), en asociación con INPEX Corporation (Japón) para el componente de amoniaco</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ABB (automatización/control, vía MOU)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; INPEX y GHI firmaron Joint Study Agreement para avanzar el componente de amoniaco verde de exportación —Fase 1: 280,000 ton/año de H2 verde para producir 1 millón ton/año de amoniaco verde, alimentado por 3.75 GW de renovables—, sin FID formal ni EPC adjudicado aún; construcción planeada desde 2026, primera producción de amoniaco estimada 2029, e-metanol 2030)</t>
+          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/renewable-sustainability-h2-esg/green-hydrogen-international-and-inpex-corporation-project-south-texas/)</t>
+          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Targa Resources Falcon II Gas Processing Plant</t>
+          <t>Cassidy II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
+          <t>Condado de Glasscock, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Brazos Midstream</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
+          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cassidy II Gas Processing Plant</t>
+          <t>Kings Landing II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Condado de Glasscock, Texas, EE.UU.</t>
+          <t>Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Brazos Midstream</t>
+          <t>Kinetik Holdings</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2107,34 +2116,34 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
+          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
+          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kings Landing II Gas Processing Plant</t>
+          <t>Apollo Gas Plant</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Nuevo México, EE.UU.</t>
+          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Kinetik Holdings</t>
+          <t>Trace Midstream Partners II</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2144,12 +2153,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
+          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
+          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2161,17 +2170,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Apollo Gas Plant</t>
+          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
+          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Trace Midstream Partners II</t>
+          <t>IGP Methanol LLC</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2181,12 +2190,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
+          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
+          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2198,91 +2207,91 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
+          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
+          <t>Culbertson, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>IGP Methanol LLC</t>
+          <t>Cyan H2</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
+          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
+          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
+          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Culbertson, Montana, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Cyan H2</t>
+          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
+          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
+          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
+          <t>México Amoníaco y Urea (MAYU)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
+          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
+          <t>México Amoníaco y Urea (desarrollador privado)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2292,34 +2301,34 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
+          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
+          <t>[MAYU](https://mayu.com.mx/en/)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (MAYU)</t>
+          <t>Ampliación Terminal de Exportación NGL Nederland</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
+          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (desarrollador privado)</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2329,34 +2338,34 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
+          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>[MAYU](https://mayu.com.mx/en/)</t>
+          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ampliación Terminal de Exportación NGL Nederland</t>
+          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
+          <t>El Dorado, Arkansas, EE.UU.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>LSB Industries</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2366,34 +2375,34 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
+          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
+          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
+          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>El Dorado, Arkansas, EE.UU.</t>
+          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LSB Industries</t>
+          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2403,12 +2412,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
+          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
+          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2420,91 +2429,91 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
+          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
+          <t>Tuscola, Illinois, EE.UU.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
+          <t>Cronus Chemicals LLC</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
+          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
+          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
+          <t>CHS/OCP North America — Planta de Fertilizante Fosfatado</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Tuscola, Illinois, EE.UU.</t>
+          <t>Cornerstone Energy Park, Waggaman, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Cronus Chemicals LLC</t>
+          <t>CHS Inc. / OCP North America (JV 50/50)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
+          <t>Planeación/pre-construcción (JV anunciada 26-ago-2026 en ceremonia con la Secretaria de Agricultura de EE.UU., Brooke Rollins; sería la primera planta nueva de fertilizante fosfatado construida en EE.UU. desde 1984; capacidad hasta 1.3 millones ton/año, inversión hasta US$450 millones; solicitud de financiamiento presentada al programa USDA FIELDS; construcción prevista antes de fin de 2026, producción posible a fines de 2028)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
+          <t>[CHS Inc.](https://www.chsinc.com/news-and-stories/2026/08/26/chs-ocp-domestic-fertilizer-production-announcement); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/chs-ocp-plan-up-to-450m-louisiana-fertilizer-plant/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CHS/OCP North America — Planta de Fertilizante Fosfatado</t>
+          <t>CITGO Lake Charles Refinery — Depentanizer Project (mejora de naphtha upgrading)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cornerstone Energy Park, Waggaman, Luisiana, EE.UU.</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CHS Inc. / OCP North America (JV 50/50)</t>
+          <t>CITGO Petroleum Corporation</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2514,52 +2523,15 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (JV anunciada 26-ago-2026 en ceremonia con la Secretaria de Agricultura de EE.UU., Brooke Rollins; sería la primera planta nueva de fertilizante fosfatado construida en EE.UU. desde 1984; capacidad hasta 1.3 millones ton/año, inversión hasta US$450 millones; solicitud de financiamiento presentada al programa USDA FIELDS; construcción prevista antes de fin de 2026, producción posible a fines de 2028)</t>
+          <t>Aprobado/Ingeniería (proyecto de US$310 millones aprobado 1-sep-2026; agrega instalaciones y equipo para mejorar el upgrading de nafta, convirtiendo corrientes de menor valor en componentes de gasolina de mayor valor; entrada en operación prevista 2029)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[CHS Inc.](https://www.chsinc.com/news-and-stories/2026/08/26/chs-ocp-domestic-fertilizer-production-announcement); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/chs-ocp-plan-up-to-450m-louisiana-fertilizer-plant/)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/09/citgo-to-invest-310-mm-to-improve-naphtha-upgrading-at-lake-charles-refinery-us/); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/citgo-strengthens-lake-charles-refinerys-future-with-310-million-project/)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>CITGO Lake Charles Refinery — Depentanizer Project (mejora de naphtha upgrading)</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>CITGO Petroleum Corporation</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Aprobado/Ingeniería (proyecto de US$310 millones aprobado 1-sep-2026; agrega instalaciones y equipo para mejorar el upgrading de nafta, convirtiendo corrientes de menor valor en componentes de gasolina de mayor valor; entrada en operación prevista 2029)</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/09/citgo-to-invest-310-mm-to-improve-naphtha-upgrading-at-lake-charles-refinery-us/); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/downstream/citgo-strengthens-lake-charles-refinerys-future-with-310-million-project/)</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
@@ -2578,6 +2550,15 @@
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4403,8 +4384,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4466,17 +4456,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins; excavación del box-cut programada para 3T2026</t>
+          <t>Construcción (Estudio de Prefactibilidad —PFS— 2026 publicado 23-sep-2026: capex inicial elevado a US$1,430 millones, costo operativo US$1.47/lb, VPN después de impuestos US$3,500 millones, TIR 30%; mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; "box cut" —corte de acceso a la mina— previsto para iniciar octubre 2026; carta preliminar de US$1,100 millones del Export-Import Bank de EE.UU., aprobación final esperada primavera 2027; primera producción de cátodo de cobre prevista 2029) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/) ; [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
+          <t>[Ivanhoe Electric — PFS 2026](https://ivanhoeelectric.com/news/2026-preliminary-feasibility-study-for-the-santa-cruz-copper-project-in-arizona-confirms-high-grade-low-cost-project-with-strong-economics/); [Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -4873,17 +4863,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Directorio del Export-Import Bank de EE.UU. aprobó por unanimidad, 20-ago-2026, el préstamo garantizado senior de USD 2,900 millones para financiar el desarrollo; Corte Federal de Distrito de Idaho confirmó 18-ago-2026 la mayoría de las aprobaciones federales del USFS, aunque encontró insuficientes las declaraciones de captura incidental para carcayú y trucha toro, lo que motivó una apelación ante el Noveno Circuito presentada ~25-ago-2026 por una coalición conservacionista —la Tribu Nez Perce mantiene demanda separada—, sin que ello detenga la obra; actualización de construcción del 31-ago-2026 reporta fabricación/enrolado en Europa de los componentes del doble autoclave y avance ~50% en la entrega de módulos de vivienda permanente para trabajadores —ATCO—, con primer oro previsto 2029)</t>
+          <t>Construcción (actualización de construcción y exploración del 28-sep-2026 confirma actividades activas de "critical path": ruta Burntlog, vivienda para trabajadores, desarrollo de infraestructura de línea de transmisión; postes de energía y equipo auxiliar ya entregados en los patios de acopio —laydown areas— de Donnelly y Cascade, Idaho; permisos federales asegurados desde 2025; corte federal de Idaho negó en jun-2026 moción para detener obras; EXIM Bank aprobó 20-ago-2026 préstamo garantizado senior de USD 2,900 millones; apelación ante el Noveno Circuito sobre declaraciones de captura incidental —presentada ~25-ago-2026— continúa sin detener la obra; primer oro previsto 2029)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html); [Northern Miner](https://www.northernminer.com/news/court-ruling-backs-perpetuas-1-3b-stibnite-build/1003894465/); [PRNewswire](https://www.prnewswire.com/news-releases/perpetua-resources-provides-construction-update-on-the-stibnite-gold-project-and-exploration-activities-302864546.html); [Center for Biological Diversity](https://biologicaldiversity.org/w/news/press-releases/appeal-targets-federal-approval-of-massive-idaho-gold-mine-2026-08-25/)</t>
+          <t>[PR Newswire — actualización 28-sep-2026](https://www.prnewswire.com/news-releases/perpetua-resources-provides-construction--exploration-update-302891031.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html); [Northern Miner](https://www.northernminer.com/news/court-ruling-backs-perpetuas-1-3b-stibnite-build/1003894465/); [Center for Biological Diversity](https://biologicaldiversity.org/w/news/press-releases/appeal-targets-federal-approval-of-massive-idaho-gold-mine-2026-08-25/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -7147,12 +7137,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Angangueo</t>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Angangueo, Michoacán, México</t>
+          <t>Empalme, Sonora, México</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -7167,7 +7157,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos con gobierno federal)</t>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -7184,17 +7174,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Chalchihuites</t>
+          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Chalchihuites, Zacatecas, México</t>
+          <t>Condado de Coosa, Alabama, EE.UU.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Westwater Resources Inc.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7204,34 +7194,34 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Modernización Complejo Metalúrgico Empalme</t>
+          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Empalme, Sonora, México</t>
+          <t>Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Global Advanced Metals</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7241,34 +7231,34 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
+          <t>Boron Americas Project (Fort Cady)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Condado de Coosa, Alabama, EE.UU.</t>
+          <t>California, EE.UU.</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Westwater Resources Inc.</t>
+          <t>5E Advanced Materials</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7278,12 +7268,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -7295,54 +7285,54 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
+          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Pensilvania, EE.UU.</t>
+          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Global Advanced Metals</t>
+          <t>Ramaco Resources</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
+          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Boron Americas Project (Fort Cady)</t>
+          <t>Dewey-Burdock Uranium ISR Project</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>California, EE.UU.</t>
+          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>5E Advanced Materials</t>
+          <t>enCore Energy (Powertech USA)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7352,71 +7342,71 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
+          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
+          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
+          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ramaco Resources</t>
+          <t>Niron Magnetics</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
+          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
+          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Dewey-Burdock Uranium ISR Project</t>
+          <t>Louisiana Strategic Metals Complex</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
+          <t>Alexandria, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>enCore Energy (Powertech USA)</t>
+          <t>Ucore Rare Metals Inc.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7426,34 +7416,34 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
+          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
+          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
+          <t>Distrito Copper Creek / San Manuel</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
+          <t>Condado de Pinal, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Niron Magnetics</t>
+          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7463,71 +7453,71 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
+          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
+          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Louisiana Strategic Metals Complex</t>
+          <t>IMA Mine</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Alexandria, Luisiana, EE.UU.</t>
+          <t>Condado de Lemhi, Idaho, EE.UU.</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Ucore Rare Metals Inc.</t>
+          <t>American Tungsten Corp.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
+          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
+          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Distrito Copper Creek / San Manuel</t>
+          <t>Railroad Valley Minerals / Super-Brine Complex</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Condado de Pinal, Arizona, EE.UU.</t>
+          <t>Railroad Valley, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
+          <t>3 Proton Lithium (3PL Operating Inc.)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -7537,12 +7527,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
+          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
+          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -7554,32 +7544,32 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IMA Mine</t>
+          <t>New Amalga Gold Project</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Condado de Lemhi, Idaho, EE.UU.</t>
+          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>American Tungsten Corp.</t>
+          <t>Grande Portage Resources Ltd.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
+          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -7591,17 +7581,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Railroad Valley Minerals / Super-Brine Complex</t>
+          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Railroad Valley, Nevada, EE.UU.</t>
+          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>3 Proton Lithium (3PL Operating Inc.)</t>
+          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7611,71 +7601,71 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
+          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
+          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>New Amalga Gold Project</t>
+          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
+          <t>Marion, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Grande Portage Resources Ltd.</t>
+          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
+          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
+          <t>La Preciosa Project</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
+          <t>Durango, México</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -7685,71 +7675,71 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
+          <t>Great Salt Lake Lithium Facility</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Marion, Indiana, EE.UU.</t>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>La Preciosa Project</t>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Durango, México</t>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+          <t>Nth Cycle, Inc.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -7759,49 +7749,49 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Great Salt Lake Lithium Facility</t>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Condado de Box Elder, Utah, EE.UU.</t>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -7813,106 +7803,106 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+          <t>Copperwood Project</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Nth Cycle, Inc.</t>
+          <t>Highland Copper Company</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>DRA Americas Inc. (FEED)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+          <t>Modernización Refinería de Cobre El Paso</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
+          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Copperwood Project</t>
+          <t>Round Top Rare Earth Project</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
+          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Highland Copper Company</t>
+          <t>USA Rare Earth Inc.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>DRA Americas Inc. (FEED)</t>
+          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
+          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -7924,32 +7914,32 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Modernización Refinería de Cobre El Paso</t>
+          <t>Expansión Fundición de Antimonio Thompson Falls</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Thompson Falls, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>United States Antimony Corporation (USAC)</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
+          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
+          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -7961,32 +7951,32 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Round Top Rare Earth Project</t>
+          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
+          <t>Morenci, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>USA Rare Earth Inc.</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
+          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
+          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -7998,17 +7988,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Expansión Fundición de Antimonio Thompson Falls</t>
+          <t>Reconstrucción Fundición y Refinería Kennecott</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Thompson Falls, Montana, EE.UU.</t>
+          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>United States Antimony Corporation (USAC)</t>
+          <t>Rio Tinto (Kennecott Utah Copper)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8018,12 +8008,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
+          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
+          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -8035,32 +8025,32 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
+          <t>Fourmile (decline Bullion Hill)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Morenci, Arizona, EE.UU.</t>
+          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
+          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -8072,17 +8062,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Reconstrucción Fundición y Refinería Kennecott</t>
+          <t>Puerto del Aire (distrito Mulatos)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Rio Tinto (Kennecott Utah Copper)</t>
+          <t>Alamos Gold Inc.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8092,12 +8082,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
+          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
+          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -8109,54 +8099,54 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Fourmile (decline Bullion Hill)</t>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
+          <t>Clarksville, Tennessee, EE.UU.</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Puerto del Aire (distrito Mulatos)</t>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Alamos Gold Inc.</t>
+          <t>Aclara Resources Inc.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8166,34 +8156,34 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+          <t>Archimedes Project (i-80 Gold)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Clarksville, Tennessee, EE.UU.</t>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+          <t>i-80 Gold Corp</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8203,12 +8193,12 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -8220,17 +8210,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Aclara Heavy Rare Earth Separation Facility</t>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Aclara Resources Inc.</t>
+          <t>Sweetwater Uranium, Inc.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8240,12 +8230,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -8257,17 +8247,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Archimedes Project (i-80 Gold)</t>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+          <t>San Juan County, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>i-80 Gold Corp</t>
+          <t>Anfield Energy Inc.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8277,12 +8267,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -8294,350 +8284,350 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+          <t>Twin Metals Minnesota</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Sweetwater County, Wyoming, EE.UU.</t>
+          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium, Inc.</t>
+          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+          <t>Permitting/Pre-EIS con retroceso regulatorio (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026 mediante orden ejecutiva que prohíbe minería no ferrosa en la cuenca del Rainy River Headwaters; el DNR de Minnesota canceló uno de los arrendamientos minerales de Twin Metals cerca de Babbitt por incumplimiento de requisitos de desempeño/producción, anunciado 14-sep-2026 y efectivo 10-nov-2026; grupos ambientalistas lo ven como precedente para cancelar los arrendamientos restantes; proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242); [KAXE](https://www.kaxe.org/local-news/2026-09-14/dnr-cancels-1-twin-metals-mineral-lease-near-babbitt); [Voyageurs Conservancy](https://www.voyageurs.org/news/2026/9/22/what-the-walz-order-and-the-twin-metals-lease-cancellation-mean-for-voyageurs)</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Velvet-Wood Uranium-Vanadium Project</t>
+          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>San Juan County, Utah, EE.UU.</t>
+          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Anfield Energy Inc.</t>
+          <t>Falcon Copper Corp. (MOU con Glencore)</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Twin Metals Minnesota</t>
+          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
+          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
+          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>Metso Finland Oy (estudio de alcance)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS con retroceso regulatorio (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026 mediante orden ejecutiva que prohíbe minería no ferrosa en la cuenca del Rainy River Headwaters; el DNR de Minnesota canceló uno de los arrendamientos minerales de Twin Metals cerca de Babbitt por incumplimiento de requisitos de desempeño/producción, anunciado 14-sep-2026 y efectivo 10-nov-2026; grupos ambientalistas lo ven como precedente para cancelar los arrendamientos restantes; proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242); [KAXE](https://www.kaxe.org/local-news/2026-09-14/dnr-cancels-1-twin-metals-mineral-lease-near-babbitt); [Voyageurs Conservancy](https://www.voyageurs.org/news/2026/9/22/what-the-walz-order-and-the-twin-metals-lease-cancellation-mean-for-voyageurs)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
+          <t>Spring Valley Gold Mine</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
+          <t>Condado de Pershing, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Falcon Copper Corp. (MOU con Glencore)</t>
+          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
+          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
+          <t>Pitarrilla Project (plata-plomo-zinc)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
+          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
+          <t>Endeavour Silver Corp.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Metso Finland Oy (estudio de alcance)</t>
+          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
+          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Spring Valley Gold Mine</t>
+          <t>Red Dog Mine Life Extension Project</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Condado de Pershing, Nevada, EE.UU.</t>
+          <t>Distrito Minero de NANA, noroeste de Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
+          <t>Teck American Incorporated (Teck Resources), en tierras de NANA Regional Corporation</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>U.S. Army Corps of Engineers (agencia líder de permisos)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
+          <t>Prefactibilidad (estudio en curso; Teck destina US$200-250 millones en 2026 a obras tempranas —camino de acceso todo-el-año, perforación— y avance del estudio de prefactibilidad; minado subterráneo por realces largos (long-hole stoping) propuesto para los yacimientos Aktigiruq y Anarraaq, alimentando el molino existente de Red Dog; minerales: zinc, plomo, plata, germanio; proyecto obtuvo cobertura FAST-41 en sep-2026)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
+          <t>[Permitting.gov](https://www.permitting.gov/newsroom/press-releases/red-dog-mine-life-extension-project-gains-fast-41-coverage); [Mining News North](https://www.miningnewsnorth.com/story/2026/09/04/news/red-dog-extension-gains-fast-41-permitting/9851.html)</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Pitarrilla Project (plata-plomo-zinc)</t>
+          <t>Kings Mountain Lithium Material Processing Plant</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
+          <t>Kings Mountain, Carolina del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Endeavour Silver Corp.</t>
+          <t>Albemarle Corporation</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
+          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión; DOE anunció 14-sep-2026 US$16 millones adicionales para programas de educación minera durante visita al sitio —14 escuelas mineras acreditadas—; proyecto sigue a la espera de permisos estatales y locales, tajo ya drenado)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
+          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf); [WFAE](https://www.wfae.org/energy-environment/2026-09-14/trump-administration-announces-16-million-for-mining-education-at-kings-mountain-lithium-site)</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Red Dog Mine Life Extension Project</t>
+          <t>Tonopah Flats Lithium Project</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Distrito Minero de NANA, noroeste de Alaska, EE.UU.</t>
+          <t>Condados de Esmeralda y Nye, Nevada, EE.UU. (~11 km al noroeste de Tonopah)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Teck American Incorporated (Teck Resources), en tierras de NANA Regional Corporation</t>
+          <t>American Battery Technology Company (ABTC)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>U.S. Army Corps of Engineers (agencia líder de permisos)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Prefactibilidad (estudio en curso; Teck destina US$200-250 millones en 2026 a obras tempranas —camino de acceso todo-el-año, perforación— y avance del estudio de prefactibilidad; minado subterráneo por realces largos (long-hole stoping) propuesto para los yacimientos Aktigiruq y Anarraaq, alimentando el molino existente de Red Dog; minerales: zinc, plomo, plata, germanio; proyecto obtuvo cobertura FAST-41 en sep-2026)</t>
+          <t>Permitting (BLM aceptó formalmente el Plan of Operations de mina y refinería el 8-sep-2026, hito mayor hacia autorización NEPA; proyecto usa proceso propietario de lixiviación selectiva —SLE—; recurso estimado de 21.3 millones de toneladas de hidróxido de litio monohidratado accesible; mina y refinería en pleno desarrollo proyectadas a producir hasta 30,000 t/año de hidróxido de litio, ~1,300 empleos de construcción)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>[Permitting.gov](https://www.permitting.gov/newsroom/press-releases/red-dog-mine-life-extension-project-gains-fast-41-coverage); [Mining News North](https://www.miningnewsnorth.com/story/2026/09/04/news/red-dog-extension-gains-fast-41-permitting/9851.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/08/3357682/0/en/american-battery-technology-company-achieves-major-milestone-with-u-s-blm-acceptance-of-plan-of-operations-for-tonopah-flats-lithium-project.html); [Mining Technology](https://www.mining-technology.com/projects/tonopah-flats-lithium-project-us/)</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Kings Mountain Lithium Material Processing Plant</t>
+          <t>Angel Island Lithium Project</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Kings Mountain, Carolina del Norte, EE.UU.</t>
+          <t>Esmeralda County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Albemarle Corporation</t>
+          <t>Century Lithium Corp.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Fluor Corporation</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Permisos completados/pre-construcción (planta de procesamiento mineral con capacidad de ~420,000 t/año de concentrado de espodumeno; completó el proceso de permisos federales bajo el programa FAST-41 el 30-mar-2026; DOE propone financiamiento de US$149.7 millones dentro de un costo total del proyecto de ~US$394 millones, resto aportado por Albemarle; construcción plurianual pendiente de decisión final de inversión; DOE anunció 14-sep-2026 US$16 millones adicionales para programas de educación minera durante visita al sitio —14 escuelas mineras acreditadas—; proyecto sigue a la espera de permisos estatales y locales, tajo ya drenado)</t>
+          <t>Permitting (presentó Plan de Operaciones Minero y solicitud de Permiso de Reclamación de Nevada ante BLM el 3-sep-2026; proyecto bajo programa FAST-41; meta de completar permisos federales para feb-2028)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>[Permitting Council](https://www.permitting.gov/newsroom/press-releases/kings-mountain-lithium-material-processing-plant-project-completes-federal); [DOE](https://www.energy.gov/sites/default/files/2026-03/fonsi-ea-2265-albemarle-2026-03.pdf); [WFAE](https://www.wfae.org/energy-environment/2026-09-14/trump-administration-announces-16-million-for-mining-education-at-kings-mountain-lithium-site)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/CYDVF/century-lithium-files-mine-plan-of-operations-for-angel-island-0v6ql6hprbzu.html)</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Tonopah Flats Lithium Project</t>
+          <t>Silver Peak Lithium Mine (Expansión)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Condados de Esmeralda y Nye, Nevada, EE.UU. (~11 km al noroeste de Tonopah)</t>
+          <t>Esmeralda County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>American Battery Technology Company (ABTC)</t>
+          <t>Albemarle Corporation</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -8647,49 +8637,49 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Permitting (BLM aceptó formalmente el Plan of Operations de mina y refinería el 8-sep-2026, hito mayor hacia autorización NEPA; proyecto usa proceso propietario de lixiviación selectiva —SLE—; recurso estimado de 21.3 millones de toneladas de hidróxido de litio monohidratado accesible; mina y refinería en pleno desarrollo proyectadas a producir hasta 30,000 t/año de hidróxido de litio, ~1,300 empleos de construcción)</t>
+          <t>Permitting completo (BLM completó el permitting federal el 27-feb-2026; autorizada operación/expansión en 8,058 acres; incluye construcción de 2 estaciones de bombeo, 2 piscinas de salmuera y tuberías de proceso)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/08/3357682/0/en/american-battery-technology-company-achieves-major-milestone-with-u-s-blm-acceptance-of-plan-of-operations-for-tonopah-flats-lithium-project.html); [Mining Technology](https://www.mining-technology.com/projects/tonopah-flats-lithium-project-us/)</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-silver-peak-lithium-mine-expansion); [Permitting.gov](https://www.permitting.gov/newsroom/press-releases/silver-peak-lithium-mine-project-completes-federal-permitting)</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Angel Island Lithium Project</t>
+          <t>McDermitt Lithium Project (lado Jindalee)</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Esmeralda County, Nevada, EE.UU.</t>
+          <t>Condado de Malheur, Oregón (límite con Nevada), EE.UU.</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Century Lithium Corp.</t>
+          <t>Jindalee Lithium (ASX:JLL / OTCQX:JNDAF)</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (contratista de perforación contratado)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Permitting (presentó Plan de Operaciones Minero y solicitud de Permiso de Reclamación de Nevada ante BLM el 3-sep-2026; proyecto bajo programa FAST-41; meta de completar permisos federales para feb-2028)</t>
+          <t>Exploración (permiso estatal de Oregón obtenido para perforación; inicio de perforación de Fase 1 de exploración contratado para sep-2026; etapa muy temprana)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/CYDVF/century-lithium-files-mine-plan-of-operations-for-angel-island-0v6ql6hprbzu.html)</t>
+          <t>[Kalkine](https://kalkine.com.au/news/announcements/jindalee-lithium-secures-state-permit-for-mcdermitt-drilling-program-contractor-engaged-for-september-2026-start)</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -8701,32 +8691,32 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Silver Peak Lithium Mine (Expansión)</t>
+          <t>Burke Hollow ISR Uranium Project</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Esmeralda County, Nevada, EE.UU.</t>
+          <t>Sur de Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Albemarle Corporation</t>
+          <t>Uranium Energy Corp (UEC)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (operación propia, ISR)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Permitting completo (BLM completó el permitting federal el 27-feb-2026; autorizada operación/expansión en 8,058 acres; incluye construcción de 2 estaciones de bombeo, 2 piscinas de salmuera y tuberías de proceso)</t>
+          <t>Producción (iniciada abr-2026; primera mina ISR nueva en EE.UU. en más de una década; procesa vía Hobson Central Processing Plant bajo modelo hub-and-spoke; expansión continua con nuevos "spokes" satélite en desarrollo en el cinturón de uranio de Texas — infraestructura de tuberías de proceso en expansión activa)</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/press-release/blm-approves-silver-peak-lithium-mine-expansion); [Permitting.gov](https://www.permitting.gov/newsroom/press-releases/silver-peak-lithium-mine-project-completes-federal-permitting)</t>
+          <t>[ANS Nuclear Newswire](https://www.ans.org/news/2026-04-17/article-7945/uranium-energy-corp-begins-production-at-burke-hollow/)</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -8738,32 +8728,32 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>McDermitt Lithium Project (lado Jindalee)</t>
+          <t>Sage Plain Potash Project</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Condado de Malheur, Oregón (límite con Nevada), EE.UU.</t>
+          <t>San Juan County, Utah (cuenca Paradox), EE.UU.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Jindalee Lithium (ASX:JLL / OTCQX:JNDAF)</t>
+          <t>Sage Potash Corp / Critical Mineral Co.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>No especificado (contratista de perforación contratado)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Exploración (permiso estatal de Oregón obtenido para perforación; inicio de perforación de Fase 1 de exploración contratado para sep-2026; etapa muy temprana)</t>
+          <t>Prefactibilidad (avanzando hacia estudio de factibilidad, jun-2026; recibió subvención USDA de US$14 millones —Fertilizer Production Expansion Program—; meta de 300,000 t/año de potasa)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>[Kalkine](https://kalkine.com.au/news/announcements/jindalee-lithium-secures-state-permit-for-mcdermitt-drilling-program-contractor-engaged-for-september-2026-start)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/sage-plain-potash-project-usda-grant/); [Streetwise Reports](https://www.streetwisereports.com/article/2026/06/24/critical-mineral-co-advances-high-grade-utah-potash-project-toward-feasibility.html)</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -8775,32 +8765,32 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Burke Hollow ISR Uranium Project</t>
+          <t>Ann Mason Copper-Molybdenum Project</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sur de Texas, EE.UU.</t>
+          <t>Yerington, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Uranium Energy Corp (UEC)</t>
+          <t>Hudbay Minerals (vía Mason Resources)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>No especificado (operación propia, ISR)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Producción (iniciada abr-2026; primera mina ISR nueva en EE.UU. en más de una década; procesa vía Hobson Central Processing Plant bajo modelo hub-and-spoke; expansión continua con nuevos "spokes" satélite en desarrollo en el cinturón de uranio de Texas — infraestructura de tuberías de proceso en expansión activa)</t>
+          <t>Evaluación Económica Preliminar (PEA) avanzada; 4° depósito porfídico de cobre más grande de Norteamérica; vida de mina de 21 años proyectada; aún no en permisos/construcción formal</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>[ANS Nuclear Newswire](https://www.ans.org/news/2026-04-17/article-7945/uranium-energy-corp-begins-production-at-burke-hollow/)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/projects/ann-mason-copper-molybdenum-project-nevada/)</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -8812,17 +8802,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Sage Plain Potash Project</t>
+          <t>Fresnillo — Portafolio próxima generación (Rodeo, Tajitos, Guanajuato Sur, Novador)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>San Juan County, Utah (cuenca Paradox), EE.UU.</t>
+          <t>Sonora y Guanajuato, México (varias ubicaciones)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Sage Potash Corp / Critical Mineral Co.</t>
+          <t>Fresnillo plc</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -8832,12 +8822,12 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Prefactibilidad (avanzando hacia estudio de factibilidad, jun-2026; recibió subvención USDA de US$14 millones —Fertilizer Production Expansion Program—; meta de 300,000 t/año de potasa)</t>
+          <t>Exploración/prefactibilidad/ingeniería temprana (anunciado 7-sep-2026; Tajitos: capex preliminar US$400-450M, proyecto brownfield junto a Herradura, Sonora; Rodeo: PEA revisada, ~90-110k oz Au/año, arranque fin-2029/2030 sujeto a permisos; Guanajuato Sur: 15-17M oz Ag/año desde ~2033; Novador: ~200k oz Au/año potencial; etapa muy temprana, solo para monitoreo)</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/sage-plain-potash-project-usda-grant/); [Streetwise Reports](https://www.streetwisereports.com/article/2026/06/24/critical-mineral-co-advances-high-grade-utah-potash-project-toward-feasibility.html)</t>
+          <t>[MineAcademy](https://mineacademy.mx/fresnillo-plc-fortalece-su-cartera-de-proyectos-para-sostener-el-crecimiento-de-largo-plazo/)</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -8849,17 +8839,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Ann Mason Copper-Molybdenum Project</t>
+          <t>Reina del Cobre (proyecto polimetálico)</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Yerington, Nevada, EE.UU.</t>
+          <t>Cuencamé, Durango, México (junto a Velardeña)</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Hudbay Minerals (vía Mason Resources)</t>
+          <t>Industrias Peñoles</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -8869,12 +8859,12 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Evaluación Económica Preliminar (PEA) avanzada; 4° depósito porfídico de cobre más grande de Norteamérica; vida de mina de 21 años proyectada; aún no en permisos/construcción formal</t>
+          <t>Exploración (11,071 m perforados en 16 barrenos completos, ago-2026; recursos inferidos ~28.8-30 Mt @ ~2.0% CuEq; estudio económico preliminar planeado; etapa muy temprana)</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/projects/ann-mason-copper-molybdenum-project-nevada/)</t>
+          <t>[Milenio](https://www.milenio.com/estados/mina-velardena-pieza-clave-produccion-zinc-penoles)</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -8886,17 +8876,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Fresnillo — Portafolio próxima generación (Rodeo, Tajitos, Guanajuato Sur, Novador)</t>
+          <t>Springer Tungsten Complex</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sonora y Guanajuato, México (varias ubicaciones)</t>
+          <t>Imlay, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Fresnillo plc</t>
+          <t>Blue Moon Metals Inc. (mina y molino) / JV planta APT: The Elmet Group (70%), Blue Moon Metals (20%), EQ Resources (10%)</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -8906,34 +8896,34 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Exploración/prefactibilidad/ingeniería temprana (anunciado 7-sep-2026; Tajitos: capex preliminar US$400-450M, proyecto brownfield junto a Herradura, Sonora; Rodeo: PEA revisada, ~90-110k oz Au/año, arranque fin-2029/2030 sujeto a permisos; Guanajuato Sur: 15-17M oz Ag/año desde ~2033; Novador: ~200k oz Au/año potencial; etapa muy temprana, solo para monitoreo)</t>
+          <t>Reactivación anunciada (inversión US$150-175 millones, 11-14-sep-2026: mina open-pit + subterránea, molino de 1,200 tpd, y planta de paratungstato de amonio —APT— hasta 4,000 ton/año; Departamento de Guerra de EE.UU. comprometió US$450 millones adicionales a The Elmet Group, 14-sep-2026, para asegurar cadena de suministro de tungsteno; reinicio mina/molino previsto Q4 2027, planta APT H2 2028)</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>[MineAcademy](https://mineacademy.mx/fresnillo-plc-fortalece-su-cartera-de-proyectos-para-sostener-el-crecimiento-de-largo-plazo/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/blue-moon-the-elmet-group-and-eq-resources-announce-a-us150-175-million-investment-into-the-springer-tungsten-complex-nevada-to-strengthen-the-us-tungsten-supply-chain-302877075.html); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/14/3360841/0/en/department-of-war-makes-landmark-450-million-committed-investment-in-the-elmet-group-to-secure-america-s-tungsten-supply-chain.html)</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Reina del Cobre (proyecto polimetálico)</t>
+          <t>Sunshine Complex (Molino, Refinería Plata-Cobre y Planta de Antimonio)</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Cuencamé, Durango, México (junto a Velardeña)</t>
+          <t>Kellogg, Idaho (Silver Valley), EE.UU.</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Industrias Peñoles</t>
+          <t>Sunshine Silver Mining &amp; Refining Co.</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -8943,12 +8933,12 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Exploración (11,071 m perforados en 16 barrenos completos, ago-2026; recursos inferidos ~28.8-30 Mt @ ~2.0% CuEq; estudio económico preliminar planeado; etapa muy temprana)</t>
+          <t>Estudios de factibilidad en curso (desmantelación del molino existente para construir uno nuevo, a completarse fin de 2026; estudios de factibilidad para reabrir la Refinería Plata-Cobre y construir una nueva Planta de Antimonio —hasta 34.5 millones lb/año—, entrega prevista inicios de 2027; estudio de factibilidad de la mina concluye Q2 2027; meta de reinicio de producción de plata fin de 2028)</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>[Milenio](https://www.milenio.com/estados/mina-velardena-pieza-clave-produccion-zinc-penoles)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/sunshine-silver-mining--refining-reports-second-quarter-2026-results-302850131.html); [World Energy](https://www.world-energy.org/article/54143.html)</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -8960,17 +8950,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Springer Tungsten Complex</t>
+          <t>USA Rare Earth — Planta de Metal y Magnetos Blacksburg</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Imlay, Nevada, EE.UU.</t>
+          <t>Blacksburg, Carolina del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Blue Moon Metals Inc. (mina y molino) / JV planta APT: The Elmet Group (70%), Blue Moon Metals (20%), EQ Resources (10%)</t>
+          <t>USA Rare Earth (recién fusionada con Serra Verde Group, anunciado 4-sep-2026)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -8980,34 +8970,34 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Reactivación anunciada (inversión US$150-175 millones, 11-14-sep-2026: mina open-pit + subterránea, molino de 1,200 tpd, y planta de paratungstato de amonio —APT— hasta 4,000 ton/año; Departamento de Guerra de EE.UU. comprometió US$450 millones adicionales a The Elmet Group, 14-sep-2026, para asegurar cadena de suministro de tungsteno; reinicio mina/molino previsto Q4 2027, planta APT H2 2028)</t>
+          <t>Construcción (groundbreaking 9-sep-2026; inversión ~US$1,200 millones; ~490 empleos; planta de metal y manufactura de magnetos de tierras raras)</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/blue-moon-the-elmet-group-and-eq-resources-announce-a-us150-175-million-investment-into-the-springer-tungsten-complex-nevada-to-strengthen-the-us-tungsten-supply-chain-302877075.html); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/14/3360841/0/en/department-of-war-makes-landmark-450-million-committed-investment-in-the-elmet-group-to-secure-america-s-tungsten-supply-chain.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/09/3358813/0/en/usa-rare-earth-breaks-ground-on-advanced-rare-earth-metal-and-magnet-manufacturing-facility-in-blacksburg-south-carolina.html)</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Sunshine Complex (Molino, Refinería Plata-Cobre y Planta de Antimonio)</t>
+          <t>La Negra Project (expansión)</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Kellogg, Idaho (Silver Valley), EE.UU.</t>
+          <t>Ciudad de Querétaro, Querétaro, México</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Sunshine Silver Mining &amp; Refining Co.</t>
+          <t>Silverco Mining (ex Nuevo Silver; adquisición completada may-2026)</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -9017,89 +9007,15 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Estudios de factibilidad en curso (desmantelación del molino existente para construir uno nuevo, a completarse fin de 2026; estudios de factibilidad para reabrir la Refinería Plata-Cobre y construir una nueva Planta de Antimonio —hasta 34.5 millones lb/año—, entrega prevista inicios de 2027; estudio de factibilidad de la mina concluye Q2 2027; meta de reinicio de producción de plata fin de 2028)</t>
+          <t>Ingeniería/optimización (mina de plata-plomo-zinc-cobre tipo skarn en operación con más de 5 décadas de historia; PEA publicado 23-sep-2026 con VAN de US$329 millones sobre inversión de solo US$20.9 millones, vida de mina de 8.2 años; meta de expansión de capacidad de procesamiento a 2,500 tpd para 2S-2027, producción promedio estimada 4.1 millones oz eq. plata/año; programa de 15,000 m de perforación en curso para revalidar el depósito skarn)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/sunshine-silver-mining--refining-reports-second-quarter-2026-results-302850131.html); [World Energy](https://www.world-energy.org/article/54143.html)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/09/silverco-mining-proyecto-la-negra-en-queretaro-proyecta-van-de-us329-millones/); [Minart](https://minart.pe/2026/09/23/silverco-proyecta-us329-millones-de-valor-para-la-mina-la-negra-y-una-vida-util-de-82-anos/)</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>USA Rare Earth — Planta de Metal y Magnetos Blacksburg</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Blacksburg, Carolina del Sur, EE.UU.</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>USA Rare Earth (recién fusionada con Serra Verde Group, anunciado 4-sep-2026)</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Construcción (groundbreaking 9-sep-2026; inversión ~US$1,200 millones; ~490 empleos; planta de metal y manufactura de magnetos de tierras raras)</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/09/09/3358813/0/en/usa-rare-earth-breaks-ground-on-advanced-rare-earth-metal-and-magnet-manufacturing-facility-in-blacksburg-south-carolina.html)</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>La Negra Project (expansión)</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Ciudad de Querétaro, Querétaro, México</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Silverco Mining (ex Nuevo Silver; adquisición completada may-2026)</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Ingeniería/optimización (mina de plata-plomo-zinc-cobre tipo skarn en operación con más de 5 décadas de historia; PEA publicado 23-sep-2026 con VAN de US$329 millones sobre inversión de solo US$20.9 millones, vida de mina de 8.2 años; meta de expansión de capacidad de procesamiento a 2,500 tpd para 2S-2027, producción promedio estimada 4.1 millones oz eq. plata/año; programa de 15,000 m de perforación en curso para revalidar el depósito skarn)</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/09/silverco-mining-proyecto-la-negra-en-queretaro-proyecta-van-de-us329-millones/); [Minart](https://minart.pe/2026/09/23/silverco-proyecta-us329-millones-de-valor-para-la-mina-la-negra-y-una-vida-util-de-82-anos/)</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
@@ -9116,8 +9032,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9253,17 +9178,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales</t>
+          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales (expansión de 10 a 49 turbinas); TCEQ otorgó reunión pública sobre esta solicitud a petición del representante estatal Stan Lambert (~10-sep-2026), periodo de comentarios abierto; además, el gobernador Greg Abbott ordenó el 21-sep-2026 a la TCEQ pausar toda emisión de permisos nuevos para proyectos de data centers en Texas —incluidas instalaciones con generación propia "behind-the-meter"— hasta que ERCOT complete una auditoría de red (esperada mediados de dic-2026; TCEQ debe reportar cumplimiento al 19-oct-2026), lo que podría retrasar trámites pendientes de este y otros proyectos texanos del tracker</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/); [Texas Tribune](https://www.texastribune.org/2026/09/21/texas-data-center-moratorium-water-energy/); [Bracewell](https://www.bracewell.com/resources/governor-abbott-orders-tceq-to-pause-all-permit-issuance-for-data-center-projects/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -10585,17 +10510,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total); Fermi Inc. anunció 28-sep-2026 acuerdo de operación y mantenimiento (O&amp;M) con NAES Corporation —mayor operador independiente de plantas de energía de EE.UU.— para operar y mantener la flota de turbinas de gas natural del campus; Fermi retiene la propiedad de los activos, NAES opera; primeras turbinas de gas Siemens Energy SGT6-5000F ya llegaron a sitio; a inicios de sep-2026 Fermi también contrató a CBRE para operar/mantener su primer data center en Matador</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [StockTitan — NAES O&amp;M](https://www.stocktitan.net/news/FRMI/fermi-selects-naes-to-operate-and-maintain-its-natural-gas-turbine-qvztuks7g3tn.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -13556,6 +13481,43 @@
       <c r="G120" t="inlineStr">
         <is>
           <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Encinal Gas Power Plant</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Encinal, Webb County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Propuesta como JV 50/50 entre inversionistas surcoreanos (bajo el pacto comercial Corea-EE.UU. de US$350,000 millones) y socios estadounidenses; sin hyperscaler/cliente de cómputo IA nombrado aún</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Negociación/no confirmado (acuerdo de ~US$22,300 millones para planta de 6.3 GW —sería la más grande de ERCOT, ninguna planta de gas en Texas supera ~2 GW hoy—, destinada a alimentar data centers de IA y plantas de semiconductores; Fase 2 convertiría turbinas de Fase 1 a ciclo combinado y añadiría 4.9 GW; el Ministerio de Industria de Corea del Sur desmintió que el acuerdo esté cerrado, señalando que las consultas con Washington continúan, pendiente revisión parlamentaria coreana y aprobación de comité de inversión de EE.UU.; mantener en watch-list hasta anuncio oficial)</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>[TechRadar Pro](https://www.techradar.com/pro/south-korea-us-agree-on-usd22-billion-deal-for-6-3-gw-texas-gas-power-plant-encinal-facility-to-feed-ai-data-centers-under-washington-and-seouls-usd350-billion-pact); [Construction Review Online](https://constructionreviewonline.com/south-korea-eyes-22-3bn-encinal-gas-fired-power-plant-in-texas-for-ai-data-center-operations/); [Korean Tech Texas](https://koreantechtexas.com/korea-encinal-texas-gas-power-plant/)</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker 2026-09-30: +Rio Grande LNG Train 6, +Vantage Frontier (#51)
* Tracker: agrega Rio Grande LNG Train 6 y Vantage Frontier (2026-09-30)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015QnCKhKz6BMFtFnzkH6UtU

* Actualiza proyectos.xlsx

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015QnCKhKz6BMFtFnzkH6UtU

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -418,15 +418,6 @@
   </sheetPr>
   <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2548,17 +2539,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4370,6 +4352,43 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Rio Grande LNG Train 6 (expansión)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Brownsville, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NextDecade</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>No especificado (Trenes 4-5 con Bechtel)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Pre-permisos: pre-filing FERC iniciado (nov-2025), solicitud completa esperada en 2026; FID del Tren 6 planeado para 2027</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>[Argus](https://www.argusmedia.com/en/news-and-insights/latest-market-news/2781660-rio-grande-lng-plans-train-6-fid-in-2027-ceo); [BusinessWire](https://www.businesswire.com/news/home/20251124057319/en/NextDecade-Initiates-Pre-Filing-Process-with-FERC-for-Train-6-at-Rio-Grande-LNG)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -4386,15 +4405,6 @@
   </sheetPr>
   <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9032,17 +9042,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -13518,6 +13519,43 @@
       <c r="G121" t="inlineStr">
         <is>
           <t>2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers "Frontier" (mega-campus 1.4 GW, ~USD 25 mil millones)</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Shackelford County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Anunciado / desarrollo y construcción por fases</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>[Intelligent CIO](https://www.intelligentcio.com/north-america/?p=48937)</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenera proyectos.xlsx (incluye Layer 9 Project Falcon)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EfBbFfvL1AEkibF837j3Dg
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -9042,7 +9042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13559,6 +13559,43 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Layer 9 Data Centers — Project Falcon (campus 96 MW)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Celaya, Guanajuato, México</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Layer 9 Data Centers</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Planeación/desarrollo (fase exacta no verificada; fuente consultada solo vía resumen de búsqueda)</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>[BNamericas](https://bnamericas.com/en/news/snapshot-layer-9-data-centers-massive-mexican-project); [DataCenterMap](https://datacentermap.com/mexico/celaya/layer-9-project-falcon)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-01: agrega Layer 9 Project Falcon (Data Centers) (#52)
* Monitoreo 2026-10-01: agrega Layer 9 Project Falcon (Data Centers)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EfBbFfvL1AEkibF837j3Dg

* Regenera proyectos.xlsx (incluye Layer 9 Project Falcon)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EfBbFfvL1AEkibF837j3Dg

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -9042,7 +9042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13559,6 +13559,43 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Layer 9 Data Centers — Project Falcon (campus 96 MW)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Celaya, Guanajuato, México</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Layer 9 Data Centers</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Planeación/desarrollo (fase exacta no verificada; fuente consultada solo vía resumen de búsqueda)</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>[BNamericas](https://bnamericas.com/en/news/snapshot-layer-9-data-centers-massive-mexican-project); [DataCenterMap](https://datacentermap.com/mexico/celaya/layer-9-project-falcon)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-02: +Beaumont New Ammonia T2 (Petroquímica), +Crow Holdings Dallas (Data Centers)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVtyJb7WXDMJBzyNjYsXGX
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2525,6 +2525,43 @@
       <c r="G57" t="inlineStr">
         <is>
           <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Beaumont New Ammonia — Tren 2 (amoniaco azul, 1.1 Mtpa)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Beaumont, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Woodside Energy (ex-OCI Clean Ammonia)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Por definir (Tren 1 en comisionamiento; Tren 2 aprobado por TCEQ)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Pre-FID — Woodside apunta a tener el Tren 2 listo para FID en 2026</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>[QCIntel](https://www.qcintel.com/ammonia/article/woodside-eyes-second-beaumont-blue-ammonia-fid-in-2026-33250.html); [QCIntel TCEQ](https://www.qcintel.com/ammonia/article/tceq-approves-second-ammonia-train-for-beaumont-new-ammonia-47266.html)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -9042,7 +9079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13596,6 +13633,43 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Crow Holdings / CleanArc — Campus Stemmons Corridor (245 MW)</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Dallas, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Crow Holdings (con CleanArc Data Centers)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Ingeniería/diseño iniciado; primer edificio de 70 MW previsto para finales de 2027</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cleanarc-partners-with-crow-holdings-for-245mw-campus-in-dallas-texas/); [BusinessWire](https://www.businesswire.com/news/home/20260120363268/en/Crow-Holdings-Announces-245MW-Flagship-Data-Center-Campus-in-Central-Dallas)</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-02: +Beaumont New Ammonia T2 (Petroquímica), +Crow Holdings Dallas (Data Centers) (#53)
Claude-Session: https://claude.ai/code/session_01RVtyJb7WXDMJBzyNjYsXGX

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2525,6 +2525,43 @@
       <c r="G57" t="inlineStr">
         <is>
           <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Beaumont New Ammonia — Tren 2 (amoniaco azul, 1.1 Mtpa)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Beaumont, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Woodside Energy (ex-OCI Clean Ammonia)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Por definir (Tren 1 en comisionamiento; Tren 2 aprobado por TCEQ)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Pre-FID — Woodside apunta a tener el Tren 2 listo para FID en 2026</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>[QCIntel](https://www.qcintel.com/ammonia/article/woodside-eyes-second-beaumont-blue-ammonia-fid-in-2026-33250.html); [QCIntel TCEQ](https://www.qcintel.com/ammonia/article/tceq-approves-second-ammonia-train-for-beaumont-new-ammonia-47266.html)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -9042,7 +9079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13596,6 +13633,43 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Crow Holdings / CleanArc — Campus Stemmons Corridor (245 MW)</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Dallas, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Crow Holdings (con CleanArc Data Centers)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Ingeniería/diseño iniciado; primer edificio de 70 MW previsto para finales de 2027</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cleanarc-partners-with-crow-holdings-for-245mw-campus-in-dallas-texas/); [BusinessWire](https://www.businesswire.com/news/home/20260120363268/en/Crow-Holdings-Announces-245MW-Flagship-Data-Center-Campus-in-Central-Dallas)</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-07: +River Run Energy Center, +Nakota AI Data Campus (Data Centers)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012eYRucRGmNsGBzVTEPQFYP
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LNG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mining" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9079,7 +9079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13670,6 +13670,80 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>NextEra / Basin Electric — River Run Energy Center (1,450 MW ciclo combinado para campus de data centers)</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Mercer County, North Dakota, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>NextEra Energy Resources / Basin Electric Power Cooperative</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Planeación/ingeniería temprana (MOU dic-2025; solicitud de estudio de interconexión SPP ERAS presentada)</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>[Basin Electric](https://www.basinelectric.com/News-Center/news-releases/Basin-Electric-Power-Cooperative-and-NextEra-Energy-Resources-announce-collaboration-to-bring-responsible-growth-jobs-and-economic-benefits-to-North-Dakota-through-development-of-the-River-Run-Energy-Center); [NextEra](https://www.nexteraenergyresources.com/river-run-energy-center/faq.html)</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Nakota AI Data Campus (hasta 1 GW, energía a gas detrás del medidor, USD 1,000 M)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Williston Basin, North Dakota, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Tachyon9 Corp. / Nixxy Inc. (offtake: Nidar Infrastructure / Yotta)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Planeación/financiamiento; primeros 120-150 MW previstos 2T-2027</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>[PGJ Online](https://www.pgjonline.com/news/2026/june/north-dakota-ai-campus-plans-1-gw-of-gas-fired-power); [BusinessWire](https://secure.businesswire.com/news/home/20260618848981/en/Tachyon9-Secures-Offtake-Agreement-Supporting-%24156-Million-Annual-Revenue-Platform-and-Up-to-1-GW-of-Grid-Independent-AI-Infrastructure-Powered-by-Abundant-North-Dakota-Natural-Gas)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-07: +River Run Energy Center, +Nakota AI Data Campus (Data Centers) (#54)
Claude-Session: https://claude.ai/code/session_012eYRucRGmNsGBzVTEPQFYP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LNG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mining" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9079,7 +9079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13670,6 +13670,80 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>NextEra / Basin Electric — River Run Energy Center (1,450 MW ciclo combinado para campus de data centers)</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Mercer County, North Dakota, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>NextEra Energy Resources / Basin Electric Power Cooperative</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Planeación/ingeniería temprana (MOU dic-2025; solicitud de estudio de interconexión SPP ERAS presentada)</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>[Basin Electric](https://www.basinelectric.com/News-Center/news-releases/Basin-Electric-Power-Cooperative-and-NextEra-Energy-Resources-announce-collaboration-to-bring-responsible-growth-jobs-and-economic-benefits-to-North-Dakota-through-development-of-the-River-Run-Energy-Center); [NextEra](https://www.nexteraenergyresources.com/river-run-energy-center/faq.html)</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Nakota AI Data Campus (hasta 1 GW, energía a gas detrás del medidor, USD 1,000 M)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Williston Basin, North Dakota, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Tachyon9 Corp. / Nixxy Inc. (offtake: Nidar Infrastructure / Yotta)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Planeación/financiamiento; primeros 120-150 MW previstos 2T-2027</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>[PGJ Online](https://www.pgjonline.com/news/2026/june/north-dakota-ai-campus-plans-1-gw-of-gas-fired-power); [BusinessWire](https://secure.businesswire.com/news/home/20260618848981/en/Tachyon9-Secures-Offtake-Agreement-Supporting-%24156-Million-Annual-Revenue-Platform-and-Up-to-1-GW-of-Grid-Independent-AI-Infrastructure-Powered-by-Abundant-North-Dakota-Natural-Gas)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-08: +Nebius Pensilvania, +T5 Grayslake (Data Centers)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChjyMTdHZ5qMXChSLwHLXU
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -9079,7 +9079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13744,6 +13744,80 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Nebius Pensilvania AI Campus (2do campus gigawatt de Nebius en EE.UU.; posible sitio "Highridge", sin confirmar)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Pensilvania, EE.UU. (ubicación exacta no divulgada)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Nebius Group</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Planeación/desarrollo (energía asegurada hasta 1.2 GW; primeros 250-300 MW previstos a fines de 2027, 1.2 GW completos hacia 2030)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>[DCD](https://datacenterdynamics.com/en/news/nebius-plans-second-us-gigawatt-scale-data-center-campus-in-pennsylvania/)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>T5 Grayslake Campus (Chicago; parte de plan de 5 campus de 1 GW con QuadReal)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Grayslake, Illinois, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>T5 Data Centers (JV con QuadReal Property Group)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Desarrollo/construcción temprana (reportes varían: 480 MW originales a 1.2 GW en 20 edificios de 60 MW; primera fase prevista 2027)</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>[DCD](https://datacenterdynamics.com/en/news/t5-plans-five-gigawatt-scale-data-center-campuses-announces-chicago-campus); [Bisnow](https://www.bisnow.com/news/national/deal-sheet/data-center-firm-t5-expanding-footprint-in-atlanta-and-chicago-129337)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-10-08: +Nebius Pensilvania, +T5 Grayslake (Data Centers) (#55)
Claude-Session: https://claude.ai/code/session_01ChjyMTdHZ5qMXChSLwHLXU

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -9079,7 +9079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13744,6 +13744,80 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Nebius Pensilvania AI Campus (2do campus gigawatt de Nebius en EE.UU.; posible sitio "Highridge", sin confirmar)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Pensilvania, EE.UU. (ubicación exacta no divulgada)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Nebius Group</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Planeación/desarrollo (energía asegurada hasta 1.2 GW; primeros 250-300 MW previstos a fines de 2027, 1.2 GW completos hacia 2030)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>[DCD](https://datacenterdynamics.com/en/news/nebius-plans-second-us-gigawatt-scale-data-center-campus-in-pennsylvania/)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>T5 Grayslake Campus (Chicago; parte de plan de 5 campus de 1 GW con QuadReal)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Grayslake, Illinois, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>T5 Data Centers (JV con QuadReal Property Group)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Desarrollo/construcción temprana (reportes varían: 480 MW originales a 1.2 GW en 20 edificios de 60 MW; primera fase prevista 2027)</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>[DCD](https://datacenterdynamics.com/en/news/t5-plans-five-gigawatt-scale-data-center-campuses-announces-chicago-campus); [Bisnow](https://www.bisnow.com/news/national/deal-sheet/data-center-firm-t5-expanding-footprint-in-atlanta-and-chicago-129337)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenera proyectos.xlsx con Taylor Technology Campus
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LPB5RkHTWVc9WNK7uiZ9mZ
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -516,19 +516,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción; contrato EPC de Technip Energies valuado en más de €1,000 millones; capex conjunto 2026 proyectado en US$600 millones prorrateado entre CF Industries (40%), JERA y Mitsui</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/); [DecarbonFuse](https://decarbonfuse.com/posts/blue-point-breaks-ground-what-changes-now-it-s-building)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción; contrato EPC de Technip Energies valuado en más de €1,000 millones; capex conjunto 2026 proyectado en US$600 millones prorrateado entre CF Industries (40%), JERA y Mitsui| [FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/); [DecarbonFuse](https://decarbonfuse.com/posts/blue-point-breaks-ground-what-changes-now-it-s-building)| 2026-09-24</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -595,14 +587,10 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[MEES](https://www.mees.com/2026/9/25/corporate/qatarenergy-poised-to-start-up-texas-ethane-cracker/0ff02300-b8df-11f1-8f86-2b8776a66cca); [BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>[MEES](https://www.mees.com/2026/9/25/corporate/qatarenergy-poised-to-start-up-texas-ethane-cracker/0ff02300-b8df-11f1-8f86-2b8776a66cca); [BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2787,19 +2775,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028) ; Williams Companies sancionó (FID) el gasoducto "Delta Access" (US$1,500 millones, 2.25 Bcf/d iniciales ampliable a 3.5 Bcf/d, de Gillis LA hacia el corredor Transco, en servicio 1T2029) diseñado para alimentar esta expansión vía interconexión con el gasoducto intraestatal Cloud Connector de Venture Global, confirmado en su reporte 2T2026 (4-ago-2026); Baker Hughes recibió (13-sep-2026) nuevas órdenes de equipo mayor para esta expansión: 4 bloques de licuefacción (8 módulos SMR con motor eléctrico, alcance similar al ya adjudicado para CP2) y una segunda orden de paquetes de compresión Frame 5/2E para el gasoducto de alimentación intraestatal Cloud Connector, ampliando la flota total a 23 unidades — confirma actividad activa de fabricación de equipo mayor</t>
+          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028) ; Williams Companies sancionó (FID) el gasoducto "Delta Access" (US$1,500 millones, 2.25 Bcf/d iniciales ampliable a 3.5 Bcf/d, de Gillis LA hacia el corredor Transco, en servicio 1T2029) diseñado para alimentar esta expansión vía interconexión con el gasoducto intraestatal Cloud Connector de Venture Global, confirmado en su reporte 2T2026 (4-ago-2026); Baker Hughes recibió (13-sep-2026) nuevas órdenes de equipo mayor para esta expansión: 4 bloques de licuefacción (8 módulos SMR con motor eléctrico, alcance similar al ya adjudicado para CP2) y una segunda orden de paquetes de compresión Frame 5/2E para el gasoducto de alimentación intraestatal Cloud Connector, ampliando la flota total a 23 unidades — confirma actividad activa de fabricación de equipo mayor| [Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848); [Natural Gas Intel](https://www.naturalgasintel.com/news/plaquemines-expansion-to-anchor-east-end-of-williams-delta-access/); [World Pipelines](https://www.worldpipelines.com/contracts-and-tenders/14092026/baker-hughes-and-venture-global-advance-next-phase-of-us-gas-infrastructure-growth/)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848); [Natural Gas Intel](https://www.naturalgasintel.com/news/plaquemines-expansion-to-anchor-east-end-of-williams-delta-access/); [World Pipelines](https://www.worldpipelines.com/contracts-and-tenders/14092026/baker-hughes-and-venture-global-advance-next-phase-of-us-gas-infrastructure-growth/)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
           <t>2026-09-13</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4503,19 +4487,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (Estudio de Prefactibilidad —PFS— 2026 publicado 23-sep-2026: capex inicial elevado a US$1,430 millones, costo operativo US$1.47/lb, VPN después de impuestos US$3,500 millones, TIR 30%; mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; "box cut" —corte de acceso a la mina— previsto para iniciar octubre 2026; carta preliminar de US$1,100 millones del Export-Import Bank de EE.UU., aprobación final esperada primavera 2027; primera producción de cátodo de cobre prevista 2029) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>[Ivanhoe Electric — PFS 2026](https://ivanhoeelectric.com/news/2026-preliminary-feasibility-study-for-the-santa-cruz-copper-project-in-arizona-confirms-high-grade-low-cost-project-with-strong-economics/); [Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>Construcción (Estudio de Prefactibilidad —PFS— 2026 publicado 23-sep-2026: capex inicial elevado a US$1,430 millones, costo operativo US$1.47/lb, VPN después de impuestos US$3,500 millones, TIR 30%; mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; "box cut" —corte de acceso a la mina— previsto para iniciar octubre 2026; carta preliminar de US$1,100 millones del Export-Import Bank de EE.UU., aprobación final esperada primavera 2027; primera producción de cátodo de cobre prevista 2029) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins| [Ivanhoe Electric — PFS 2026](https://ivanhoeelectric.com/news/2026-preliminary-feasibility-study-for-the-santa-cruz-copper-project-in-arizona-confirms-high-grade-low-cost-project-with-strong-economics/); [Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4540,19 +4516,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción) ; bajo Hudbay Minerals (tras adquisición de Arizona Sonoran Copper, jun-2026), definitive feasibility study previsto para mediados de 2026, con FID esperada después en 2026</t>
+          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción) ; bajo Hudbay Minerals (tras adquisición de Arizona Sonoran Copper, jun-2026), definitive feasibility study previsto para mediados de 2026, con FID esperada después en 2026| [SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4577,19 +4549,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones ; otorgó contratos por ~US$110 millones a Major Drilling America y Redpath USA Corporation para avanzar exploración y desarrollo subterráneo</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/) ; [Mining Technology](https://www.mining-technology.com/news/resolution-copper-110m-contracts-arizona-mine-2/)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones ; otorgó contratos por ~US$110 millones a Major Drilling America y Redpath USA Corporation para avanzar exploración y desarrollo subterráneo| [SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/) ; [Mining Technology](https://www.mining-technology.com/news/resolution-copper-110m-contracts-arizona-mine-2/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4614,19 +4578,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; obra estructural/concreto de la planta de proceso avanzando con transición a oficios de tubería (piping) y eléctricos; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027; energización prevista 4T2026) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx) ; [Carbon Credits](https://carboncredits.com/u-s-doe-approves-2-26-billion-for-nevada-lithium-mine/)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; obra estructural/concreto de la planta de proceso avanzando con transición a oficios de tubería (piping) y eléctricos; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027; energización prevista 4T2026) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026| [Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx) ; [Carbon Credits](https://carboncredits.com/u-s-doe-approves-2-26-billion-for-nevada-lithium-mine/)| 2026-08-28</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4651,19 +4607,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026; confirmado (sep-2026) como parte de paquete de 6 complejos mineros en Zacatecas con autorizaciones federales principales (incl. Semarnat) ya obtenidas, inversión conjunta ~US$6,500 millones y ~15,000 empleos directos proyectados a partir de 2027; suministro de agua vía acueducto de ~50 km mediante convenio con la Junta Intermunicipal de Agua Potable y Alcantarillado de Zacatecas (JIAPAZ), con objetivo de reciclar el agua usada por la mina</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/) ; [Forbes México](https://forbes.com.mx/destraban-proyectos-mineros-en-zacatecas-por-6500-mdd/)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026; confirmado (sep-2026) como parte de paquete de 6 complejos mineros en Zacatecas con autorizaciones federales principales (incl. Semarnat) ya obtenidas, inversión conjunta ~US$6,500 millones y ~15,000 empleos directos proyectados a partir de 2027; suministro de agua vía acueducto de ~50 km mediante convenio con la Junta Intermunicipal de Agua Potable y Alcantarillado de Zacatecas (JIAPAZ), con objetivo de reciclar el agua usada por la mina| [Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/) ; [Forbes México](https://forbes.com.mx/destraban-proyectos-mineros-en-zacatecas-por-6500-mdd/)| 2026-09-21</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4725,19 +4673,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu) ; Southern Copper obtuvo los permisos ambientales necesarios; trabajos preliminares de sitio inician sep-2026, con construcción del proyecto arrancando en 1T2027</t>
+          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu) ; Southern Copper obtuvo los permisos ambientales necesarios; trabajos preliminares de sitio inician sep-2026, con construcción del proyecto arrancando en 1T2027| [BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico); [Dossier Político](https://dossierpolitico.com/2026/07/28/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/); [Mexico Business News](https://mexicobusiness.news/mining/news/southern-copper-unlocks-environmental-permits-el-pilar)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico); [Dossier Político](https://dossierpolitico.com/2026/07/28/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/); [Mexico Business News](https://mexicobusiness.news/mining/news/southern-copper-unlocks-environmental-permits-el-pilar)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4947,19 +4891,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027) ; en construcción con presupuesto de US$180 millones; inicio de operaciones proyectado en 2026</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027) ; en construcción con presupuesto de US$180 millones; inicio de operaciones proyectado en 2026| [Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5021,19 +4957,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción) ; BLM aprobó el proyecto el 14-ago-2026, habilitando a Gold Standard Ventures (US) Inc. a iniciar la mina; construcción emplearía hasta 600 personas</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production) ; [BLM](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción) ; BLM aprobó el proyecto el 14-ago-2026, habilitando a Gold Standard Ventures (US) Inc. a iniciar la mina; construcción emplearía hasta 600 personas| [StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production) ; [BLM](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5169,19 +5097,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026) ; equipos mayores (espesador, filtro prensa, planta de mezcla) en fabricación con entregas desde jun-2026; construcción civil en marcha desde may-2026; puesta en marcha prevista 4T2026; capex total US$11.9 millones</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html) ; [SEC 6-K Americas Gold &amp; Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002149/exhibit99-1.htm)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026) ; equipos mayores (espesador, filtro prensa, planta de mezcla) en fabricación con entregas desde jun-2026; construcción civil en marcha desde may-2026; puesta en marcha prevista 4T2026; capex total US$11.9 millones| [GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html) ; [SEC 6-K Americas Gold &amp; Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002149/exhibit99-1.htm)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5761,19 +5681,15 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029) ; Standard Lithium completó el definitive feasibility study (DFS) tras finalizar el FEED; se espera FID y arranque de construcción en 2026, con 2-3 años de construcción/comisionamiento</t>
+          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029) ; Standard Lithium completó el definitive feasibility study (DFS) tras finalizar el FEED; se espera FID y arranque de construcción en 2026, con 2-3 años de construcción/comisionamiento| [InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); [StockTitan/SEC 6-K](https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); [StockTitan/SEC 6-K](https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5872,19 +5788,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028) ; Centerra Gold finalizará estudios de ingeniería, lanzará adquisiciones de largo plazo e iniciará trabajos de establecimiento de sitio durante 2026</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/) ; [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028) ; Centerra Gold finalizará estudios de ingeniería, lanzará adquisiciones de largo plazo e iniciará trabajos de establecimiento de sitio durante 2026| [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/) ; [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5909,19 +5817,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027) ; Hudbay Minerals completó la adquisición de Arizona Sonoran Copper el 24-jun-2026, creando el tercer distrito cuprífero más grande de Norteamérica; feasibility study esperado 2S2026, FID posible 4T2026</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/) ; [Hudbay Minerals](https://hudbayminerals.com/investors/press-releases/press-release-details/2026/Hudbay-Completes-Acquisition-of-Arizona-Sonoran-to-Create-the-Third-Largest-Copper-District-in-North-America/default.aspx)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027) ; Hudbay Minerals completó la adquisición de Arizona Sonoran Copper el 24-jun-2026, creando el tercer distrito cuprífero más grande de Norteamérica; feasibility study esperado 2S2026, FID posible 4T2026| [GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/) ; [Hudbay Minerals](https://hudbayminerals.com/investors/press-releases/press-release-details/2026/Hudbay-Completes-Acquisition-of-Arizona-Sonoran-to-Create-the-Third-Largest-Copper-District-in-North-America/default.aspx)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6057,19 +5957,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027 ; RMS preparó estimación de capital para planta de relleno en pasta: US$99 millones en construcción inicial más US$20 millones en capital sostenido para expansión del sistema de distribución subterránea</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data) ; [SEC 6-K Pan American Silver](https://www.sec.gov/Archives/edgar/data/0000771992/000077199226000047/a20260428pasni43-101xworki.htm)</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027 ; RMS preparó estimación de capital para planta de relleno en pasta: US$99 millones en construcción inicial más US$20 millones en capital sostenido para expansión del sistema de distribución subterránea| [Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data) ; [SEC 6-K Pan American Silver](https://www.sec.gov/Archives/edgar/data/0000771992/000077199226000047/a20260428pasni43-101xworki.htm)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6945,19 +6837,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027| [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7759,19 +7643,11 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028| [KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7833,19 +7709,11 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar| [Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9079,7 +8947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9142,19 +9010,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026) ; VoltaGrid fue aprobado por TCEQ para operar 210 generadores industriales a gas (700 MW: 197 generación primaria + 13 respaldo) con motores Jenbacher; Vantage Data Centers confirmado como socio desarrollador; primer edificio previsto para fines de 2026</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid) ; [Construction Owners Association](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026) ; VoltaGrid fue aprobado por TCEQ para operar 210 generadores industriales a gas (700 MW: 197 generación primaria + 13 respaldo) con motores Jenbacher; Vantage Data Centers confirmado como socio desarrollador; primer edificio previsto para fines de 2026| [DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid) ; [Construction Owners Association](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9216,19 +9076,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales (expansión de 10 a 49 turbinas); TCEQ otorgó reunión pública sobre esta solicitud a petición del representante estatal Stan Lambert (~10-sep-2026), periodo de comentarios abierto; además, el gobernador Greg Abbott ordenó el 21-sep-2026 a la TCEQ pausar toda emisión de permisos nuevos para proyectos de data centers en Texas —incluidas instalaciones con generación propia "behind-the-meter"— hasta que ERCOT complete una auditoría de red (esperada mediados de dic-2026; TCEQ debe reportar cumplimiento al 19-oct-2026), lo que podría retrasar trámites pendientes de este y otros proyectos texanos del tracker</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/); [Texas Tribune](https://www.texastribune.org/2026/09/21/texas-data-center-moratorium-water-energy/); [Bracewell](https://www.bracewell.com/resources/governor-abbott-orders-tceq-to-pause-all-permit-issuance-for-data-center-projects/)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales (expansión de 10 a 49 turbinas); TCEQ otorgó reunión pública sobre esta solicitud a petición del representante estatal Stan Lambert (~10-sep-2026), periodo de comentarios abierto; además, el gobernador Greg Abbott ordenó el 21-sep-2026 a la TCEQ pausar toda emisión de permisos nuevos para proyectos de data centers en Texas —incluidas instalaciones con generación propia "behind-the-meter"— hasta que ERCOT complete una auditoría de red (esperada mediados de dic-2026; TCEQ debe reportar cumplimiento al 19-oct-2026), lo que podría retrasar trámites pendientes de este y otros proyectos texanos del tracker| [DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/); [Texas Tribune](https://www.texastribune.org/2026/09/21/texas-data-center-moratorium-water-energy/); [Bracewell](https://www.bracewell.com/resources/governor-abbott-orders-tceq-to-pause-all-permit-issuance-for-data-center-projects/)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9253,19 +9105,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026) ; Chevron (vía subsidiaria Energy Forge One LLC) firmó PPA a 20 años con Microsoft; 2.67 GW de capacidad, turbinas principalmente GE Vernova más Solar Turbines (Caterpillar); ubicación precisada en Condado de Reeves (2,000+ acres); FID esperada fin de 2026, arranque 2028</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center) ; [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026) ; Chevron (vía subsidiaria Energy Forge One LLC) firmó PPA a 20 años con Microsoft; 2.67 GW de capacidad, turbinas principalmente GE Vernova más Solar Turbines (Caterpillar); ubicación precisada en Condado de Reeves (2,000+ acres); FID esperada fin de 2026, arranque 2028| [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center) ; [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9475,19 +9319,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT) ; Amazon confirmó públicamente su propiedad del proyecto; permiso otorgado para 35 turbinas de gas natural (hasta 7.65 GW), el permiso de emisiones más grande otorgado este año en el país (~33 millones de toneladas de CO2/año); incluye hasta 750 MW solar y 1.8 GW de almacenamiento en baterías; primera energía prevista 1T2027, 1 GW en servicio en 2028</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases) ; [ENR](https://www.enr.com/articles/63464-amazon-discloses-ownership-of-gw-ranch-giant-texas-data-center-gas-power-complex)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT) ; Amazon confirmó públicamente su propiedad del proyecto; permiso otorgado para 35 turbinas de gas natural (hasta 7.65 GW), el permiso de emisiones más grande otorgado este año en el país (~33 millones de toneladas de CO2/año); incluye hasta 750 MW solar y 1.8 GW de almacenamiento en baterías; primera energía prevista 1T2027, 1 GW en servicio en 2028| [Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases) ; [ENR](https://www.enr.com/articles/63464-amazon-discloses-ownership-of-gw-ranch-giant-texas-data-center-gas-power-complex)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9623,19 +9459,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027) ; Oracle/BorderPlex Digital Assets cambiaron el plan de generación de turbinas de gas/generadores diésel a un microgrid de celdas de combustible para reducir uso de agua e impacto en calidad del aire; gasoducto asociado 'Green Chile Project' (~US$60 millones, 17.7 millas) bajo revisión FERC enfrenta protesta de personal regulador federal, entrada en servicio prevista ago-2026</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027) ; [Source NM](https://sourcenm.com/2026/04/27/nm-project-jupiter-data-center-developers-announce-new-plans-for-generating-power/)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027) ; Oracle/BorderPlex Digital Assets cambiaron el plan de generación de turbinas de gas/generadores diésel a un microgrid de celdas de combustible para reducir uso de agua e impacto en calidad del aire; gasoducto asociado 'Green Chile Project' (~US$60 millones, 17.7 millas) bajo revisión FERC enfrenta protesta de personal regulador federal, entrada en servicio prevista ago-2026| [Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027) ; [Source NM](https://sourcenm.com/2026/04/27/nm-project-jupiter-data-center-developers-announce-new-plans-for-generating-power/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9734,19 +9562,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Planeación temprana (opción de terreno) ; se formalizó opción de compra de ~3,500 acres en Condado de Lea, Nuevo México, para hub de IA de 7 GW; marca el primer desarrollo enteramente propio, separado del joint venture TCDC; planea &gt;2 GW de gas natural más 5+ GW de generación nuclear</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/) ; [Barchart](https://www.barchart.com/story/news/35949566/new-era-energy-digital-enters-into-land-option-purchase-agreement-for-3-500-acres-in-new-mexico-for-7gw-ai-data-center-hub-marks-first-wholly-owned-development-separate-from-tcdc-joint-venture)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Planeación temprana (opción de terreno) ; se formalizó opción de compra de ~3,500 acres en Condado de Lea, Nuevo México, para hub de IA de 7 GW; marca el primer desarrollo enteramente propio, separado del joint venture TCDC; planea &gt;2 GW de gas natural más 5+ GW de generación nuclear| [PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/) ; [Barchart](https://www.barchart.com/story/news/35949566/new-era-energy-digital-enters-into-land-option-purchase-agreement-for-3-500-acres-in-new-mexico-for-7gw-ai-data-center-hub-marks-first-wholly-owned-development-separate-from-tcdc-joint-venture)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10289,19 +10109,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos) ; OpenAI se unió como inversionista/arrendatario; Nvidia garantiza hasta US$105,000 millones en obligaciones de arrendamiento y pago de energía; escala confirmada en 8 IT-GW de cómputo/10 GW de generación nueva (9.2 GW de gas natural); costo total potencial hasta US$500,000 millones; primera fase de 800 MW en operación en 2028</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html) ; [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos) ; OpenAI se unió como inversionista/arrendatario; Nvidia garantiza hasta US$105,000 millones en obligaciones de arrendamiento y pago de energía; escala confirmada en 8 IT-GW de cómputo/10 GW de generación nueva (9.2 GW de gas natural); costo total potencial hasta US$500,000 millones; primera fase de 800 MW en operación en 2028| [DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html) ; [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10548,19 +10360,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total); Fermi Inc. anunció 28-sep-2026 acuerdo de operación y mantenimiento (O&amp;M) con NAES Corporation —mayor operador independiente de plantas de energía de EE.UU.— para operar y mantener la flota de turbinas de gas natural del campus; Fermi retiene la propiedad de los activos, NAES opera; primeras turbinas de gas Siemens Energy SGT6-5000F ya llegaron a sitio; a inicios de sep-2026 Fermi también contrató a CBRE para operar/mantener su primer data center en Matador</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [StockTitan — NAES O&amp;M](https://www.stocktitan.net/news/FRMI/fermi-selects-naes-to-operate-and-maintain-its-natural-gas-turbine-qvztuks7g3tn.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total); Fermi Inc. anunció 28-sep-2026 acuerdo de operación y mantenimiento (O&amp;M) con NAES Corporation —mayor operador independiente de plantas de energía de EE.UU.— para operar y mantener la flota de turbinas de gas natural del campus; Fermi retiene la propiedad de los activos, NAES opera; primeras turbinas de gas Siemens Energy SGT6-5000F ya llegaron a sitio; a inicios de sep-2026 Fermi también contrató a CBRE para operar/mantener su primer data center en Matador| [StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [StockTitan — NAES O&amp;M](https://www.stocktitan.net/news/FRMI/fermi-selects-naes-to-operate-and-maintain-its-natural-gas-turbine-qvztuks7g3tn.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -10955,19 +10759,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta; oct-2026: AWS presentó plan preliminar de desarrollo de terreno (PLDP) para campus de 36-39 edificios en 4 fases con inicio previsto dic-2026, pendiente de aprobación del condado, como parte de su compromiso de invertir US$20,000 millones en Pensilvania) ; Kiewit confirmado como EPC; turbinas GE Vernova habilitadas para hidrógeno con primeras entregas iniciando en 2026; planta de 4.5 GW, la más grande de Norteamérica</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053) ; [ENR](https://www.enr.com/articles/60531-kiewit-to-build-record-45-gw-gas-power-plant-for-pa-data-center-complex); [DCD](https://datacenterdynamics.com/en/news/aws-plans-36-building-data-center-campus-in-indiana-county-pennsylvania)</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
+          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta; oct-2026: AWS presentó plan preliminar de desarrollo de terreno (PLDP) para campus de 36-39 edificios en 4 fases con inicio previsto dic-2026, pendiente de aprobación del condado, como parte de su compromiso de invertir US$20,000 millones en Pensilvania) ; Kiewit confirmado como EPC; turbinas GE Vernova habilitadas para hidrógeno con primeras entregas iniciando en 2026; planta de 4.5 GW, la más grande de Norteamérica| [Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053) ; [ENR](https://www.enr.com/articles/60531-kiewit-to-build-record-45-gw-gas-power-plant-for-pa-data-center-complex); [DCD](https://datacenterdynamics.com/en/news/aws-plans-36-building-data-center-campus-in-indiana-county-pennsylvania)| 2026-10-12</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11140,19 +10936,11 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios) ; Mississippi Department of Environmental Quality otorgó permiso para 41 turbinas de gas permanentes en la planta de Southaven (~1.2 GW) que alimentará Colossus 2 (Memphis) y el próximo Colossus 3 en Mississippi; investigaciones revelaron que xAI operó 59 turbinas sin permiso (el doble de lo declarado), generando demanda legal de Earthjustice/SELC</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/) ; [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios) ; Mississippi Department of Environmental Quality otorgó permiso para 41 turbinas de gas permanentes en la planta de Southaven (~1.2 GW) que alimentará Colossus 2 (Memphis) y el próximo Colossus 3 en Mississippi; investigaciones revelaron que xAI operó 59 turbinas sin permiso (el doble de lo declarado), generando demanda legal de Earthjustice/SELC| [Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/) ; [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11177,19 +10965,11 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027) ; Babcock &amp; Wilcox firmó Limited Notice to Proceed (LNTP) por un proyecto valuado en &gt;US$1,500 millones para diseñar e instalar 1 GW de generación adicional (cuatro plantas de 300 MW a gas natural con calderas y turbinas de vapor); contrato completo esperado 1T2026; arranque operativo 2028</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/) ; [Babcock &amp; Wilcox](https://www.babcock.com/home/about/corporate/news/babcock-and-wilcox-announces-ai-data-center-power-generation-solution-and-signs-lntp-with-applied-digital-to-design-and-install-one-gigawatt-of-electric-power)</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027) ; Babcock &amp; Wilcox firmó Limited Notice to Proceed (LNTP) por un proyecto valuado en &gt;US$1,500 millones para diseñar e instalar 1 GW de generación adicional (cuatro plantas de 300 MW a gas natural con calderas y turbinas de vapor); contrato completo esperado 1T2026; arranque operativo 2028| [Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/) ; [Babcock &amp; Wilcox](https://www.babcock.com/home/about/corporate/news/babcock-and-wilcox-announces-ai-data-center-power-generation-solution-and-signs-lntp-with-applied-digital-to-design-and-install-one-gigawatt-of-electric-power)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11362,19 +11142,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky) ; Brookfield y NextEra Energy lanzaron formalmente el campus en el sitio DOE de Paducah; &gt;US$100,000 millones de inversión privada; campus de IA de 1.8 GW respaldado por 2 GW de generación a gas natural nueva más hasta 2.6 GW de almacenamiento en baterías; ~8,000 empleos de construcción</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/) ; [Data Center Knowledge](https://www.datacenterknowledge.com/data-center-construction/brookfield-nextera-launch-100b-ai-campus-at-doe-s-paducah-site)</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky) ; Brookfield y NextEra Energy lanzaron formalmente el campus en el sitio DOE de Paducah; &gt;US$100,000 millones de inversión privada; campus de IA de 1.8 GW respaldado por 2 GW de generación a gas natural nueva más hasta 2.6 GW de almacenamiento en baterías; ~8,000 empleos de construcción| [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/) ; [Data Center Knowledge](https://www.datacenterknowledge.com/data-center-construction/brookfield-nextera-launch-100b-ai-campus-at-doe-s-paducah-site)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11695,19 +11467,11 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026) ; Calpine/CyrusOne anunciaron Fase 2 del acuerdo de tierra energizada en el Thad Hill Energy Center, añadiendo 210 MW (total 400 MW); campus en construcción, operación prevista 4T2026</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/) ; [CyrusOne](https://www.cyrusone.com/resources/press-releases/calpine-and-cyrusone-announce-phase-2-of-powered-land-agreement-to-support-hyperscale-data-center-at-thad-hill-energy-center-in-texas)</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026) ; Calpine/CyrusOne anunciaron Fase 2 del acuerdo de tierra energizada en el Thad Hill Energy Center, añadiendo 210 MW (total 400 MW); campus en construcción, operación prevista 4T2026| [Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/) ; [CyrusOne](https://www.cyrusone.com/resources/press-releases/calpine-and-cyrusone-announce-phase-2-of-powered-land-agreement-to-support-hyperscale-data-center-at-thad-hill-energy-center-in-texas)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12102,19 +11866,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal) ; planta de energía asociada identificada como 'Westline 2335' (desarrollador Westline TX Holdings LLC, vinculado a Beacon Data Centers); solicitud de permiso TCEQ para 2,409 MW mediante 240 motores reciprocantes a gas en 20 'engine halls', cerca de San Angelo</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/) ; [San Angelo LIVE!](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know)</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal) ; planta de energía asociada identificada como 'Westline 2335' (desarrollador Westline TX Holdings LLC, vinculado a Beacon Data Centers); solicitud de permiso TCEQ para 2,409 MW mediante 240 motores reciprocantes a gas en 20 'engine halls', cerca de San Angelo| [San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/) ; [San Angelo LIVE!](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -14037,6 +13793,43 @@
       <c r="G134" t="inlineStr">
         <is>
           <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Taylor Technology Campus (ex-Project Mustang; 1 GW, 664 acres)</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Taylor, Condado de Williamson, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Big Watt Digital / PowerHouse Data Centers</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Ingeniería/Permisos (concejo de Taylor aprobó acuerdo de desarrollo económico oct-2026; planta de gas propia de 750 MW behind-the-meter; primera fase 500 MW, primera energía 1S2028; sujeto a pausa de interconexión ERCOT/Abbott)</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>[DCD](https://datacenterdynamics.com/en/news/powerhouse-big-watt-secure-approval-for-1gw-behind-the-meter-campus-in-taylor-texas); [KUT](https://www.kut.org/energy-environment/2026-10-09/taylor-tx-annex-data-center-power-plant)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-10-21: agrega Taylor Technology Campus (Data Centers) (#61)
* Monitoreo 2026-10-21: agrega Taylor Technology Campus (Data Centers)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LPB5RkHTWVc9WNK7uiZ9mZ

* Regenera proyectos.xlsx con Taylor Technology Campus

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LPB5RkHTWVc9WNK7uiZ9mZ

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -516,19 +516,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción; contrato EPC de Technip Energies valuado en más de €1,000 millones; capex conjunto 2026 proyectado en US$600 millones prorrateado entre CF Industries (40%), JERA y Mitsui</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/); [DecarbonFuse](https://decarbonfuse.com/posts/blue-point-breaks-ground-what-changes-now-it-s-building)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción; contrato EPC de Technip Energies valuado en más de €1,000 millones; capex conjunto 2026 proyectado en US$600 millones prorrateado entre CF Industries (40%), JERA y Mitsui| [FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/); [DecarbonFuse](https://decarbonfuse.com/posts/blue-point-breaks-ground-what-changes-now-it-s-building)| 2026-09-24</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -595,14 +587,10 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[MEES](https://www.mees.com/2026/9/25/corporate/qatarenergy-poised-to-start-up-texas-ethane-cracker/0ff02300-b8df-11f1-8f86-2b8776a66cca); [BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>[MEES](https://www.mees.com/2026/9/25/corporate/qatarenergy-poised-to-start-up-texas-ethane-cracker/0ff02300-b8df-11f1-8f86-2b8776a66cca); [BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2787,19 +2775,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028) ; Williams Companies sancionó (FID) el gasoducto "Delta Access" (US$1,500 millones, 2.25 Bcf/d iniciales ampliable a 3.5 Bcf/d, de Gillis LA hacia el corredor Transco, en servicio 1T2029) diseñado para alimentar esta expansión vía interconexión con el gasoducto intraestatal Cloud Connector de Venture Global, confirmado en su reporte 2T2026 (4-ago-2026); Baker Hughes recibió (13-sep-2026) nuevas órdenes de equipo mayor para esta expansión: 4 bloques de licuefacción (8 módulos SMR con motor eléctrico, alcance similar al ya adjudicado para CP2) y una segunda orden de paquetes de compresión Frame 5/2E para el gasoducto de alimentación intraestatal Cloud Connector, ampliando la flota total a 23 unidades — confirma actividad activa de fabricación de equipo mayor</t>
+          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028) ; Williams Companies sancionó (FID) el gasoducto "Delta Access" (US$1,500 millones, 2.25 Bcf/d iniciales ampliable a 3.5 Bcf/d, de Gillis LA hacia el corredor Transco, en servicio 1T2029) diseñado para alimentar esta expansión vía interconexión con el gasoducto intraestatal Cloud Connector de Venture Global, confirmado en su reporte 2T2026 (4-ago-2026); Baker Hughes recibió (13-sep-2026) nuevas órdenes de equipo mayor para esta expansión: 4 bloques de licuefacción (8 módulos SMR con motor eléctrico, alcance similar al ya adjudicado para CP2) y una segunda orden de paquetes de compresión Frame 5/2E para el gasoducto de alimentación intraestatal Cloud Connector, ampliando la flota total a 23 unidades — confirma actividad activa de fabricación de equipo mayor| [Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848); [Natural Gas Intel](https://www.naturalgasintel.com/news/plaquemines-expansion-to-anchor-east-end-of-williams-delta-access/); [World Pipelines](https://www.worldpipelines.com/contracts-and-tenders/14092026/baker-hughes-and-venture-global-advance-next-phase-of-us-gas-infrastructure-growth/)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848); [Natural Gas Intel](https://www.naturalgasintel.com/news/plaquemines-expansion-to-anchor-east-end-of-williams-delta-access/); [World Pipelines](https://www.worldpipelines.com/contracts-and-tenders/14092026/baker-hughes-and-venture-global-advance-next-phase-of-us-gas-infrastructure-growth/)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
           <t>2026-09-13</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4503,19 +4487,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (Estudio de Prefactibilidad —PFS— 2026 publicado 23-sep-2026: capex inicial elevado a US$1,430 millones, costo operativo US$1.47/lb, VPN después de impuestos US$3,500 millones, TIR 30%; mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; "box cut" —corte de acceso a la mina— previsto para iniciar octubre 2026; carta preliminar de US$1,100 millones del Export-Import Bank de EE.UU., aprobación final esperada primavera 2027; primera producción de cátodo de cobre prevista 2029) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>[Ivanhoe Electric — PFS 2026](https://ivanhoeelectric.com/news/2026-preliminary-feasibility-study-for-the-santa-cruz-copper-project-in-arizona-confirms-high-grade-low-cost-project-with-strong-economics/); [Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>Construcción (Estudio de Prefactibilidad —PFS— 2026 publicado 23-sep-2026: capex inicial elevado a US$1,430 millones, costo operativo US$1.47/lb, VPN después de impuestos US$3,500 millones, TIR 30%; mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; "box cut" —corte de acceso a la mina— previsto para iniciar octubre 2026; carta preliminar de US$1,100 millones del Export-Import Bank de EE.UU., aprobación final esperada primavera 2027; primera producción de cátodo de cobre prevista 2029) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins| [Ivanhoe Electric — PFS 2026](https://ivanhoeelectric.com/news/2026-preliminary-feasibility-study-for-the-santa-cruz-copper-project-in-arizona-confirms-high-grade-low-cost-project-with-strong-economics/); [Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4540,19 +4516,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción) ; bajo Hudbay Minerals (tras adquisición de Arizona Sonoran Copper, jun-2026), definitive feasibility study previsto para mediados de 2026, con FID esperada después en 2026</t>
+          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción) ; bajo Hudbay Minerals (tras adquisición de Arizona Sonoran Copper, jun-2026), definitive feasibility study previsto para mediados de 2026, con FID esperada después en 2026| [SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4577,19 +4549,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones ; otorgó contratos por ~US$110 millones a Major Drilling America y Redpath USA Corporation para avanzar exploración y desarrollo subterráneo</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/) ; [Mining Technology](https://www.mining-technology.com/news/resolution-copper-110m-contracts-arizona-mine-2/)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones ; otorgó contratos por ~US$110 millones a Major Drilling America y Redpath USA Corporation para avanzar exploración y desarrollo subterráneo| [SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/) ; [Mining Technology](https://www.mining-technology.com/news/resolution-copper-110m-contracts-arizona-mine-2/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4614,19 +4578,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; obra estructural/concreto de la planta de proceso avanzando con transición a oficios de tubería (piping) y eléctricos; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027; energización prevista 4T2026) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx) ; [Carbon Credits](https://carboncredits.com/u-s-doe-approves-2-26-billion-for-nevada-lithium-mine/)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; obra estructural/concreto de la planta de proceso avanzando con transición a oficios de tubería (piping) y eléctricos; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027; energización prevista 4T2026) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026| [Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx) ; [Carbon Credits](https://carboncredits.com/u-s-doe-approves-2-26-billion-for-nevada-lithium-mine/)| 2026-08-28</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4651,19 +4607,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026; confirmado (sep-2026) como parte de paquete de 6 complejos mineros en Zacatecas con autorizaciones federales principales (incl. Semarnat) ya obtenidas, inversión conjunta ~US$6,500 millones y ~15,000 empleos directos proyectados a partir de 2027; suministro de agua vía acueducto de ~50 km mediante convenio con la Junta Intermunicipal de Agua Potable y Alcantarillado de Zacatecas (JIAPAZ), con objetivo de reciclar el agua usada por la mina</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/) ; [Forbes México](https://forbes.com.mx/destraban-proyectos-mineros-en-zacatecas-por-6500-mdd/)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026; confirmado (sep-2026) como parte de paquete de 6 complejos mineros en Zacatecas con autorizaciones federales principales (incl. Semarnat) ya obtenidas, inversión conjunta ~US$6,500 millones y ~15,000 empleos directos proyectados a partir de 2027; suministro de agua vía acueducto de ~50 km mediante convenio con la Junta Intermunicipal de Agua Potable y Alcantarillado de Zacatecas (JIAPAZ), con objetivo de reciclar el agua usada por la mina| [Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/) ; [Forbes México](https://forbes.com.mx/destraban-proyectos-mineros-en-zacatecas-por-6500-mdd/)| 2026-09-21</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4725,19 +4673,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu) ; Southern Copper obtuvo los permisos ambientales necesarios; trabajos preliminares de sitio inician sep-2026, con construcción del proyecto arrancando en 1T2027</t>
+          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu) ; Southern Copper obtuvo los permisos ambientales necesarios; trabajos preliminares de sitio inician sep-2026, con construcción del proyecto arrancando en 1T2027| [BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico); [Dossier Político](https://dossierpolitico.com/2026/07/28/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/); [Mexico Business News](https://mexicobusiness.news/mining/news/southern-copper-unlocks-environmental-permits-el-pilar)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico); [Dossier Político](https://dossierpolitico.com/2026/07/28/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/); [Mexico Business News](https://mexicobusiness.news/mining/news/southern-copper-unlocks-environmental-permits-el-pilar)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4947,19 +4891,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027) ; en construcción con presupuesto de US$180 millones; inicio de operaciones proyectado en 2026</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027) ; en construcción con presupuesto de US$180 millones; inicio de operaciones proyectado en 2026| [Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5021,19 +4957,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción) ; BLM aprobó el proyecto el 14-ago-2026, habilitando a Gold Standard Ventures (US) Inc. a iniciar la mina; construcción emplearía hasta 600 personas</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production) ; [BLM](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción) ; BLM aprobó el proyecto el 14-ago-2026, habilitando a Gold Standard Ventures (US) Inc. a iniciar la mina; construcción emplearía hasta 600 personas| [StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production) ; [BLM](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5169,19 +5097,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026) ; equipos mayores (espesador, filtro prensa, planta de mezcla) en fabricación con entregas desde jun-2026; construcción civil en marcha desde may-2026; puesta en marcha prevista 4T2026; capex total US$11.9 millones</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html) ; [SEC 6-K Americas Gold &amp; Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002149/exhibit99-1.htm)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026) ; equipos mayores (espesador, filtro prensa, planta de mezcla) en fabricación con entregas desde jun-2026; construcción civil en marcha desde may-2026; puesta en marcha prevista 4T2026; capex total US$11.9 millones| [GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html) ; [SEC 6-K Americas Gold &amp; Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002149/exhibit99-1.htm)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5761,19 +5681,15 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029) ; Standard Lithium completó el definitive feasibility study (DFS) tras finalizar el FEED; se espera FID y arranque de construcción en 2026, con 2-3 años de construcción/comisionamiento</t>
+          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029) ; Standard Lithium completó el definitive feasibility study (DFS) tras finalizar el FEED; se espera FID y arranque de construcción en 2026, con 2-3 años de construcción/comisionamiento| [InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); [StockTitan/SEC 6-K](https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); [StockTitan/SEC 6-K](https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
           <t>2026-08-27</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5872,19 +5788,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028) ; Centerra Gold finalizará estudios de ingeniería, lanzará adquisiciones de largo plazo e iniciará trabajos de establecimiento de sitio durante 2026</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/) ; [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028) ; Centerra Gold finalizará estudios de ingeniería, lanzará adquisiciones de largo plazo e iniciará trabajos de establecimiento de sitio durante 2026| [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/) ; [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5909,19 +5817,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027) ; Hudbay Minerals completó la adquisición de Arizona Sonoran Copper el 24-jun-2026, creando el tercer distrito cuprífero más grande de Norteamérica; feasibility study esperado 2S2026, FID posible 4T2026</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/) ; [Hudbay Minerals](https://hudbayminerals.com/investors/press-releases/press-release-details/2026/Hudbay-Completes-Acquisition-of-Arizona-Sonoran-to-Create-the-Third-Largest-Copper-District-in-North-America/default.aspx)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027) ; Hudbay Minerals completó la adquisición de Arizona Sonoran Copper el 24-jun-2026, creando el tercer distrito cuprífero más grande de Norteamérica; feasibility study esperado 2S2026, FID posible 4T2026| [GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/) ; [Hudbay Minerals](https://hudbayminerals.com/investors/press-releases/press-release-details/2026/Hudbay-Completes-Acquisition-of-Arizona-Sonoran-to-Create-the-Third-Largest-Copper-District-in-North-America/default.aspx)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6057,19 +5957,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027 ; RMS preparó estimación de capital para planta de relleno en pasta: US$99 millones en construcción inicial más US$20 millones en capital sostenido para expansión del sistema de distribución subterránea</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data) ; [SEC 6-K Pan American Silver](https://www.sec.gov/Archives/edgar/data/0000771992/000077199226000047/a20260428pasni43-101xworki.htm)</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027 ; RMS preparó estimación de capital para planta de relleno en pasta: US$99 millones en construcción inicial más US$20 millones en capital sostenido para expansión del sistema de distribución subterránea| [Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data) ; [SEC 6-K Pan American Silver](https://www.sec.gov/Archives/edgar/data/0000771992/000077199226000047/a20260428pasni43-101xworki.htm)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6945,19 +6837,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027| [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7759,19 +7643,11 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028| [KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7833,19 +7709,11 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar| [Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9079,7 +8947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9142,19 +9010,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026) ; VoltaGrid fue aprobado por TCEQ para operar 210 generadores industriales a gas (700 MW: 197 generación primaria + 13 respaldo) con motores Jenbacher; Vantage Data Centers confirmado como socio desarrollador; primer edificio previsto para fines de 2026</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid) ; [Construction Owners Association](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026) ; VoltaGrid fue aprobado por TCEQ para operar 210 generadores industriales a gas (700 MW: 197 generación primaria + 13 respaldo) con motores Jenbacher; Vantage Data Centers confirmado como socio desarrollador; primer edificio previsto para fines de 2026| [DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid) ; [Construction Owners Association](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9216,19 +9076,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales (expansión de 10 a 49 turbinas); TCEQ otorgó reunión pública sobre esta solicitud a petición del representante estatal Stan Lambert (~10-sep-2026), periodo de comentarios abierto; además, el gobernador Greg Abbott ordenó el 21-sep-2026 a la TCEQ pausar toda emisión de permisos nuevos para proyectos de data centers en Texas —incluidas instalaciones con generación propia "behind-the-meter"— hasta que ERCOT complete una auditoría de red (esperada mediados de dic-2026; TCEQ debe reportar cumplimiento al 19-oct-2026), lo que podría retrasar trámites pendientes de este y otros proyectos texanos del tracker</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/); [Texas Tribune](https://www.texastribune.org/2026/09/21/texas-data-center-moratorium-water-energy/); [Bracewell](https://www.bracewell.com/resources/governor-abbott-orders-tceq-to-pause-all-permit-issuance-for-data-center-projects/)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales (expansión de 10 a 49 turbinas); TCEQ otorgó reunión pública sobre esta solicitud a petición del representante estatal Stan Lambert (~10-sep-2026), periodo de comentarios abierto; además, el gobernador Greg Abbott ordenó el 21-sep-2026 a la TCEQ pausar toda emisión de permisos nuevos para proyectos de data centers en Texas —incluidas instalaciones con generación propia "behind-the-meter"— hasta que ERCOT complete una auditoría de red (esperada mediados de dic-2026; TCEQ debe reportar cumplimiento al 19-oct-2026), lo que podría retrasar trámites pendientes de este y otros proyectos texanos del tracker| [DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/); [Texas Tribune](https://www.texastribune.org/2026/09/21/texas-data-center-moratorium-water-energy/); [Bracewell](https://www.bracewell.com/resources/governor-abbott-orders-tceq-to-pause-all-permit-issuance-for-data-center-projects/)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9253,19 +9105,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026) ; Chevron (vía subsidiaria Energy Forge One LLC) firmó PPA a 20 años con Microsoft; 2.67 GW de capacidad, turbinas principalmente GE Vernova más Solar Turbines (Caterpillar); ubicación precisada en Condado de Reeves (2,000+ acres); FID esperada fin de 2026, arranque 2028</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center) ; [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026) ; Chevron (vía subsidiaria Energy Forge One LLC) firmó PPA a 20 años con Microsoft; 2.67 GW de capacidad, turbinas principalmente GE Vernova más Solar Turbines (Caterpillar); ubicación precisada en Condado de Reeves (2,000+ acres); FID esperada fin de 2026, arranque 2028| [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center) ; [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9475,19 +9319,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT) ; Amazon confirmó públicamente su propiedad del proyecto; permiso otorgado para 35 turbinas de gas natural (hasta 7.65 GW), el permiso de emisiones más grande otorgado este año en el país (~33 millones de toneladas de CO2/año); incluye hasta 750 MW solar y 1.8 GW de almacenamiento en baterías; primera energía prevista 1T2027, 1 GW en servicio en 2028</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases) ; [ENR](https://www.enr.com/articles/63464-amazon-discloses-ownership-of-gw-ranch-giant-texas-data-center-gas-power-complex)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT) ; Amazon confirmó públicamente su propiedad del proyecto; permiso otorgado para 35 turbinas de gas natural (hasta 7.65 GW), el permiso de emisiones más grande otorgado este año en el país (~33 millones de toneladas de CO2/año); incluye hasta 750 MW solar y 1.8 GW de almacenamiento en baterías; primera energía prevista 1T2027, 1 GW en servicio en 2028| [Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases) ; [ENR](https://www.enr.com/articles/63464-amazon-discloses-ownership-of-gw-ranch-giant-texas-data-center-gas-power-complex)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9623,19 +9459,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027) ; Oracle/BorderPlex Digital Assets cambiaron el plan de generación de turbinas de gas/generadores diésel a un microgrid de celdas de combustible para reducir uso de agua e impacto en calidad del aire; gasoducto asociado 'Green Chile Project' (~US$60 millones, 17.7 millas) bajo revisión FERC enfrenta protesta de personal regulador federal, entrada en servicio prevista ago-2026</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027) ; [Source NM](https://sourcenm.com/2026/04/27/nm-project-jupiter-data-center-developers-announce-new-plans-for-generating-power/)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027) ; Oracle/BorderPlex Digital Assets cambiaron el plan de generación de turbinas de gas/generadores diésel a un microgrid de celdas de combustible para reducir uso de agua e impacto en calidad del aire; gasoducto asociado 'Green Chile Project' (~US$60 millones, 17.7 millas) bajo revisión FERC enfrenta protesta de personal regulador federal, entrada en servicio prevista ago-2026| [Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027) ; [Source NM](https://sourcenm.com/2026/04/27/nm-project-jupiter-data-center-developers-announce-new-plans-for-generating-power/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9734,19 +9562,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Planeación temprana (opción de terreno) ; se formalizó opción de compra de ~3,500 acres en Condado de Lea, Nuevo México, para hub de IA de 7 GW; marca el primer desarrollo enteramente propio, separado del joint venture TCDC; planea &gt;2 GW de gas natural más 5+ GW de generación nuclear</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/) ; [Barchart](https://www.barchart.com/story/news/35949566/new-era-energy-digital-enters-into-land-option-purchase-agreement-for-3-500-acres-in-new-mexico-for-7gw-ai-data-center-hub-marks-first-wholly-owned-development-separate-from-tcdc-joint-venture)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Planeación temprana (opción de terreno) ; se formalizó opción de compra de ~3,500 acres en Condado de Lea, Nuevo México, para hub de IA de 7 GW; marca el primer desarrollo enteramente propio, separado del joint venture TCDC; planea &gt;2 GW de gas natural más 5+ GW de generación nuclear| [PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/) ; [Barchart](https://www.barchart.com/story/news/35949566/new-era-energy-digital-enters-into-land-option-purchase-agreement-for-3-500-acres-in-new-mexico-for-7gw-ai-data-center-hub-marks-first-wholly-owned-development-separate-from-tcdc-joint-venture)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10289,19 +10109,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos) ; OpenAI se unió como inversionista/arrendatario; Nvidia garantiza hasta US$105,000 millones en obligaciones de arrendamiento y pago de energía; escala confirmada en 8 IT-GW de cómputo/10 GW de generación nueva (9.2 GW de gas natural); costo total potencial hasta US$500,000 millones; primera fase de 800 MW en operación en 2028</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html) ; [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos) ; OpenAI se unió como inversionista/arrendatario; Nvidia garantiza hasta US$105,000 millones en obligaciones de arrendamiento y pago de energía; escala confirmada en 8 IT-GW de cómputo/10 GW de generación nueva (9.2 GW de gas natural); costo total potencial hasta US$500,000 millones; primera fase de 800 MW en operación en 2028| [DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html) ; [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10548,19 +10360,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total); Fermi Inc. anunció 28-sep-2026 acuerdo de operación y mantenimiento (O&amp;M) con NAES Corporation —mayor operador independiente de plantas de energía de EE.UU.— para operar y mantener la flota de turbinas de gas natural del campus; Fermi retiene la propiedad de los activos, NAES opera; primeras turbinas de gas Siemens Energy SGT6-5000F ya llegaron a sitio; a inicios de sep-2026 Fermi también contrató a CBRE para operar/mantener su primer data center en Matador</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [StockTitan — NAES O&amp;M](https://www.stocktitan.net/news/FRMI/fermi-selects-naes-to-operate-and-maintain-its-natural-gas-turbine-qvztuks7g3tn.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año; Fermi Inc. y TensorWave firmaron 22-sep-2026 una Primera Enmienda al contrato de arrendamiento, extendiendo el cierre financiero del 30-sep-2026 al 31-oct-2026 mientras se negocia una garantía con contraparte investment-grade; Fermi realizó un giro inicial de su línea de financiamiento de equipo de US$200 millones (Keystone National Group/Cape Commercial Finance) para acelerar adquisición de transformadores, subestaciones y switchgear de los primeros 2.3GW de la fase HyperGrid (11GW total); Fermi Inc. anunció 28-sep-2026 acuerdo de operación y mantenimiento (O&amp;M) con NAES Corporation —mayor operador independiente de plantas de energía de EE.UU.— para operar y mantener la flota de turbinas de gas natural del campus; Fermi retiene la propiedad de los activos, NAES opera; primeras turbinas de gas Siemens Energy SGT6-5000F ya llegaron a sitio; a inicios de sep-2026 Fermi también contrató a CBRE para operar/mantener su primer data center en Matador| [StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [StockTitan — NAES O&amp;M](https://www.stocktitan.net/news/FRMI/fermi-selects-naes-to-operate-and-maintain-its-natural-gas-turbine-qvztuks7g3tn.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/); [ValueTheMarkets](https://www.valuethemarkets.com/news/press-releases/fermi-and-tensorwave-agree-to-extend-closing-date-to-october); [PR Newswire](https://www.prnewswire.com/news-releases/fermi-america-makes-initial-draw-on-200-million-equipment-facility-from-keystone-national-group-and-cape-commercial-finance-to-accelerate-the-delivery-of-the-first-2-3gw-of-project-matadors-11gw-private-hypergrid-campus-302693111.html)| 2026-09-28</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -10955,19 +10759,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta; oct-2026: AWS presentó plan preliminar de desarrollo de terreno (PLDP) para campus de 36-39 edificios en 4 fases con inicio previsto dic-2026, pendiente de aprobación del condado, como parte de su compromiso de invertir US$20,000 millones en Pensilvania) ; Kiewit confirmado como EPC; turbinas GE Vernova habilitadas para hidrógeno con primeras entregas iniciando en 2026; planta de 4.5 GW, la más grande de Norteamérica</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053) ; [ENR](https://www.enr.com/articles/60531-kiewit-to-build-record-45-gw-gas-power-plant-for-pa-data-center-complex); [DCD](https://datacenterdynamics.com/en/news/aws-plans-36-building-data-center-campus-in-indiana-county-pennsylvania)</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
+          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta; oct-2026: AWS presentó plan preliminar de desarrollo de terreno (PLDP) para campus de 36-39 edificios en 4 fases con inicio previsto dic-2026, pendiente de aprobación del condado, como parte de su compromiso de invertir US$20,000 millones en Pensilvania) ; Kiewit confirmado como EPC; turbinas GE Vernova habilitadas para hidrógeno con primeras entregas iniciando en 2026; planta de 4.5 GW, la más grande de Norteamérica| [Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053) ; [ENR](https://www.enr.com/articles/60531-kiewit-to-build-record-45-gw-gas-power-plant-for-pa-data-center-complex); [DCD](https://datacenterdynamics.com/en/news/aws-plans-36-building-data-center-campus-in-indiana-county-pennsylvania)| 2026-10-12</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11140,19 +10936,11 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios) ; Mississippi Department of Environmental Quality otorgó permiso para 41 turbinas de gas permanentes en la planta de Southaven (~1.2 GW) que alimentará Colossus 2 (Memphis) y el próximo Colossus 3 en Mississippi; investigaciones revelaron que xAI operó 59 turbinas sin permiso (el doble de lo declarado), generando demanda legal de Earthjustice/SELC</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/) ; [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios) ; Mississippi Department of Environmental Quality otorgó permiso para 41 turbinas de gas permanentes en la planta de Southaven (~1.2 GW) que alimentará Colossus 2 (Memphis) y el próximo Colossus 3 en Mississippi; investigaciones revelaron que xAI operó 59 turbinas sin permiso (el doble de lo declarado), generando demanda legal de Earthjustice/SELC| [Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/) ; [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11177,19 +10965,11 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027) ; Babcock &amp; Wilcox firmó Limited Notice to Proceed (LNTP) por un proyecto valuado en &gt;US$1,500 millones para diseñar e instalar 1 GW de generación adicional (cuatro plantas de 300 MW a gas natural con calderas y turbinas de vapor); contrato completo esperado 1T2026; arranque operativo 2028</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/) ; [Babcock &amp; Wilcox](https://www.babcock.com/home/about/corporate/news/babcock-and-wilcox-announces-ai-data-center-power-generation-solution-and-signs-lntp-with-applied-digital-to-design-and-install-one-gigawatt-of-electric-power)</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027) ; Babcock &amp; Wilcox firmó Limited Notice to Proceed (LNTP) por un proyecto valuado en &gt;US$1,500 millones para diseñar e instalar 1 GW de generación adicional (cuatro plantas de 300 MW a gas natural con calderas y turbinas de vapor); contrato completo esperado 1T2026; arranque operativo 2028| [Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/) ; [Babcock &amp; Wilcox](https://www.babcock.com/home/about/corporate/news/babcock-and-wilcox-announces-ai-data-center-power-generation-solution-and-signs-lntp-with-applied-digital-to-design-and-install-one-gigawatt-of-electric-power)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11362,19 +11142,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky) ; Brookfield y NextEra Energy lanzaron formalmente el campus en el sitio DOE de Paducah; &gt;US$100,000 millones de inversión privada; campus de IA de 1.8 GW respaldado por 2 GW de generación a gas natural nueva más hasta 2.6 GW de almacenamiento en baterías; ~8,000 empleos de construcción</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/) ; [Data Center Knowledge](https://www.datacenterknowledge.com/data-center-construction/brookfield-nextera-launch-100b-ai-campus-at-doe-s-paducah-site)</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky) ; Brookfield y NextEra Energy lanzaron formalmente el campus en el sitio DOE de Paducah; &gt;US$100,000 millones de inversión privada; campus de IA de 1.8 GW respaldado por 2 GW de generación a gas natural nueva más hasta 2.6 GW de almacenamiento en baterías; ~8,000 empleos de construcción| [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/) ; [Data Center Knowledge](https://www.datacenterknowledge.com/data-center-construction/brookfield-nextera-launch-100b-ai-campus-at-doe-s-paducah-site)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -11695,19 +11467,11 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026) ; Calpine/CyrusOne anunciaron Fase 2 del acuerdo de tierra energizada en el Thad Hill Energy Center, añadiendo 210 MW (total 400 MW); campus en construcción, operación prevista 4T2026</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/) ; [CyrusOne](https://www.cyrusone.com/resources/press-releases/calpine-and-cyrusone-announce-phase-2-of-powered-land-agreement-to-support-hyperscale-data-center-at-thad-hill-energy-center-in-texas)</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026) ; Calpine/CyrusOne anunciaron Fase 2 del acuerdo de tierra energizada en el Thad Hill Energy Center, añadiendo 210 MW (total 400 MW); campus en construcción, operación prevista 4T2026| [Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/) ; [CyrusOne](https://www.cyrusone.com/resources/press-releases/calpine-and-cyrusone-announce-phase-2-of-powered-land-agreement-to-support-hyperscale-data-center-at-thad-hill-energy-center-in-texas)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -12102,19 +11866,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal) ; planta de energía asociada identificada como 'Westline 2335' (desarrollador Westline TX Holdings LLC, vinculado a Beacon Data Centers); solicitud de permiso TCEQ para 2,409 MW mediante 240 motores reciprocantes a gas en 20 'engine halls', cerca de San Angelo</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/) ; [San Angelo LIVE!](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know)</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal) ; planta de energía asociada identificada como 'Westline 2335' (desarrollador Westline TX Holdings LLC, vinculado a Beacon Data Centers); solicitud de permiso TCEQ para 2,409 MW mediante 240 motores reciprocantes a gas en 20 'engine halls', cerca de San Angelo| [San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/) ; [San Angelo LIVE!](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know)| 2026-08-27</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -14037,6 +13793,43 @@
       <c r="G134" t="inlineStr">
         <is>
           <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Taylor Technology Campus (ex-Project Mustang; 1 GW, 664 acres)</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Taylor, Condado de Williamson, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Big Watt Digital / PowerHouse Data Centers</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Ingeniería/Permisos (concejo de Taylor aprobó acuerdo de desarrollo económico oct-2026; planta de gas propia de 750 MW behind-the-meter; primera fase 500 MW, primera energía 1S2028; sujeto a pausa de interconexión ERCOT/Abbott)</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>[DCD](https://datacenterdynamics.com/en/news/powerhouse-big-watt-secure-approval-for-1gw-behind-the-meter-campus-in-taylor-texas); [KUT](https://www.kut.org/energy-environment/2026-10-09/taylor-tx-annex-data-center-power-plant)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>